<commit_message>
Add product documentation for archive-base ARPU initiative
Discovery, international benchmarks, EASY/HARD initiative portfolio,
unit economics, success probabilities, CJM, roadmap with stage gates,
data-driven experiment design, analyst data request, risks and
regulatory analysis, RACI, and defense pitch with Q&A. Model now
excludes the rejected B4 from portfolios and applies overlap to
margin rather than costs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXPWSEPNsscJqgN9a1CPPP
</commit_message>
<xml_diff>
--- a/model/Ucell_Archive_ARPU_Model.xlsx
+++ b/model/Ucell_Archive_ARPU_Model.xlsx
@@ -1332,7 +1332,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="329">
   <si>
     <t xml:space="preserve">Ucell — модель роста ARPU архивной базы</t>
   </si>
@@ -1646,10 +1646,10 @@
     <t xml:space="preserve">complexity</t>
   </si>
   <si>
-    <t xml:space="preserve">Опция вне базового портфеля (1=да)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">optional</t>
+    <t xml:space="preserve">Портфель: 1 = базовый, 2 = опция (Stretch), 0 = не рекомендуется</t>
+  </si>
+  <si>
+    <t xml:space="preserve">portfolio</t>
   </si>
   <si>
     <t xml:space="preserve">ARPU целевого сегмента, сум</t>
@@ -2081,7 +2081,7 @@
     <t xml:space="preserve">B5 — Персональные лимиты «Mobil avans» на ML-скоринге</t>
   </si>
   <si>
-    <t xml:space="preserve">ПОРТФЕЛЬ (детерминированный, все инициативы запущены)</t>
+    <t xml:space="preserve">ПОРТФЕЛЬ (детерминированный, все рекомендуемые инициативы запущены)</t>
   </si>
   <si>
     <t xml:space="preserve">Базовый: Σ выручка когорты до перекрытия</t>
@@ -2132,7 +2132,7 @@
     <t xml:space="preserve">Группа</t>
   </si>
   <si>
-    <t xml:space="preserve">Опция</t>
+    <t xml:space="preserve">Портфель (1/2/0)</t>
   </si>
   <si>
     <t xml:space="preserve">Выручка Y1</t>
@@ -2147,6 +2147,9 @@
     <t xml:space="preserve">Вклад 24 мес</t>
   </si>
   <si>
+    <t xml:space="preserve">Затраты 24 мес</t>
+  </si>
+  <si>
     <t xml:space="preserve">ROI</t>
   </si>
   <si>
@@ -2177,7 +2180,7 @@
     <t xml:space="preserve">Базовый: run-rate/год, USD</t>
   </si>
   <si>
-    <t xml:space="preserve">Базовый: вклад 24 мес. (перекрытие снижает положительный вклад)</t>
+    <t xml:space="preserve">Базовый: вклад 24 мес. = маржа × (1 − перекрытие) − затраты</t>
   </si>
   <si>
     <t xml:space="preserve">Базовый: ARPU когорты до, сум</t>
@@ -2919,58 +2922,58 @@
                   <c:v>0.060889228198737</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.0621315570872716</c:v>
+                  <c:v>0.061985033613716</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.069418719511358</c:v>
+                  <c:v>0.0691235127657535</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.0770839389395031</c:v>
+                  <c:v>0.0766379481432185</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.0847730367239115</c:v>
+                  <c:v>0.084174219083041</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.0924824310559202</c:v>
+                  <c:v>0.0917288044418745</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.15810325983979</c:v>
+                  <c:v>0.157189107476957</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.159703081199678</c:v>
+                  <c:v>0.158785562750602</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.159597929317036</c:v>
+                  <c:v>0.158681525125549</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.159498244825305</c:v>
+                  <c:v>0.158582953831683</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.159403667150353</c:v>
+                  <c:v>0.158489488369902</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.159313860994026</c:v>
+                  <c:v>0.158400793510755</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.159228514564728</c:v>
+                  <c:v>0.158316557525587</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.15914733793189</c:v>
+                  <c:v>0.158236490541512</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.159070061495652</c:v>
+                  <c:v>0.158160323011566</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.158996434563685</c:v>
+                  <c:v>0.158087804291958</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.158926224027667</c:v>
+                  <c:v>0.158018701318935</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.158859213132414</c:v>
+                  <c:v>0.157952797378276</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.158795200331197</c:v>
+                  <c:v>0.157889890960932</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3135,58 +3138,58 @@
                   <c:v>0.060889228198737</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.0621315570872716</c:v>
+                  <c:v>0.061985033613716</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.069418719511358</c:v>
+                  <c:v>0.0691235127657535</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.0770839389395031</c:v>
+                  <c:v>0.0766379481432185</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.0847730367239115</c:v>
+                  <c:v>0.084174219083041</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.0924824310559202</c:v>
+                  <c:v>0.0917288044418745</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.15810325983979</c:v>
+                  <c:v>0.157189107476957</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.159703081199678</c:v>
+                  <c:v>0.158785562750602</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.192147052111267</c:v>
+                  <c:v>0.191229662214945</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.19140071552816</c:v>
+                  <c:v>0.190482823907693</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.191280992647323</c:v>
+                  <c:v>0.190364386863735</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.191166085856019</c:v>
+                  <c:v>0.190250764970839</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.191055682056861</c:v>
+                  <c:v>0.190141645195647</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.190949490101003</c:v>
+                  <c:v>0.190036736448046</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.190847239251648</c:v>
+                  <c:v>0.18993576804514</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.190748677755125</c:v>
+                  <c:v>0.189838488282769</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.190653571512023</c:v>
+                  <c:v>0.189744663107028</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.190561702841365</c:v>
+                  <c:v>0.189654074878809</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.190472869331314</c:v>
+                  <c:v>0.189566521224838</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3201,11 +3204,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="52797063"/>
-        <c:axId val="70033722"/>
+        <c:axId val="60557033"/>
+        <c:axId val="58042223"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="52797063"/>
+        <c:axId val="60557033"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3271,7 +3274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70033722"/>
+        <c:crossAx val="58042223"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3279,7 +3282,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="70033722"/>
+        <c:axId val="58042223"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3355,7 +3358,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52797063"/>
+        <c:crossAx val="60557033"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4427,43 +4430,43 @@
         <v>105</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="L8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24594,100 +24597,100 @@
       </c>
       <c r="B190" s="4"/>
       <c r="C190" s="8" t="n">
-        <f aca="false">C14*(1-Initiatives!$C$8)+C28*(1-Initiatives!$D$8)+C42*(1-Initiatives!$E$8)+C56*(1-Initiatives!$F$8)+C70*(1-Initiatives!$G$8)+C84*(1-Initiatives!$H$8)+C98*(1-Initiatives!$I$8)+C112*(1-Initiatives!$J$8)+C126*(1-Initiatives!$K$8)+C140*(1-Initiatives!$L$8)+C154*(1-Initiatives!$M$8)+C168*(1-Initiatives!$N$8)+C182*(1-Initiatives!$O$8)</f>
+        <f aca="false">C14*(Initiatives!$C$8=1)+C28*(Initiatives!$D$8=1)+C42*(Initiatives!$E$8=1)+C56*(Initiatives!$F$8=1)+C70*(Initiatives!$G$8=1)+C84*(Initiatives!$H$8=1)+C98*(Initiatives!$I$8=1)+C112*(Initiatives!$J$8=1)+C126*(Initiatives!$K$8=1)+C140*(Initiatives!$L$8=1)+C154*(Initiatives!$M$8=1)+C168*(Initiatives!$N$8=1)+C182*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="D190" s="8" t="n">
-        <f aca="false">D14*(1-Initiatives!$C$8)+D28*(1-Initiatives!$D$8)+D42*(1-Initiatives!$E$8)+D56*(1-Initiatives!$F$8)+D70*(1-Initiatives!$G$8)+D84*(1-Initiatives!$H$8)+D98*(1-Initiatives!$I$8)+D112*(1-Initiatives!$J$8)+D126*(1-Initiatives!$K$8)+D140*(1-Initiatives!$L$8)+D154*(1-Initiatives!$M$8)+D168*(1-Initiatives!$N$8)+D182*(1-Initiatives!$O$8)</f>
+        <f aca="false">D14*(Initiatives!$C$8=1)+D28*(Initiatives!$D$8=1)+D42*(Initiatives!$E$8=1)+D56*(Initiatives!$F$8=1)+D70*(Initiatives!$G$8=1)+D84*(Initiatives!$H$8=1)+D98*(Initiatives!$I$8=1)+D112*(Initiatives!$J$8=1)+D126*(Initiatives!$K$8=1)+D140*(Initiatives!$L$8=1)+D154*(Initiatives!$M$8=1)+D168*(Initiatives!$N$8=1)+D182*(Initiatives!$O$8=1)</f>
         <v>3129569897.14286</v>
       </c>
       <c r="E190" s="8" t="n">
-        <f aca="false">E14*(1-Initiatives!$C$8)+E28*(1-Initiatives!$D$8)+E42*(1-Initiatives!$E$8)+E56*(1-Initiatives!$F$8)+E70*(1-Initiatives!$G$8)+E84*(1-Initiatives!$H$8)+E98*(1-Initiatives!$I$8)+E112*(1-Initiatives!$J$8)+E126*(1-Initiatives!$K$8)+E140*(1-Initiatives!$L$8)+E154*(1-Initiatives!$M$8)+E168*(1-Initiatives!$N$8)+E182*(1-Initiatives!$O$8)</f>
+        <f aca="false">E14*(Initiatives!$C$8=1)+E28*(Initiatives!$D$8=1)+E42*(Initiatives!$E$8=1)+E56*(Initiatives!$F$8=1)+E70*(Initiatives!$G$8=1)+E84*(Initiatives!$H$8=1)+E98*(Initiatives!$I$8=1)+E112*(Initiatives!$J$8=1)+E126*(Initiatives!$K$8=1)+E140*(Initiatives!$L$8=1)+E154*(Initiatives!$M$8=1)+E168*(Initiatives!$N$8=1)+E182*(Initiatives!$O$8=1)</f>
         <v>3414492594.76167</v>
       </c>
       <c r="F190" s="8" t="n">
-        <f aca="false">F14*(1-Initiatives!$C$8)+F28*(1-Initiatives!$D$8)+F42*(1-Initiatives!$E$8)+F56*(1-Initiatives!$F$8)+F70*(1-Initiatives!$G$8)+F84*(1-Initiatives!$H$8)+F98*(1-Initiatives!$I$8)+F112*(1-Initiatives!$J$8)+F126*(1-Initiatives!$K$8)+F140*(1-Initiatives!$L$8)+F154*(1-Initiatives!$M$8)+F168*(1-Initiatives!$N$8)+F182*(1-Initiatives!$O$8)</f>
+        <f aca="false">F14*(Initiatives!$C$8=1)+F28*(Initiatives!$D$8=1)+F42*(Initiatives!$E$8=1)+F56*(Initiatives!$F$8=1)+F70*(Initiatives!$G$8=1)+F84*(Initiatives!$H$8=1)+F98*(Initiatives!$I$8=1)+F112*(Initiatives!$J$8=1)+F126*(Initiatives!$K$8=1)+F140*(Initiatives!$L$8=1)+F154*(Initiatives!$M$8=1)+F168*(Initiatives!$N$8=1)+F182*(Initiatives!$O$8=1)</f>
         <v>3780561440.85284</v>
       </c>
       <c r="G190" s="8" t="n">
-        <f aca="false">G14*(1-Initiatives!$C$8)+G28*(1-Initiatives!$D$8)+G42*(1-Initiatives!$E$8)+G56*(1-Initiatives!$F$8)+G70*(1-Initiatives!$G$8)+G84*(1-Initiatives!$H$8)+G98*(1-Initiatives!$I$8)+G112*(1-Initiatives!$J$8)+G126*(1-Initiatives!$K$8)+G140*(1-Initiatives!$L$8)+G154*(1-Initiatives!$M$8)+G168*(1-Initiatives!$N$8)+G182*(1-Initiatives!$O$8)</f>
+        <f aca="false">G14*(Initiatives!$C$8=1)+G28*(Initiatives!$D$8=1)+G42*(Initiatives!$E$8=1)+G56*(Initiatives!$F$8=1)+G70*(Initiatives!$G$8=1)+G84*(Initiatives!$H$8=1)+G98*(Initiatives!$I$8=1)+G112*(Initiatives!$J$8=1)+G126*(Initiatives!$K$8=1)+G140*(Initiatives!$L$8=1)+G154*(Initiatives!$M$8=1)+G168*(Initiatives!$N$8=1)+G182*(Initiatives!$O$8=1)</f>
         <v>4048474712.29852</v>
       </c>
       <c r="H190" s="8" t="n">
-        <f aca="false">H14*(1-Initiatives!$C$8)+H28*(1-Initiatives!$D$8)+H42*(1-Initiatives!$E$8)+H56*(1-Initiatives!$F$8)+H70*(1-Initiatives!$G$8)+H84*(1-Initiatives!$H$8)+H98*(1-Initiatives!$I$8)+H112*(1-Initiatives!$J$8)+H126*(1-Initiatives!$K$8)+H140*(1-Initiatives!$L$8)+H154*(1-Initiatives!$M$8)+H168*(1-Initiatives!$N$8)+H182*(1-Initiatives!$O$8)</f>
+        <f aca="false">H14*(Initiatives!$C$8=1)+H28*(Initiatives!$D$8=1)+H42*(Initiatives!$E$8=1)+H56*(Initiatives!$F$8=1)+H70*(Initiatives!$G$8=1)+H84*(Initiatives!$H$8=1)+H98*(Initiatives!$I$8=1)+H112*(Initiatives!$J$8=1)+H126*(Initiatives!$K$8=1)+H140*(Initiatives!$L$8=1)+H154*(Initiatives!$M$8=1)+H168*(Initiatives!$N$8=1)+H182*(Initiatives!$O$8=1)</f>
         <v>4133341488.32033</v>
       </c>
       <c r="I190" s="8" t="n">
-        <f aca="false">I14*(1-Initiatives!$C$8)+I28*(1-Initiatives!$D$8)+I42*(1-Initiatives!$E$8)+I56*(1-Initiatives!$F$8)+I70*(1-Initiatives!$G$8)+I84*(1-Initiatives!$H$8)+I98*(1-Initiatives!$I$8)+I112*(1-Initiatives!$J$8)+I126*(1-Initiatives!$K$8)+I140*(1-Initiatives!$L$8)+I154*(1-Initiatives!$M$8)+I168*(1-Initiatives!$N$8)+I182*(1-Initiatives!$O$8)</f>
-        <v>4170600474.76252</v>
+        <f aca="false">I14*(Initiatives!$C$8=1)+I28*(Initiatives!$D$8=1)+I42*(Initiatives!$E$8=1)+I56*(Initiatives!$F$8=1)+I70*(Initiatives!$G$8=1)+I84*(Initiatives!$H$8=1)+I98*(Initiatives!$I$8=1)+I112*(Initiatives!$J$8=1)+I126*(Initiatives!$K$8=1)+I140*(Initiatives!$L$8=1)+I154*(Initiatives!$M$8=1)+I168*(Initiatives!$N$8=1)+I182*(Initiatives!$O$8=1)</f>
+        <v>4159923141.42919</v>
       </c>
       <c r="J190" s="8" t="n">
-        <f aca="false">J14*(1-Initiatives!$C$8)+J28*(1-Initiatives!$D$8)+J42*(1-Initiatives!$E$8)+J56*(1-Initiatives!$F$8)+J70*(1-Initiatives!$G$8)+J84*(1-Initiatives!$H$8)+J98*(1-Initiatives!$I$8)+J112*(1-Initiatives!$J$8)+J126*(1-Initiatives!$K$8)+J140*(1-Initiatives!$L$8)+J154*(1-Initiatives!$M$8)+J168*(1-Initiatives!$N$8)+J182*(1-Initiatives!$O$8)</f>
-        <v>4652264753.93452</v>
+        <f aca="false">J14*(Initiatives!$C$8=1)+J28*(Initiatives!$D$8=1)+J42*(Initiatives!$E$8=1)+J56*(Initiatives!$F$8=1)+J70*(Initiatives!$G$8=1)+J84*(Initiatives!$H$8=1)+J98*(Initiatives!$I$8=1)+J112*(Initiatives!$J$8=1)+J126*(Initiatives!$K$8=1)+J140*(Initiatives!$L$8=1)+J154*(Initiatives!$M$8=1)+J168*(Initiatives!$N$8=1)+J182*(Initiatives!$O$8=1)</f>
+        <v>4631006183.26785</v>
       </c>
       <c r="K190" s="8" t="n">
-        <f aca="false">K14*(1-Initiatives!$C$8)+K28*(1-Initiatives!$D$8)+K42*(1-Initiatives!$E$8)+K56*(1-Initiatives!$F$8)+K70*(1-Initiatives!$G$8)+K84*(1-Initiatives!$H$8)+K98*(1-Initiatives!$I$8)+K112*(1-Initiatives!$J$8)+K126*(1-Initiatives!$K$8)+K140*(1-Initiatives!$L$8)+K154*(1-Initiatives!$M$8)+K168*(1-Initiatives!$N$8)+K182*(1-Initiatives!$O$8)</f>
-        <v>5157982161.11338</v>
+        <f aca="false">K14*(Initiatives!$C$8=1)+K28*(Initiatives!$D$8=1)+K42*(Initiatives!$E$8=1)+K56*(Initiatives!$F$8=1)+K70*(Initiatives!$G$8=1)+K84*(Initiatives!$H$8=1)+K98*(Initiatives!$I$8=1)+K112*(Initiatives!$J$8=1)+K126*(Initiatives!$K$8=1)+K140*(Initiatives!$L$8=1)+K154*(Initiatives!$M$8=1)+K168*(Initiatives!$N$8=1)+K182*(Initiatives!$O$8=1)</f>
+        <v>5126237776.44138</v>
       </c>
       <c r="L190" s="8" t="n">
-        <f aca="false">L14*(1-Initiatives!$C$8)+L28*(1-Initiatives!$D$8)+L42*(1-Initiatives!$E$8)+L56*(1-Initiatives!$F$8)+L70*(1-Initiatives!$G$8)+L84*(1-Initiatives!$H$8)+L98*(1-Initiatives!$I$8)+L112*(1-Initiatives!$J$8)+L126*(1-Initiatives!$K$8)+L140*(1-Initiatives!$L$8)+L154*(1-Initiatives!$M$8)+L168*(1-Initiatives!$N$8)+L182*(1-Initiatives!$O$8)</f>
-        <v>5661543864.11443</v>
+        <f aca="false">L14*(Initiatives!$C$8=1)+L28*(Initiatives!$D$8=1)+L42*(Initiatives!$E$8=1)+L56*(Initiatives!$F$8=1)+L70*(Initiatives!$G$8=1)+L84*(Initiatives!$H$8=1)+L98*(Initiatives!$I$8=1)+L112*(Initiatives!$J$8=1)+L126*(Initiatives!$K$8=1)+L140*(Initiatives!$L$8=1)+L154*(Initiatives!$M$8=1)+L168*(Initiatives!$N$8=1)+L182*(Initiatives!$O$8=1)</f>
+        <v>5619408416.95796</v>
       </c>
       <c r="M190" s="8" t="n">
-        <f aca="false">M14*(1-Initiatives!$C$8)+M28*(1-Initiatives!$D$8)+M42*(1-Initiatives!$E$8)+M56*(1-Initiatives!$F$8)+M70*(1-Initiatives!$G$8)+M84*(1-Initiatives!$H$8)+M98*(1-Initiatives!$I$8)+M112*(1-Initiatives!$J$8)+M126*(1-Initiatives!$K$8)+M140*(1-Initiatives!$L$8)+M154*(1-Initiatives!$M$8)+M168*(1-Initiatives!$N$8)+M182*(1-Initiatives!$O$8)</f>
-        <v>6162706605.69958</v>
+        <f aca="false">M14*(Initiatives!$C$8=1)+M28*(Initiatives!$D$8=1)+M42*(Initiatives!$E$8=1)+M56*(Initiatives!$F$8=1)+M70*(Initiatives!$G$8=1)+M84*(Initiatives!$H$8=1)+M98*(Initiatives!$I$8=1)+M112*(Initiatives!$J$8=1)+M126*(Initiatives!$K$8=1)+M140*(Initiatives!$L$8=1)+M154*(Initiatives!$M$8=1)+M168*(Initiatives!$N$8=1)+M182*(Initiatives!$O$8=1)</f>
+        <v>6110274176.73496</v>
       </c>
       <c r="N190" s="8" t="n">
-        <f aca="false">N14*(1-Initiatives!$C$8)+N28*(1-Initiatives!$D$8)+N42*(1-Initiatives!$E$8)+N56*(1-Initiatives!$F$8)+N70*(1-Initiatives!$G$8)+N84*(1-Initiatives!$H$8)+N98*(1-Initiatives!$I$8)+N112*(1-Initiatives!$J$8)+N126*(1-Initiatives!$K$8)+N140*(1-Initiatives!$L$8)+N154*(1-Initiatives!$M$8)+N168*(1-Initiatives!$N$8)+N182*(1-Initiatives!$O$8)</f>
-        <v>10195808742.3138</v>
+        <f aca="false">N14*(Initiatives!$C$8=1)+N28*(Initiatives!$D$8=1)+N42*(Initiatives!$E$8=1)+N56*(Initiatives!$F$8=1)+N70*(Initiatives!$G$8=1)+N84*(Initiatives!$H$8=1)+N98*(Initiatives!$I$8=1)+N112*(Initiatives!$J$8=1)+N126*(Initiatives!$K$8=1)+N140*(Initiatives!$L$8=1)+N154*(Initiatives!$M$8=1)+N168*(Initiatives!$N$8=1)+N182*(Initiatives!$O$8=1)</f>
+        <v>10133172742.4303</v>
       </c>
       <c r="O190" s="8" t="n">
-        <f aca="false">O14*(1-Initiatives!$C$8)+O28*(1-Initiatives!$D$8)+O42*(1-Initiatives!$E$8)+O56*(1-Initiatives!$F$8)+O70*(1-Initiatives!$G$8)+O84*(1-Initiatives!$H$8)+O98*(1-Initiatives!$I$8)+O112*(1-Initiatives!$J$8)+O126*(1-Initiatives!$K$8)+O140*(1-Initiatives!$L$8)+O154*(1-Initiatives!$M$8)+O168*(1-Initiatives!$N$8)+O182*(1-Initiatives!$O$8)</f>
-        <v>9830944741.69652</v>
+        <f aca="false">O14*(Initiatives!$C$8=1)+O28*(Initiatives!$D$8=1)+O42*(Initiatives!$E$8=1)+O56*(Initiatives!$F$8=1)+O70*(Initiatives!$G$8=1)+O84*(Initiatives!$H$8=1)+O98*(Initiatives!$I$8=1)+O112*(Initiatives!$J$8=1)+O126*(Initiatives!$K$8=1)+O140*(Initiatives!$L$8=1)+O154*(Initiatives!$M$8=1)+O168*(Initiatives!$N$8=1)+O182*(Initiatives!$O$8=1)</f>
+        <v>9768875246.47958</v>
       </c>
       <c r="P190" s="8" t="n">
-        <f aca="false">P14*(1-Initiatives!$C$8)+P28*(1-Initiatives!$D$8)+P42*(1-Initiatives!$E$8)+P56*(1-Initiatives!$F$8)+P70*(1-Initiatives!$G$8)+P84*(1-Initiatives!$H$8)+P98*(1-Initiatives!$I$8)+P112*(1-Initiatives!$J$8)+P126*(1-Initiatives!$K$8)+P140*(1-Initiatives!$L$8)+P154*(1-Initiatives!$M$8)+P168*(1-Initiatives!$N$8)+P182*(1-Initiatives!$O$8)</f>
-        <v>9735173106.45962</v>
+        <f aca="false">P14*(Initiatives!$C$8=1)+P28*(Initiatives!$D$8=1)+P42*(Initiatives!$E$8=1)+P56*(Initiatives!$F$8=1)+P70*(Initiatives!$G$8=1)+P84*(Initiatives!$H$8=1)+P98*(Initiatives!$I$8=1)+P112*(Initiatives!$J$8=1)+P126*(Initiatives!$K$8=1)+P140*(Initiatives!$L$8=1)+P154*(Initiatives!$M$8=1)+P168*(Initiatives!$N$8=1)+P182*(Initiatives!$O$8=1)</f>
+        <v>9673666094.76317</v>
       </c>
       <c r="Q190" s="8" t="n">
-        <f aca="false">Q14*(1-Initiatives!$C$8)+Q28*(1-Initiatives!$D$8)+Q42*(1-Initiatives!$E$8)+Q56*(1-Initiatives!$F$8)+Q70*(1-Initiatives!$G$8)+Q84*(1-Initiatives!$H$8)+Q98*(1-Initiatives!$I$8)+Q112*(1-Initiatives!$J$8)+Q126*(1-Initiatives!$K$8)+Q140*(1-Initiatives!$L$8)+Q154*(1-Initiatives!$M$8)+Q168*(1-Initiatives!$N$8)+Q182*(1-Initiatives!$O$8)</f>
-        <v>9640433184.64252</v>
+        <f aca="false">Q14*(Initiatives!$C$8=1)+Q28*(Initiatives!$D$8=1)+Q42*(Initiatives!$E$8=1)+Q56*(Initiatives!$F$8=1)+Q70*(Initiatives!$G$8=1)+Q84*(Initiatives!$H$8=1)+Q98*(Initiatives!$I$8=1)+Q112*(Initiatives!$J$8=1)+Q126*(Initiatives!$K$8=1)+Q140*(Initiatives!$L$8=1)+Q154*(Initiatives!$M$8=1)+Q168*(Initiatives!$N$8=1)+Q182*(Initiatives!$O$8=1)</f>
+        <v>9579484641.92066</v>
       </c>
       <c r="R190" s="8" t="n">
-        <f aca="false">R14*(1-Initiatives!$C$8)+R28*(1-Initiatives!$D$8)+R42*(1-Initiatives!$E$8)+R56*(1-Initiatives!$F$8)+R70*(1-Initiatives!$G$8)+R84*(1-Initiatives!$H$8)+R98*(1-Initiatives!$I$8)+R112*(1-Initiatives!$J$8)+R126*(1-Initiatives!$K$8)+R140*(1-Initiatives!$L$8)+R154*(1-Initiatives!$M$8)+R168*(1-Initiatives!$N$8)+R182*(1-Initiatives!$O$8)</f>
-        <v>9546688054.41627</v>
+        <f aca="false">R14*(Initiatives!$C$8=1)+R28*(Initiatives!$D$8=1)+R42*(Initiatives!$E$8=1)+R56*(Initiatives!$F$8=1)+R70*(Initiatives!$G$8=1)+R84*(Initiatives!$H$8=1)+R98*(Initiatives!$I$8=1)+R112*(Initiatives!$J$8=1)+R126*(Initiatives!$K$8=1)+R140*(Initiatives!$L$8=1)+R154*(Initiatives!$M$8=1)+R168*(Initiatives!$N$8=1)+R182*(Initiatives!$O$8=1)</f>
+        <v>9486293973.26879</v>
       </c>
       <c r="S190" s="8" t="n">
-        <f aca="false">S14*(1-Initiatives!$C$8)+S28*(1-Initiatives!$D$8)+S42*(1-Initiatives!$E$8)+S56*(1-Initiatives!$F$8)+S70*(1-Initiatives!$G$8)+S84*(1-Initiatives!$H$8)+S98*(1-Initiatives!$I$8)+S112*(1-Initiatives!$J$8)+S126*(1-Initiatives!$K$8)+S140*(1-Initiatives!$L$8)+S154*(1-Initiatives!$M$8)+S168*(1-Initiatives!$N$8)+S182*(1-Initiatives!$O$8)</f>
-        <v>9453903921.80989</v>
+        <f aca="false">S14*(Initiatives!$C$8=1)+S28*(Initiatives!$D$8=1)+S42*(Initiatives!$E$8=1)+S56*(Initiatives!$F$8=1)+S70*(Initiatives!$G$8=1)+S84*(Initiatives!$H$8=1)+S98*(Initiatives!$I$8=1)+S112*(Initiatives!$J$8=1)+S126*(Initiatives!$K$8=1)+S140*(Initiatives!$L$8=1)+S154*(Initiatives!$M$8=1)+S168*(Initiatives!$N$8=1)+S182*(Initiatives!$O$8=1)</f>
+        <v>9394060302.51197</v>
       </c>
       <c r="T190" s="8" t="n">
-        <f aca="false">T14*(1-Initiatives!$C$8)+T28*(1-Initiatives!$D$8)+T42*(1-Initiatives!$E$8)+T56*(1-Initiatives!$F$8)+T70*(1-Initiatives!$G$8)+T84*(1-Initiatives!$H$8)+T98*(1-Initiatives!$I$8)+T112*(1-Initiatives!$J$8)+T126*(1-Initiatives!$K$8)+T140*(1-Initiatives!$L$8)+T154*(1-Initiatives!$M$8)+T168*(1-Initiatives!$N$8)+T182*(1-Initiatives!$O$8)</f>
-        <v>9362049848.14285</v>
+        <f aca="false">T14*(Initiatives!$C$8=1)+T28*(Initiatives!$D$8=1)+T42*(Initiatives!$E$8=1)+T56*(Initiatives!$F$8=1)+T70*(Initiatives!$G$8=1)+T84*(Initiatives!$H$8=1)+T98*(Initiatives!$I$8=1)+T112*(Initiatives!$J$8=1)+T126*(Initiatives!$K$8=1)+T140*(Initiatives!$L$8=1)+T154*(Initiatives!$M$8=1)+T168*(Initiatives!$N$8=1)+T182*(Initiatives!$O$8=1)</f>
+        <v>9302752699.15915</v>
       </c>
       <c r="U190" s="8" t="n">
-        <f aca="false">U14*(1-Initiatives!$C$8)+U28*(1-Initiatives!$D$8)+U42*(1-Initiatives!$E$8)+U56*(1-Initiatives!$F$8)+U70*(1-Initiatives!$G$8)+U84*(1-Initiatives!$H$8)+U98*(1-Initiatives!$I$8)+U112*(1-Initiatives!$J$8)+U126*(1-Initiatives!$K$8)+U140*(1-Initiatives!$L$8)+U154*(1-Initiatives!$M$8)+U168*(1-Initiatives!$N$8)+U182*(1-Initiatives!$O$8)</f>
-        <v>9271097500.49486</v>
+        <f aca="false">U14*(Initiatives!$C$8=1)+U28*(Initiatives!$D$8=1)+U42*(Initiatives!$E$8=1)+U56*(Initiatives!$F$8=1)+U70*(Initiatives!$G$8=1)+U84*(Initiatives!$H$8=1)+U98*(Initiatives!$I$8=1)+U112*(Initiatives!$J$8=1)+U126*(Initiatives!$K$8=1)+U140*(Initiatives!$L$8=1)+U154*(Initiatives!$M$8=1)+U168*(Initiatives!$N$8=1)+U182*(Initiatives!$O$8=1)</f>
+        <v>9212342838.97838</v>
       </c>
       <c r="V190" s="8" t="n">
-        <f aca="false">V14*(1-Initiatives!$C$8)+V28*(1-Initiatives!$D$8)+V42*(1-Initiatives!$E$8)+V56*(1-Initiatives!$F$8)+V70*(1-Initiatives!$G$8)+V84*(1-Initiatives!$H$8)+V98*(1-Initiatives!$I$8)+V112*(1-Initiatives!$J$8)+V126*(1-Initiatives!$K$8)+V140*(1-Initiatives!$L$8)+V154*(1-Initiatives!$M$8)+V168*(1-Initiatives!$N$8)+V182*(1-Initiatives!$O$8)</f>
-        <v>9181020923.28772</v>
+        <f aca="false">V14*(Initiatives!$C$8=1)+V28*(Initiatives!$D$8=1)+V42*(Initiatives!$E$8=1)+V56*(Initiatives!$F$8=1)+V70*(Initiatives!$G$8=1)+V84*(Initiatives!$H$8=1)+V98*(Initiatives!$I$8=1)+V112*(Initiatives!$J$8=1)+V126*(Initiatives!$K$8=1)+V140*(Initiatives!$L$8=1)+V154*(Initiatives!$M$8=1)+V168*(Initiatives!$N$8=1)+V182*(Initiatives!$O$8=1)</f>
+        <v>9122804775.56366</v>
       </c>
       <c r="W190" s="8" t="n">
-        <f aca="false">W14*(1-Initiatives!$C$8)+W28*(1-Initiatives!$D$8)+W42*(1-Initiatives!$E$8)+W56*(1-Initiatives!$F$8)+W70*(1-Initiatives!$G$8)+W84*(1-Initiatives!$H$8)+W98*(1-Initiatives!$I$8)+W112*(1-Initiatives!$J$8)+W126*(1-Initiatives!$K$8)+W140*(1-Initiatives!$L$8)+W154*(1-Initiatives!$M$8)+W168*(1-Initiatives!$N$8)+W182*(1-Initiatives!$O$8)</f>
-        <v>9091796329.21429</v>
+        <f aca="false">W14*(Initiatives!$C$8=1)+W28*(Initiatives!$D$8=1)+W42*(Initiatives!$E$8=1)+W56*(Initiatives!$F$8=1)+W70*(Initiatives!$G$8=1)+W84*(Initiatives!$H$8=1)+W98*(Initiatives!$I$8=1)+W112*(Initiatives!$J$8=1)+W126*(Initiatives!$K$8=1)+W140*(Initiatives!$L$8=1)+W154*(Initiatives!$M$8=1)+W168*(Initiatives!$N$8=1)+W182*(Initiatives!$O$8=1)</f>
+        <v>9034114731.24932</v>
       </c>
       <c r="X190" s="8" t="n">
-        <f aca="false">X14*(1-Initiatives!$C$8)+X28*(1-Initiatives!$D$8)+X42*(1-Initiatives!$E$8)+X56*(1-Initiatives!$F$8)+X70*(1-Initiatives!$G$8)+X84*(1-Initiatives!$H$8)+X98*(1-Initiatives!$I$8)+X112*(1-Initiatives!$J$8)+X126*(1-Initiatives!$K$8)+X140*(1-Initiatives!$L$8)+X154*(1-Initiatives!$M$8)+X168*(1-Initiatives!$N$8)+X182*(1-Initiatives!$O$8)</f>
-        <v>9003401907.8967</v>
+        <f aca="false">X14*(Initiatives!$C$8=1)+X28*(Initiatives!$D$8=1)+X42*(Initiatives!$E$8=1)+X56*(Initiatives!$F$8=1)+X70*(Initiatives!$G$8=1)+X84*(Initiatives!$H$8=1)+X98*(Initiatives!$I$8=1)+X112*(Initiatives!$J$8=1)+X126*(Initiatives!$K$8=1)+X140*(Initiatives!$L$8=1)+X154*(Initiatives!$M$8=1)+X168*(Initiatives!$N$8=1)+X182*(Initiatives!$O$8=1)</f>
+        <v>8946250905.75393</v>
       </c>
       <c r="Y190" s="8" t="n">
-        <f aca="false">Y14*(1-Initiatives!$C$8)+Y28*(1-Initiatives!$D$8)+Y42*(1-Initiatives!$E$8)+Y56*(1-Initiatives!$F$8)+Y70*(1-Initiatives!$G$8)+Y84*(1-Initiatives!$H$8)+Y98*(1-Initiatives!$I$8)+Y112*(1-Initiatives!$J$8)+Y126*(1-Initiatives!$K$8)+Y140*(1-Initiatives!$L$8)+Y154*(1-Initiatives!$M$8)+Y168*(1-Initiatives!$N$8)+Y182*(1-Initiatives!$O$8)</f>
-        <v>8915817650.79102</v>
+        <f aca="false">Y14*(Initiatives!$C$8=1)+Y28*(Initiatives!$D$8=1)+Y42*(Initiatives!$E$8=1)+Y56*(Initiatives!$F$8=1)+Y70*(Initiatives!$G$8=1)+Y84*(Initiatives!$H$8=1)+Y98*(Initiatives!$I$8=1)+Y112*(Initiatives!$J$8=1)+Y126*(Initiatives!$K$8=1)+Y140*(Initiatives!$L$8=1)+Y154*(Initiatives!$M$8=1)+Y168*(Initiatives!$N$8=1)+Y182*(Initiatives!$O$8=1)</f>
+        <v>8859193301.07087</v>
       </c>
       <c r="Z190" s="8" t="n">
-        <f aca="false">Z14*(1-Initiatives!$C$8)+Z28*(1-Initiatives!$D$8)+Z42*(1-Initiatives!$E$8)+Z56*(1-Initiatives!$F$8)+Z70*(1-Initiatives!$G$8)+Z84*(1-Initiatives!$H$8)+Z98*(1-Initiatives!$I$8)+Z112*(1-Initiatives!$J$8)+Z126*(1-Initiatives!$K$8)+Z140*(1-Initiatives!$L$8)+Z154*(1-Initiatives!$M$8)+Z168*(1-Initiatives!$N$8)+Z182*(1-Initiatives!$O$8)</f>
-        <v>8829025190.9786</v>
+        <f aca="false">Z14*(Initiatives!$C$8=1)+Z28*(Initiatives!$D$8=1)+Z42*(Initiatives!$E$8=1)+Z56*(Initiatives!$F$8=1)+Z70*(Initiatives!$G$8=1)+Z84*(Initiatives!$H$8=1)+Z98*(Initiatives!$I$8=1)+Z112*(Initiatives!$J$8=1)+Z126*(Initiatives!$K$8=1)+Z140*(Initiatives!$L$8=1)+Z154*(Initiatives!$M$8=1)+Z168*(Initiatives!$N$8=1)+Z182*(Initiatives!$O$8=1)</f>
+        <v>8772923561.24605</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24696,99 +24699,99 @@
       </c>
       <c r="B191" s="4"/>
       <c r="C191" s="8" t="n">
-        <f aca="false">C15*(1-Initiatives!$C$8)+C29*(1-Initiatives!$D$8)+C43*(1-Initiatives!$E$8)+C57*(1-Initiatives!$F$8)+C71*(1-Initiatives!$G$8)+C85*(1-Initiatives!$H$8)+C99*(1-Initiatives!$I$8)+C113*(1-Initiatives!$J$8)+C127*(1-Initiatives!$K$8)+C141*(1-Initiatives!$L$8)+C155*(1-Initiatives!$M$8)+C169*(1-Initiatives!$N$8)+C183*(1-Initiatives!$O$8)</f>
+        <f aca="false">C15*(Initiatives!$C$8=1)+C29*(Initiatives!$D$8=1)+C43*(Initiatives!$E$8=1)+C57*(Initiatives!$F$8=1)+C71*(Initiatives!$G$8=1)+C85*(Initiatives!$H$8=1)+C99*(Initiatives!$I$8=1)+C113*(Initiatives!$J$8=1)+C127*(Initiatives!$K$8=1)+C141*(Initiatives!$L$8=1)+C155*(Initiatives!$M$8=1)+C169*(Initiatives!$N$8=1)+C183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="D191" s="8" t="n">
-        <f aca="false">D15*(1-Initiatives!$C$8)+D29*(1-Initiatives!$D$8)+D43*(1-Initiatives!$E$8)+D57*(1-Initiatives!$F$8)+D71*(1-Initiatives!$G$8)+D85*(1-Initiatives!$H$8)+D99*(1-Initiatives!$I$8)+D113*(1-Initiatives!$J$8)+D127*(1-Initiatives!$K$8)+D141*(1-Initiatives!$L$8)+D155*(1-Initiatives!$M$8)+D169*(1-Initiatives!$N$8)+D183*(1-Initiatives!$O$8)</f>
+        <f aca="false">D15*(Initiatives!$C$8=1)+D29*(Initiatives!$D$8=1)+D43*(Initiatives!$E$8=1)+D57*(Initiatives!$F$8=1)+D71*(Initiatives!$G$8=1)+D85*(Initiatives!$H$8=1)+D99*(Initiatives!$I$8=1)+D113*(Initiatives!$J$8=1)+D127*(Initiatives!$K$8=1)+D141*(Initiatives!$L$8=1)+D155*(Initiatives!$M$8=1)+D169*(Initiatives!$N$8=1)+D183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="E191" s="8" t="n">
-        <f aca="false">E15*(1-Initiatives!$C$8)+E29*(1-Initiatives!$D$8)+E43*(1-Initiatives!$E$8)+E57*(1-Initiatives!$F$8)+E71*(1-Initiatives!$G$8)+E85*(1-Initiatives!$H$8)+E99*(1-Initiatives!$I$8)+E113*(1-Initiatives!$J$8)+E127*(1-Initiatives!$K$8)+E141*(1-Initiatives!$L$8)+E155*(1-Initiatives!$M$8)+E169*(1-Initiatives!$N$8)+E183*(1-Initiatives!$O$8)</f>
+        <f aca="false">E15*(Initiatives!$C$8=1)+E29*(Initiatives!$D$8=1)+E43*(Initiatives!$E$8=1)+E57*(Initiatives!$F$8=1)+E71*(Initiatives!$G$8=1)+E85*(Initiatives!$H$8=1)+E99*(Initiatives!$I$8=1)+E113*(Initiatives!$J$8=1)+E127*(Initiatives!$K$8=1)+E141*(Initiatives!$L$8=1)+E155*(Initiatives!$M$8=1)+E169*(Initiatives!$N$8=1)+E183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="F191" s="8" t="n">
-        <f aca="false">F15*(1-Initiatives!$C$8)+F29*(1-Initiatives!$D$8)+F43*(1-Initiatives!$E$8)+F57*(1-Initiatives!$F$8)+F71*(1-Initiatives!$G$8)+F85*(1-Initiatives!$H$8)+F99*(1-Initiatives!$I$8)+F113*(1-Initiatives!$J$8)+F127*(1-Initiatives!$K$8)+F141*(1-Initiatives!$L$8)+F155*(1-Initiatives!$M$8)+F169*(1-Initiatives!$N$8)+F183*(1-Initiatives!$O$8)</f>
+        <f aca="false">F15*(Initiatives!$C$8=1)+F29*(Initiatives!$D$8=1)+F43*(Initiatives!$E$8=1)+F57*(Initiatives!$F$8=1)+F71*(Initiatives!$G$8=1)+F85*(Initiatives!$H$8=1)+F99*(Initiatives!$I$8=1)+F113*(Initiatives!$J$8=1)+F127*(Initiatives!$K$8=1)+F141*(Initiatives!$L$8=1)+F155*(Initiatives!$M$8=1)+F169*(Initiatives!$N$8=1)+F183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="G191" s="8" t="n">
-        <f aca="false">G15*(1-Initiatives!$C$8)+G29*(1-Initiatives!$D$8)+G43*(1-Initiatives!$E$8)+G57*(1-Initiatives!$F$8)+G71*(1-Initiatives!$G$8)+G85*(1-Initiatives!$H$8)+G99*(1-Initiatives!$I$8)+G113*(1-Initiatives!$J$8)+G127*(1-Initiatives!$K$8)+G141*(1-Initiatives!$L$8)+G155*(1-Initiatives!$M$8)+G169*(1-Initiatives!$N$8)+G183*(1-Initiatives!$O$8)</f>
+        <f aca="false">G15*(Initiatives!$C$8=1)+G29*(Initiatives!$D$8=1)+G43*(Initiatives!$E$8=1)+G57*(Initiatives!$F$8=1)+G71*(Initiatives!$G$8=1)+G85*(Initiatives!$H$8=1)+G99*(Initiatives!$I$8=1)+G113*(Initiatives!$J$8=1)+G127*(Initiatives!$K$8=1)+G141*(Initiatives!$L$8=1)+G155*(Initiatives!$M$8=1)+G169*(Initiatives!$N$8=1)+G183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="H191" s="8" t="n">
-        <f aca="false">H15*(1-Initiatives!$C$8)+H29*(1-Initiatives!$D$8)+H43*(1-Initiatives!$E$8)+H57*(1-Initiatives!$F$8)+H71*(1-Initiatives!$G$8)+H85*(1-Initiatives!$H$8)+H99*(1-Initiatives!$I$8)+H113*(1-Initiatives!$J$8)+H127*(1-Initiatives!$K$8)+H141*(1-Initiatives!$L$8)+H155*(1-Initiatives!$M$8)+H169*(1-Initiatives!$N$8)+H183*(1-Initiatives!$O$8)</f>
+        <f aca="false">H15*(Initiatives!$C$8=1)+H29*(Initiatives!$D$8=1)+H43*(Initiatives!$E$8=1)+H57*(Initiatives!$F$8=1)+H71*(Initiatives!$G$8=1)+H85*(Initiatives!$H$8=1)+H99*(Initiatives!$I$8=1)+H113*(Initiatives!$J$8=1)+H127*(Initiatives!$K$8=1)+H141*(Initiatives!$L$8=1)+H155*(Initiatives!$M$8=1)+H169*(Initiatives!$N$8=1)+H183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="I191" s="8" t="n">
-        <f aca="false">I15*(1-Initiatives!$C$8)+I29*(1-Initiatives!$D$8)+I43*(1-Initiatives!$E$8)+I57*(1-Initiatives!$F$8)+I71*(1-Initiatives!$G$8)+I85*(1-Initiatives!$H$8)+I99*(1-Initiatives!$I$8)+I113*(1-Initiatives!$J$8)+I127*(1-Initiatives!$K$8)+I141*(1-Initiatives!$L$8)+I155*(1-Initiatives!$M$8)+I169*(1-Initiatives!$N$8)+I183*(1-Initiatives!$O$8)</f>
+        <f aca="false">I15*(Initiatives!$C$8=1)+I29*(Initiatives!$D$8=1)+I43*(Initiatives!$E$8=1)+I57*(Initiatives!$F$8=1)+I71*(Initiatives!$G$8=1)+I85*(Initiatives!$H$8=1)+I99*(Initiatives!$I$8=1)+I113*(Initiatives!$J$8=1)+I127*(Initiatives!$K$8=1)+I141*(Initiatives!$L$8=1)+I155*(Initiatives!$M$8=1)+I169*(Initiatives!$N$8=1)+I183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="J191" s="8" t="n">
-        <f aca="false">J15*(1-Initiatives!$C$8)+J29*(1-Initiatives!$D$8)+J43*(1-Initiatives!$E$8)+J57*(1-Initiatives!$F$8)+J71*(1-Initiatives!$G$8)+J85*(1-Initiatives!$H$8)+J99*(1-Initiatives!$I$8)+J113*(1-Initiatives!$J$8)+J127*(1-Initiatives!$K$8)+J141*(1-Initiatives!$L$8)+J155*(1-Initiatives!$M$8)+J169*(1-Initiatives!$N$8)+J183*(1-Initiatives!$O$8)</f>
+        <f aca="false">J15*(Initiatives!$C$8=1)+J29*(Initiatives!$D$8=1)+J43*(Initiatives!$E$8=1)+J57*(Initiatives!$F$8=1)+J71*(Initiatives!$G$8=1)+J85*(Initiatives!$H$8=1)+J99*(Initiatives!$I$8=1)+J113*(Initiatives!$J$8=1)+J127*(Initiatives!$K$8=1)+J141*(Initiatives!$L$8=1)+J155*(Initiatives!$M$8=1)+J169*(Initiatives!$N$8=1)+J183*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="K191" s="8" t="n">
-        <f aca="false">K15*(1-Initiatives!$C$8)+K29*(1-Initiatives!$D$8)+K43*(1-Initiatives!$E$8)+K57*(1-Initiatives!$F$8)+K71*(1-Initiatives!$G$8)+K85*(1-Initiatives!$H$8)+K99*(1-Initiatives!$I$8)+K113*(1-Initiatives!$J$8)+K127*(1-Initiatives!$K$8)+K141*(1-Initiatives!$L$8)+K155*(1-Initiatives!$M$8)+K169*(1-Initiatives!$N$8)+K183*(1-Initiatives!$O$8)</f>
+        <f aca="false">K15*(Initiatives!$C$8=1)+K29*(Initiatives!$D$8=1)+K43*(Initiatives!$E$8=1)+K57*(Initiatives!$F$8=1)+K71*(Initiatives!$G$8=1)+K85*(Initiatives!$H$8=1)+K99*(Initiatives!$I$8=1)+K113*(Initiatives!$J$8=1)+K127*(Initiatives!$K$8=1)+K141*(Initiatives!$L$8=1)+K155*(Initiatives!$M$8=1)+K169*(Initiatives!$N$8=1)+K183*(Initiatives!$O$8=1)</f>
         <v>24330240</v>
       </c>
       <c r="L191" s="8" t="n">
-        <f aca="false">L15*(1-Initiatives!$C$8)+L29*(1-Initiatives!$D$8)+L43*(1-Initiatives!$E$8)+L57*(1-Initiatives!$F$8)+L71*(1-Initiatives!$G$8)+L85*(1-Initiatives!$H$8)+L99*(1-Initiatives!$I$8)+L113*(1-Initiatives!$J$8)+L127*(1-Initiatives!$K$8)+L141*(1-Initiatives!$L$8)+L155*(1-Initiatives!$M$8)+L169*(1-Initiatives!$N$8)+L183*(1-Initiatives!$O$8)</f>
+        <f aca="false">L15*(Initiatives!$C$8=1)+L29*(Initiatives!$D$8=1)+L43*(Initiatives!$E$8=1)+L57*(Initiatives!$F$8=1)+L71*(Initiatives!$G$8=1)+L85*(Initiatives!$H$8=1)+L99*(Initiatives!$I$8=1)+L113*(Initiatives!$J$8=1)+L127*(Initiatives!$K$8=1)+L141*(Initiatives!$L$8=1)+L155*(Initiatives!$M$8=1)+L169*(Initiatives!$N$8=1)+L183*(Initiatives!$O$8=1)</f>
         <v>48405012.48</v>
       </c>
       <c r="M191" s="8" t="n">
-        <f aca="false">M15*(1-Initiatives!$C$8)+M29*(1-Initiatives!$D$8)+M43*(1-Initiatives!$E$8)+M57*(1-Initiatives!$F$8)+M71*(1-Initiatives!$G$8)+M85*(1-Initiatives!$H$8)+M99*(1-Initiatives!$I$8)+M113*(1-Initiatives!$J$8)+M127*(1-Initiatives!$K$8)+M141*(1-Initiatives!$L$8)+M155*(1-Initiatives!$M$8)+M169*(1-Initiatives!$N$8)+M183*(1-Initiatives!$O$8)</f>
+        <f aca="false">M15*(Initiatives!$C$8=1)+M29*(Initiatives!$D$8=1)+M43*(Initiatives!$E$8=1)+M57*(Initiatives!$F$8=1)+M71*(Initiatives!$G$8=1)+M85*(Initiatives!$H$8=1)+M99*(Initiatives!$I$8=1)+M113*(Initiatives!$J$8=1)+M127*(Initiatives!$K$8=1)+M141*(Initiatives!$L$8=1)+M155*(Initiatives!$M$8=1)+M169*(Initiatives!$N$8=1)+M183*(Initiatives!$O$8=1)</f>
         <v>72226999.84896</v>
       </c>
       <c r="N191" s="8" t="n">
-        <f aca="false">N15*(1-Initiatives!$C$8)+N29*(1-Initiatives!$D$8)+N43*(1-Initiatives!$E$8)+N57*(1-Initiatives!$F$8)+N71*(1-Initiatives!$G$8)+N85*(1-Initiatives!$H$8)+N99*(1-Initiatives!$I$8)+N113*(1-Initiatives!$J$8)+N127*(1-Initiatives!$K$8)+N141*(1-Initiatives!$L$8)+N155*(1-Initiatives!$M$8)+N169*(1-Initiatives!$N$8)+N183*(1-Initiatives!$O$8)</f>
+        <f aca="false">N15*(Initiatives!$C$8=1)+N29*(Initiatives!$D$8=1)+N43*(Initiatives!$E$8=1)+N57*(Initiatives!$F$8=1)+N71*(Initiatives!$G$8=1)+N85*(Initiatives!$H$8=1)+N99*(Initiatives!$I$8=1)+N113*(Initiatives!$J$8=1)+N127*(Initiatives!$K$8=1)+N141*(Initiatives!$L$8=1)+N155*(Initiatives!$M$8=1)+N169*(Initiatives!$N$8=1)+N183*(Initiatives!$O$8=1)</f>
         <v>95798856.3505459</v>
       </c>
       <c r="O191" s="8" t="n">
-        <f aca="false">O15*(1-Initiatives!$C$8)+O29*(1-Initiatives!$D$8)+O43*(1-Initiatives!$E$8)+O57*(1-Initiatives!$F$8)+O71*(1-Initiatives!$G$8)+O85*(1-Initiatives!$H$8)+O99*(1-Initiatives!$I$8)+O113*(1-Initiatives!$J$8)+O127*(1-Initiatives!$K$8)+O141*(1-Initiatives!$L$8)+O155*(1-Initiatives!$M$8)+O169*(1-Initiatives!$N$8)+O183*(1-Initiatives!$O$8)</f>
+        <f aca="false">O15*(Initiatives!$C$8=1)+O29*(Initiatives!$D$8=1)+O43*(Initiatives!$E$8=1)+O57*(Initiatives!$F$8=1)+O71*(Initiatives!$G$8=1)+O85*(Initiatives!$H$8=1)+O99*(Initiatives!$I$8=1)+O113*(Initiatives!$J$8=1)+O127*(Initiatives!$K$8=1)+O141*(Initiatives!$L$8=1)+O155*(Initiatives!$M$8=1)+O169*(Initiatives!$N$8=1)+O183*(Initiatives!$O$8=1)</f>
         <v>94792968.3588652</v>
       </c>
       <c r="P191" s="8" t="n">
-        <f aca="false">P15*(1-Initiatives!$C$8)+P29*(1-Initiatives!$D$8)+P43*(1-Initiatives!$E$8)+P57*(1-Initiatives!$F$8)+P71*(1-Initiatives!$G$8)+P85*(1-Initiatives!$H$8)+P99*(1-Initiatives!$I$8)+P113*(1-Initiatives!$J$8)+P127*(1-Initiatives!$K$8)+P141*(1-Initiatives!$L$8)+P155*(1-Initiatives!$M$8)+P169*(1-Initiatives!$N$8)+P183*(1-Initiatives!$O$8)</f>
+        <f aca="false">P15*(Initiatives!$C$8=1)+P29*(Initiatives!$D$8=1)+P43*(Initiatives!$E$8=1)+P57*(Initiatives!$F$8=1)+P71*(Initiatives!$G$8=1)+P85*(Initiatives!$H$8=1)+P99*(Initiatives!$I$8=1)+P113*(Initiatives!$J$8=1)+P127*(Initiatives!$K$8=1)+P141*(Initiatives!$L$8=1)+P155*(Initiatives!$M$8=1)+P169*(Initiatives!$N$8=1)+P183*(Initiatives!$O$8=1)</f>
         <v>93797642.1910971</v>
       </c>
       <c r="Q191" s="8" t="n">
-        <f aca="false">Q15*(1-Initiatives!$C$8)+Q29*(1-Initiatives!$D$8)+Q43*(1-Initiatives!$E$8)+Q57*(1-Initiatives!$F$8)+Q71*(1-Initiatives!$G$8)+Q85*(1-Initiatives!$H$8)+Q99*(1-Initiatives!$I$8)+Q113*(1-Initiatives!$J$8)+Q127*(1-Initiatives!$K$8)+Q141*(1-Initiatives!$L$8)+Q155*(1-Initiatives!$M$8)+Q169*(1-Initiatives!$N$8)+Q183*(1-Initiatives!$O$8)</f>
+        <f aca="false">Q15*(Initiatives!$C$8=1)+Q29*(Initiatives!$D$8=1)+Q43*(Initiatives!$E$8=1)+Q57*(Initiatives!$F$8=1)+Q71*(Initiatives!$G$8=1)+Q85*(Initiatives!$H$8=1)+Q99*(Initiatives!$I$8=1)+Q113*(Initiatives!$J$8=1)+Q127*(Initiatives!$K$8=1)+Q141*(Initiatives!$L$8=1)+Q155*(Initiatives!$M$8=1)+Q169*(Initiatives!$N$8=1)+Q183*(Initiatives!$O$8=1)</f>
         <v>92812766.9480906</v>
       </c>
       <c r="R191" s="8" t="n">
-        <f aca="false">R15*(1-Initiatives!$C$8)+R29*(1-Initiatives!$D$8)+R43*(1-Initiatives!$E$8)+R57*(1-Initiatives!$F$8)+R71*(1-Initiatives!$G$8)+R85*(1-Initiatives!$H$8)+R99*(1-Initiatives!$I$8)+R113*(1-Initiatives!$J$8)+R127*(1-Initiatives!$K$8)+R141*(1-Initiatives!$L$8)+R155*(1-Initiatives!$M$8)+R169*(1-Initiatives!$N$8)+R183*(1-Initiatives!$O$8)</f>
+        <f aca="false">R15*(Initiatives!$C$8=1)+R29*(Initiatives!$D$8=1)+R43*(Initiatives!$E$8=1)+R57*(Initiatives!$F$8=1)+R71*(Initiatives!$G$8=1)+R85*(Initiatives!$H$8=1)+R99*(Initiatives!$I$8=1)+R113*(Initiatives!$J$8=1)+R127*(Initiatives!$K$8=1)+R141*(Initiatives!$L$8=1)+R155*(Initiatives!$M$8=1)+R169*(Initiatives!$N$8=1)+R183*(Initiatives!$O$8=1)</f>
         <v>91838232.8951357</v>
       </c>
       <c r="S191" s="8" t="n">
-        <f aca="false">S15*(1-Initiatives!$C$8)+S29*(1-Initiatives!$D$8)+S43*(1-Initiatives!$E$8)+S57*(1-Initiatives!$F$8)+S71*(1-Initiatives!$G$8)+S85*(1-Initiatives!$H$8)+S99*(1-Initiatives!$I$8)+S113*(1-Initiatives!$J$8)+S127*(1-Initiatives!$K$8)+S141*(1-Initiatives!$L$8)+S155*(1-Initiatives!$M$8)+S169*(1-Initiatives!$N$8)+S183*(1-Initiatives!$O$8)</f>
+        <f aca="false">S15*(Initiatives!$C$8=1)+S29*(Initiatives!$D$8=1)+S43*(Initiatives!$E$8=1)+S57*(Initiatives!$F$8=1)+S71*(Initiatives!$G$8=1)+S85*(Initiatives!$H$8=1)+S99*(Initiatives!$I$8=1)+S113*(Initiatives!$J$8=1)+S127*(Initiatives!$K$8=1)+S141*(Initiatives!$L$8=1)+S155*(Initiatives!$M$8=1)+S169*(Initiatives!$N$8=1)+S183*(Initiatives!$O$8=1)</f>
         <v>90873931.4497368</v>
       </c>
       <c r="T191" s="8" t="n">
-        <f aca="false">T15*(1-Initiatives!$C$8)+T29*(1-Initiatives!$D$8)+T43*(1-Initiatives!$E$8)+T57*(1-Initiatives!$F$8)+T71*(1-Initiatives!$G$8)+T85*(1-Initiatives!$H$8)+T99*(1-Initiatives!$I$8)+T113*(1-Initiatives!$J$8)+T127*(1-Initiatives!$K$8)+T141*(1-Initiatives!$L$8)+T155*(1-Initiatives!$M$8)+T169*(1-Initiatives!$N$8)+T183*(1-Initiatives!$O$8)</f>
+        <f aca="false">T15*(Initiatives!$C$8=1)+T29*(Initiatives!$D$8=1)+T43*(Initiatives!$E$8=1)+T57*(Initiatives!$F$8=1)+T71*(Initiatives!$G$8=1)+T85*(Initiatives!$H$8=1)+T99*(Initiatives!$I$8=1)+T113*(Initiatives!$J$8=1)+T127*(Initiatives!$K$8=1)+T141*(Initiatives!$L$8=1)+T155*(Initiatives!$M$8=1)+T169*(Initiatives!$N$8=1)+T183*(Initiatives!$O$8=1)</f>
         <v>89919755.1695145</v>
       </c>
       <c r="U191" s="8" t="n">
-        <f aca="false">U15*(1-Initiatives!$C$8)+U29*(1-Initiatives!$D$8)+U43*(1-Initiatives!$E$8)+U57*(1-Initiatives!$F$8)+U71*(1-Initiatives!$G$8)+U85*(1-Initiatives!$H$8)+U99*(1-Initiatives!$I$8)+U113*(1-Initiatives!$J$8)+U127*(1-Initiatives!$K$8)+U141*(1-Initiatives!$L$8)+U155*(1-Initiatives!$M$8)+U169*(1-Initiatives!$N$8)+U183*(1-Initiatives!$O$8)</f>
+        <f aca="false">U15*(Initiatives!$C$8=1)+U29*(Initiatives!$D$8=1)+U43*(Initiatives!$E$8=1)+U57*(Initiatives!$F$8=1)+U71*(Initiatives!$G$8=1)+U85*(Initiatives!$H$8=1)+U99*(Initiatives!$I$8=1)+U113*(Initiatives!$J$8=1)+U127*(Initiatives!$K$8=1)+U141*(Initiatives!$L$8=1)+U155*(Initiatives!$M$8=1)+U169*(Initiatives!$N$8=1)+U183*(Initiatives!$O$8=1)</f>
         <v>88975597.7402346</v>
       </c>
       <c r="V191" s="8" t="n">
-        <f aca="false">V15*(1-Initiatives!$C$8)+V29*(1-Initiatives!$D$8)+V43*(1-Initiatives!$E$8)+V57*(1-Initiatives!$F$8)+V71*(1-Initiatives!$G$8)+V85*(1-Initiatives!$H$8)+V99*(1-Initiatives!$I$8)+V113*(1-Initiatives!$J$8)+V127*(1-Initiatives!$K$8)+V141*(1-Initiatives!$L$8)+V155*(1-Initiatives!$M$8)+V169*(1-Initiatives!$N$8)+V183*(1-Initiatives!$O$8)</f>
+        <f aca="false">V15*(Initiatives!$C$8=1)+V29*(Initiatives!$D$8=1)+V43*(Initiatives!$E$8=1)+V57*(Initiatives!$F$8=1)+V71*(Initiatives!$G$8=1)+V85*(Initiatives!$H$8=1)+V99*(Initiatives!$I$8=1)+V113*(Initiatives!$J$8=1)+V127*(Initiatives!$K$8=1)+V141*(Initiatives!$L$8=1)+V155*(Initiatives!$M$8=1)+V169*(Initiatives!$N$8=1)+V183*(Initiatives!$O$8=1)</f>
         <v>88041353.9639622</v>
       </c>
       <c r="W191" s="8" t="n">
-        <f aca="false">W15*(1-Initiatives!$C$8)+W29*(1-Initiatives!$D$8)+W43*(1-Initiatives!$E$8)+W57*(1-Initiatives!$F$8)+W71*(1-Initiatives!$G$8)+W85*(1-Initiatives!$H$8)+W99*(1-Initiatives!$I$8)+W113*(1-Initiatives!$J$8)+W127*(1-Initiatives!$K$8)+W141*(1-Initiatives!$L$8)+W155*(1-Initiatives!$M$8)+W169*(1-Initiatives!$N$8)+W183*(1-Initiatives!$O$8)</f>
+        <f aca="false">W15*(Initiatives!$C$8=1)+W29*(Initiatives!$D$8=1)+W43*(Initiatives!$E$8=1)+W57*(Initiatives!$F$8=1)+W71*(Initiatives!$G$8=1)+W85*(Initiatives!$H$8=1)+W99*(Initiatives!$I$8=1)+W113*(Initiatives!$J$8=1)+W127*(Initiatives!$K$8=1)+W141*(Initiatives!$L$8=1)+W155*(Initiatives!$M$8=1)+W169*(Initiatives!$N$8=1)+W183*(Initiatives!$O$8=1)</f>
         <v>87116919.7473406</v>
       </c>
       <c r="X191" s="8" t="n">
-        <f aca="false">X15*(1-Initiatives!$C$8)+X29*(1-Initiatives!$D$8)+X43*(1-Initiatives!$E$8)+X57*(1-Initiatives!$F$8)+X71*(1-Initiatives!$G$8)+X85*(1-Initiatives!$H$8)+X99*(1-Initiatives!$I$8)+X113*(1-Initiatives!$J$8)+X127*(1-Initiatives!$K$8)+X141*(1-Initiatives!$L$8)+X155*(1-Initiatives!$M$8)+X169*(1-Initiatives!$N$8)+X183*(1-Initiatives!$O$8)</f>
+        <f aca="false">X15*(Initiatives!$C$8=1)+X29*(Initiatives!$D$8=1)+X43*(Initiatives!$E$8=1)+X57*(Initiatives!$F$8=1)+X71*(Initiatives!$G$8=1)+X85*(Initiatives!$H$8=1)+X99*(Initiatives!$I$8=1)+X113*(Initiatives!$J$8=1)+X127*(Initiatives!$K$8=1)+X141*(Initiatives!$L$8=1)+X155*(Initiatives!$M$8=1)+X169*(Initiatives!$N$8=1)+X183*(Initiatives!$O$8=1)</f>
         <v>86202192.0899935</v>
       </c>
       <c r="Y191" s="8" t="n">
-        <f aca="false">Y15*(1-Initiatives!$C$8)+Y29*(1-Initiatives!$D$8)+Y43*(1-Initiatives!$E$8)+Y57*(1-Initiatives!$F$8)+Y71*(1-Initiatives!$G$8)+Y85*(1-Initiatives!$H$8)+Y99*(1-Initiatives!$I$8)+Y113*(1-Initiatives!$J$8)+Y127*(1-Initiatives!$K$8)+Y141*(1-Initiatives!$L$8)+Y155*(1-Initiatives!$M$8)+Y169*(1-Initiatives!$N$8)+Y183*(1-Initiatives!$O$8)</f>
+        <f aca="false">Y15*(Initiatives!$C$8=1)+Y29*(Initiatives!$D$8=1)+Y43*(Initiatives!$E$8=1)+Y57*(Initiatives!$F$8=1)+Y71*(Initiatives!$G$8=1)+Y85*(Initiatives!$H$8=1)+Y99*(Initiatives!$I$8=1)+Y113*(Initiatives!$J$8=1)+Y127*(Initiatives!$K$8=1)+Y141*(Initiatives!$L$8=1)+Y155*(Initiatives!$M$8=1)+Y169*(Initiatives!$N$8=1)+Y183*(Initiatives!$O$8=1)</f>
         <v>85297069.0730486</v>
       </c>
       <c r="Z191" s="8" t="n">
-        <f aca="false">Z15*(1-Initiatives!$C$8)+Z29*(1-Initiatives!$D$8)+Z43*(1-Initiatives!$E$8)+Z57*(1-Initiatives!$F$8)+Z71*(1-Initiatives!$G$8)+Z85*(1-Initiatives!$H$8)+Z99*(1-Initiatives!$I$8)+Z113*(1-Initiatives!$J$8)+Z127*(1-Initiatives!$K$8)+Z141*(1-Initiatives!$L$8)+Z155*(1-Initiatives!$M$8)+Z169*(1-Initiatives!$N$8)+Z183*(1-Initiatives!$O$8)</f>
+        <f aca="false">Z15*(Initiatives!$C$8=1)+Z29*(Initiatives!$D$8=1)+Z43*(Initiatives!$E$8=1)+Z57*(Initiatives!$F$8=1)+Z71*(Initiatives!$G$8=1)+Z85*(Initiatives!$H$8=1)+Z99*(Initiatives!$I$8=1)+Z113*(Initiatives!$J$8=1)+Z127*(Initiatives!$K$8=1)+Z141*(Initiatives!$L$8=1)+Z155*(Initiatives!$M$8=1)+Z169*(Initiatives!$N$8=1)+Z183*(Initiatives!$O$8=1)</f>
         <v>84401449.8477816</v>
       </c>
     </row>
@@ -24798,100 +24801,100 @@
       </c>
       <c r="B192" s="4"/>
       <c r="C192" s="8" t="n">
-        <f aca="false">C18*(1-Initiatives!$C$8)+C32*(1-Initiatives!$D$8)+C46*(1-Initiatives!$E$8)+C60*(1-Initiatives!$F$8)+C74*(1-Initiatives!$G$8)+C88*(1-Initiatives!$H$8)+C102*(1-Initiatives!$I$8)+C116*(1-Initiatives!$J$8)+C130*(1-Initiatives!$K$8)+C144*(1-Initiatives!$L$8)+C158*(1-Initiatives!$M$8)+C172*(1-Initiatives!$N$8)+C186*(1-Initiatives!$O$8)</f>
+        <f aca="false">C18*(Initiatives!$C$8=1)+C32*(Initiatives!$D$8=1)+C46*(Initiatives!$E$8=1)+C60*(Initiatives!$F$8=1)+C74*(Initiatives!$G$8=1)+C88*(Initiatives!$H$8=1)+C102*(Initiatives!$I$8=1)+C116*(Initiatives!$J$8=1)+C130*(Initiatives!$K$8=1)+C144*(Initiatives!$L$8=1)+C158*(Initiatives!$M$8=1)+C172*(Initiatives!$N$8=1)+C186*(Initiatives!$O$8=1)</f>
         <v>0</v>
       </c>
       <c r="D192" s="8" t="n">
-        <f aca="false">D18*(1-Initiatives!$C$8)+D32*(1-Initiatives!$D$8)+D46*(1-Initiatives!$E$8)+D60*(1-Initiatives!$F$8)+D74*(1-Initiatives!$G$8)+D88*(1-Initiatives!$H$8)+D102*(1-Initiatives!$I$8)+D116*(1-Initiatives!$J$8)+D130*(1-Initiatives!$K$8)+D144*(1-Initiatives!$L$8)+D158*(1-Initiatives!$M$8)+D172*(1-Initiatives!$N$8)+D186*(1-Initiatives!$O$8)</f>
+        <f aca="false">D18*(Initiatives!$C$8=1)+D32*(Initiatives!$D$8=1)+D46*(Initiatives!$E$8=1)+D60*(Initiatives!$F$8=1)+D74*(Initiatives!$G$8=1)+D88*(Initiatives!$H$8=1)+D102*(Initiatives!$I$8=1)+D116*(Initiatives!$J$8=1)+D130*(Initiatives!$K$8=1)+D144*(Initiatives!$L$8=1)+D158*(Initiatives!$M$8=1)+D172*(Initiatives!$N$8=1)+D186*(Initiatives!$O$8=1)</f>
         <v>-10597.5466666667</v>
       </c>
       <c r="E192" s="8" t="n">
-        <f aca="false">E18*(1-Initiatives!$C$8)+E32*(1-Initiatives!$D$8)+E46*(1-Initiatives!$E$8)+E60*(1-Initiatives!$F$8)+E74*(1-Initiatives!$G$8)+E88*(1-Initiatives!$H$8)+E102*(1-Initiatives!$I$8)+E116*(1-Initiatives!$J$8)+E130*(1-Initiatives!$K$8)+E144*(1-Initiatives!$L$8)+E158*(1-Initiatives!$M$8)+E172*(1-Initiatives!$N$8)+E186*(1-Initiatives!$O$8)</f>
+        <f aca="false">E18*(Initiatives!$C$8=1)+E32*(Initiatives!$D$8=1)+E46*(Initiatives!$E$8=1)+E60*(Initiatives!$F$8=1)+E74*(Initiatives!$G$8=1)+E88*(Initiatives!$H$8=1)+E102*(Initiatives!$I$8=1)+E116*(Initiatives!$J$8=1)+E130*(Initiatives!$K$8=1)+E144*(Initiatives!$L$8=1)+E158*(Initiatives!$M$8=1)+E172*(Initiatives!$N$8=1)+E186*(Initiatives!$O$8=1)</f>
         <v>-20957.9254133333</v>
       </c>
       <c r="F192" s="8" t="n">
-        <f aca="false">F18*(1-Initiatives!$C$8)+F32*(1-Initiatives!$D$8)+F46*(1-Initiatives!$E$8)+F60*(1-Initiatives!$F$8)+F74*(1-Initiatives!$G$8)+F88*(1-Initiatives!$H$8)+F102*(1-Initiatives!$I$8)+F116*(1-Initiatives!$J$8)+F130*(1-Initiatives!$K$8)+F144*(1-Initiatives!$L$8)+F158*(1-Initiatives!$M$8)+F172*(1-Initiatives!$N$8)+F186*(1-Initiatives!$O$8)</f>
+        <f aca="false">F18*(Initiatives!$C$8=1)+F32*(Initiatives!$D$8=1)+F46*(Initiatives!$E$8=1)+F60*(Initiatives!$F$8=1)+F74*(Initiatives!$G$8=1)+F88*(Initiatives!$H$8=1)+F102*(Initiatives!$I$8=1)+F116*(Initiatives!$J$8=1)+F130*(Initiatives!$K$8=1)+F144*(Initiatives!$L$8=1)+F158*(Initiatives!$M$8=1)+F172*(Initiatives!$N$8=1)+F186*(Initiatives!$O$8=1)</f>
         <v>-21364.48141542</v>
       </c>
       <c r="G192" s="8" t="n">
-        <f aca="false">G18*(1-Initiatives!$C$8)+G32*(1-Initiatives!$D$8)+G46*(1-Initiatives!$E$8)+G60*(1-Initiatives!$F$8)+G74*(1-Initiatives!$G$8)+G88*(1-Initiatives!$H$8)+G102*(1-Initiatives!$I$8)+G116*(1-Initiatives!$J$8)+G130*(1-Initiatives!$K$8)+G144*(1-Initiatives!$L$8)+G158*(1-Initiatives!$M$8)+G172*(1-Initiatives!$N$8)+G186*(1-Initiatives!$O$8)</f>
+        <f aca="false">G18*(Initiatives!$C$8=1)+G32*(Initiatives!$D$8=1)+G46*(Initiatives!$E$8=1)+G60*(Initiatives!$F$8=1)+G74*(Initiatives!$G$8=1)+G88*(Initiatives!$H$8=1)+G102*(Initiatives!$I$8=1)+G116*(Initiatives!$J$8=1)+G130*(Initiatives!$K$8=1)+G144*(Initiatives!$L$8=1)+G158*(Initiatives!$M$8=1)+G172*(Initiatives!$N$8=1)+G186*(Initiatives!$O$8=1)</f>
         <v>-20742.2805700105</v>
       </c>
       <c r="H192" s="8" t="n">
-        <f aca="false">H18*(1-Initiatives!$C$8)+H32*(1-Initiatives!$D$8)+H46*(1-Initiatives!$E$8)+H60*(1-Initiatives!$F$8)+H74*(1-Initiatives!$G$8)+H88*(1-Initiatives!$H$8)+H102*(1-Initiatives!$I$8)+H116*(1-Initiatives!$J$8)+H130*(1-Initiatives!$K$8)+H144*(1-Initiatives!$L$8)+H158*(1-Initiatives!$M$8)+H172*(1-Initiatives!$N$8)+H186*(1-Initiatives!$O$8)</f>
+        <f aca="false">H18*(Initiatives!$C$8=1)+H32*(Initiatives!$D$8=1)+H46*(Initiatives!$E$8=1)+H60*(Initiatives!$F$8=1)+H74*(Initiatives!$G$8=1)+H88*(Initiatives!$H$8=1)+H102*(Initiatives!$I$8=1)+H116*(Initiatives!$J$8=1)+H130*(Initiatives!$K$8=1)+H144*(Initiatives!$L$8=1)+H158*(Initiatives!$M$8=1)+H172*(Initiatives!$N$8=1)+H186*(Initiatives!$O$8=1)</f>
         <v>-20042.5530540993</v>
       </c>
       <c r="I192" s="8" t="n">
-        <f aca="false">I18*(1-Initiatives!$C$8)+I32*(1-Initiatives!$D$8)+I46*(1-Initiatives!$E$8)+I60*(1-Initiatives!$F$8)+I74*(1-Initiatives!$G$8)+I88*(1-Initiatives!$H$8)+I102*(1-Initiatives!$I$8)+I116*(1-Initiatives!$J$8)+I130*(1-Initiatives!$K$8)+I144*(1-Initiatives!$L$8)+I158*(1-Initiatives!$M$8)+I172*(1-Initiatives!$N$8)+I186*(1-Initiatives!$O$8)</f>
+        <f aca="false">I18*(Initiatives!$C$8=1)+I32*(Initiatives!$D$8=1)+I46*(Initiatives!$E$8=1)+I60*(Initiatives!$F$8=1)+I74*(Initiatives!$G$8=1)+I88*(Initiatives!$H$8=1)+I102*(Initiatives!$I$8=1)+I116*(Initiatives!$J$8=1)+I130*(Initiatives!$K$8=1)+I144*(Initiatives!$L$8=1)+I158*(Initiatives!$M$8=1)+I172*(Initiatives!$N$8=1)+I186*(Initiatives!$O$8=1)</f>
         <v>-19297.1486654805</v>
       </c>
       <c r="J192" s="8" t="n">
-        <f aca="false">J18*(1-Initiatives!$C$8)+J32*(1-Initiatives!$D$8)+J46*(1-Initiatives!$E$8)+J60*(1-Initiatives!$F$8)+J74*(1-Initiatives!$G$8)+J88*(1-Initiatives!$H$8)+J102*(1-Initiatives!$I$8)+J116*(1-Initiatives!$J$8)+J130*(1-Initiatives!$K$8)+J144*(1-Initiatives!$L$8)+J158*(1-Initiatives!$M$8)+J172*(1-Initiatives!$N$8)+J186*(1-Initiatives!$O$8)</f>
-        <v>-17937.9123744474</v>
+        <f aca="false">J18*(Initiatives!$C$8=1)+J32*(Initiatives!$D$8=1)+J46*(Initiatives!$E$8=1)+J60*(Initiatives!$F$8=1)+J74*(Initiatives!$G$8=1)+J88*(Initiatives!$H$8=1)+J102*(Initiatives!$I$8=1)+J116*(Initiatives!$J$8=1)+J130*(Initiatives!$K$8=1)+J144*(Initiatives!$L$8=1)+J158*(Initiatives!$M$8=1)+J172*(Initiatives!$N$8=1)+J186*(Initiatives!$O$8=1)</f>
+        <v>-17941.1155744474</v>
       </c>
       <c r="K192" s="8" t="n">
-        <f aca="false">K18*(1-Initiatives!$C$8)+K32*(1-Initiatives!$D$8)+K46*(1-Initiatives!$E$8)+K60*(1-Initiatives!$F$8)+K74*(1-Initiatives!$G$8)+K88*(1-Initiatives!$H$8)+K102*(1-Initiatives!$I$8)+K116*(1-Initiatives!$J$8)+K130*(1-Initiatives!$K$8)+K144*(1-Initiatives!$L$8)+K158*(1-Initiatives!$M$8)+K172*(1-Initiatives!$N$8)+K186*(1-Initiatives!$O$8)</f>
-        <v>-15992.1366008654</v>
+        <f aca="false">K18*(Initiatives!$C$8=1)+K32*(Initiatives!$D$8=1)+K46*(Initiatives!$E$8=1)+K60*(Initiatives!$F$8=1)+K74*(Initiatives!$G$8=1)+K88*(Initiatives!$H$8=1)+K102*(Initiatives!$I$8=1)+K116*(Initiatives!$J$8=1)+K130*(Initiatives!$K$8=1)+K144*(Initiatives!$L$8=1)+K158*(Initiatives!$M$8=1)+K172*(Initiatives!$N$8=1)+K186*(Initiatives!$O$8=1)</f>
+        <v>-16001.6597144654</v>
       </c>
       <c r="L192" s="8" t="n">
-        <f aca="false">L18*(1-Initiatives!$C$8)+L32*(1-Initiatives!$D$8)+L46*(1-Initiatives!$E$8)+L60*(1-Initiatives!$F$8)+L74*(1-Initiatives!$G$8)+L88*(1-Initiatives!$H$8)+L102*(1-Initiatives!$I$8)+L116*(1-Initiatives!$J$8)+L130*(1-Initiatives!$K$8)+L144*(1-Initiatives!$L$8)+L158*(1-Initiatives!$M$8)+L172*(1-Initiatives!$N$8)+L186*(1-Initiatives!$O$8)</f>
-        <v>-13506.2607593227</v>
+        <f aca="false">L18*(Initiatives!$C$8=1)+L32*(Initiatives!$D$8=1)+L46*(Initiatives!$E$8=1)+L60*(Initiatives!$F$8=1)+L74*(Initiatives!$G$8=1)+L88*(Initiatives!$H$8=1)+L102*(Initiatives!$I$8=1)+L116*(Initiatives!$J$8=1)+L130*(Initiatives!$K$8=1)+L144*(Initiatives!$L$8=1)+L158*(Initiatives!$M$8=1)+L172*(Initiatives!$N$8=1)+L186*(Initiatives!$O$8=1)</f>
+        <v>-13525.1357722795</v>
       </c>
       <c r="M192" s="8" t="n">
-        <f aca="false">M18*(1-Initiatives!$C$8)+M32*(1-Initiatives!$D$8)+M46*(1-Initiatives!$E$8)+M60*(1-Initiatives!$F$8)+M74*(1-Initiatives!$G$8)+M88*(1-Initiatives!$H$8)+M102*(1-Initiatives!$I$8)+M116*(1-Initiatives!$J$8)+M130*(1-Initiatives!$K$8)+M144*(1-Initiatives!$L$8)+M158*(1-Initiatives!$M$8)+M172*(1-Initiatives!$N$8)+M186*(1-Initiatives!$O$8)</f>
-        <v>-10505.3373797927</v>
+        <f aca="false">M18*(Initiatives!$C$8=1)+M32*(Initiatives!$D$8=1)+M46*(Initiatives!$E$8=1)+M60*(Initiatives!$F$8=1)+M74*(Initiatives!$G$8=1)+M88*(Initiatives!$H$8=1)+M102*(Initiatives!$I$8=1)+M116*(Initiatives!$J$8=1)+M130*(Initiatives!$K$8=1)+M144*(Initiatives!$L$8=1)+M158*(Initiatives!$M$8=1)+M172*(Initiatives!$N$8=1)+M186*(Initiatives!$O$8=1)</f>
+        <v>-10536.5132766632</v>
       </c>
       <c r="N192" s="8" t="n">
-        <f aca="false">N18*(1-Initiatives!$C$8)+N32*(1-Initiatives!$D$8)+N46*(1-Initiatives!$E$8)+N60*(1-Initiatives!$F$8)+N74*(1-Initiatives!$G$8)+N88*(1-Initiatives!$H$8)+N102*(1-Initiatives!$I$8)+N116*(1-Initiatives!$J$8)+N130*(1-Initiatives!$K$8)+N144*(1-Initiatives!$L$8)+N158*(1-Initiatives!$M$8)+N172*(1-Initiatives!$N$8)+N186*(1-Initiatives!$O$8)</f>
-        <v>-25164.1894003527</v>
+        <f aca="false">N18*(Initiatives!$C$8=1)+N32*(Initiatives!$D$8=1)+N46*(Initiatives!$E$8=1)+N60*(Initiatives!$F$8=1)+N74*(Initiatives!$G$8=1)+N88*(Initiatives!$H$8=1)+N102*(Initiatives!$I$8=1)+N116*(Initiatives!$J$8=1)+N130*(Initiatives!$K$8=1)+N144*(Initiatives!$L$8=1)+N158*(Initiatives!$M$8=1)+N172*(Initiatives!$N$8=1)+N186*(Initiatives!$O$8=1)</f>
+        <v>-25210.5338597689</v>
       </c>
       <c r="O192" s="8" t="n">
-        <f aca="false">O18*(1-Initiatives!$C$8)+O32*(1-Initiatives!$D$8)+O46*(1-Initiatives!$E$8)+O60*(1-Initiatives!$F$8)+O74*(1-Initiatives!$G$8)+O88*(1-Initiatives!$H$8)+O102*(1-Initiatives!$I$8)+O116*(1-Initiatives!$J$8)+O130*(1-Initiatives!$K$8)+O144*(1-Initiatives!$L$8)+O158*(1-Initiatives!$M$8)+O172*(1-Initiatives!$N$8)+O186*(1-Initiatives!$O$8)</f>
-        <v>-39617.6012178299</v>
+        <f aca="false">O18*(Initiatives!$C$8=1)+O32*(Initiatives!$D$8=1)+O46*(Initiatives!$E$8=1)+O60*(Initiatives!$F$8=1)+O74*(Initiatives!$G$8=1)+O88*(Initiatives!$H$8=1)+O102*(Initiatives!$I$8=1)+O116*(Initiatives!$J$8=1)+O130*(Initiatives!$K$8=1)+O144*(Initiatives!$L$8=1)+O158*(Initiatives!$M$8=1)+O172*(Initiatives!$N$8=1)+O186*(Initiatives!$O$8=1)</f>
+        <v>-39681.9022769417</v>
       </c>
       <c r="P192" s="8" t="n">
-        <f aca="false">P18*(1-Initiatives!$C$8)+P32*(1-Initiatives!$D$8)+P46*(1-Initiatives!$E$8)+P60*(1-Initiatives!$F$8)+P74*(1-Initiatives!$G$8)+P88*(1-Initiatives!$H$8)+P102*(1-Initiatives!$I$8)+P116*(1-Initiatives!$J$8)+P130*(1-Initiatives!$K$8)+P144*(1-Initiatives!$L$8)+P158*(1-Initiatives!$M$8)+P172*(1-Initiatives!$N$8)+P186*(1-Initiatives!$O$8)</f>
-        <v>-36294.3540588546</v>
+        <f aca="false">P18*(Initiatives!$C$8=1)+P32*(Initiatives!$D$8=1)+P46*(Initiatives!$E$8=1)+P60*(Initiatives!$F$8=1)+P74*(Initiatives!$G$8=1)+P88*(Initiatives!$H$8=1)+P102*(Initiatives!$I$8=1)+P116*(Initiatives!$J$8=1)+P130*(Initiatives!$K$8=1)+P144*(Initiatives!$L$8=1)+P158*(Initiatives!$M$8=1)+P172*(Initiatives!$N$8=1)+P186*(Initiatives!$O$8=1)</f>
+        <v>-36376.1185474674</v>
       </c>
       <c r="Q192" s="8" t="n">
-        <f aca="false">Q18*(1-Initiatives!$C$8)+Q32*(1-Initiatives!$D$8)+Q46*(1-Initiatives!$E$8)+Q60*(1-Initiatives!$F$8)+Q74*(1-Initiatives!$G$8)+Q88*(1-Initiatives!$H$8)+Q102*(1-Initiatives!$I$8)+Q116*(1-Initiatives!$J$8)+Q130*(1-Initiatives!$K$8)+Q144*(1-Initiatives!$L$8)+Q158*(1-Initiatives!$M$8)+Q172*(1-Initiatives!$N$8)+Q186*(1-Initiatives!$O$8)</f>
-        <v>-33060.5123908484</v>
+        <f aca="false">Q18*(Initiatives!$C$8=1)+Q32*(Initiatives!$D$8=1)+Q46*(Initiatives!$E$8=1)+Q60*(Initiatives!$F$8=1)+Q74*(Initiatives!$G$8=1)+Q88*(Initiatives!$H$8=1)+Q102*(Initiatives!$I$8=1)+Q116*(Initiatives!$J$8=1)+Q130*(Initiatives!$K$8=1)+Q144*(Initiatives!$L$8=1)+Q158*(Initiatives!$M$8=1)+Q172*(Initiatives!$N$8=1)+Q186*(Initiatives!$O$8=1)</f>
+        <v>-33159.2572221752</v>
       </c>
       <c r="R192" s="8" t="n">
-        <f aca="false">R18*(1-Initiatives!$C$8)+R32*(1-Initiatives!$D$8)+R46*(1-Initiatives!$E$8)+R60*(1-Initiatives!$F$8)+R74*(1-Initiatives!$G$8)+R88*(1-Initiatives!$H$8)+R102*(1-Initiatives!$I$8)+R116*(1-Initiatives!$J$8)+R130*(1-Initiatives!$K$8)+R144*(1-Initiatives!$L$8)+R158*(1-Initiatives!$M$8)+R172*(1-Initiatives!$N$8)+R186*(1-Initiatives!$O$8)</f>
-        <v>-29914.1582928351</v>
+        <f aca="false">R18*(Initiatives!$C$8=1)+R32*(Initiatives!$D$8=1)+R46*(Initiatives!$E$8=1)+R60*(Initiatives!$F$8=1)+R74*(Initiatives!$G$8=1)+R88*(Initiatives!$H$8=1)+R102*(Initiatives!$I$8=1)+R116*(Initiatives!$J$8=1)+R130*(Initiatives!$K$8=1)+R144*(Initiatives!$L$8=1)+R158*(Initiatives!$M$8=1)+R172*(Initiatives!$N$8=1)+R186*(Initiatives!$O$8=1)</f>
+        <v>-30029.4102800145</v>
       </c>
       <c r="S192" s="8" t="n">
-        <f aca="false">S18*(1-Initiatives!$C$8)+S32*(1-Initiatives!$D$8)+S46*(1-Initiatives!$E$8)+S60*(1-Initiatives!$F$8)+S74*(1-Initiatives!$G$8)+S88*(1-Initiatives!$H$8)+S102*(1-Initiatives!$I$8)+S116*(1-Initiatives!$J$8)+S130*(1-Initiatives!$K$8)+S144*(1-Initiatives!$L$8)+S158*(1-Initiatives!$M$8)+S172*(1-Initiatives!$N$8)+S186*(1-Initiatives!$O$8)</f>
-        <v>-26853.4110650712</v>
+        <f aca="false">S18*(Initiatives!$C$8=1)+S32*(Initiatives!$D$8=1)+S46*(Initiatives!$E$8=1)+S60*(Initiatives!$F$8=1)+S74*(Initiatives!$G$8=1)+S88*(Initiatives!$H$8=1)+S102*(Initiatives!$I$8=1)+S116*(Initiatives!$J$8=1)+S130*(Initiatives!$K$8=1)+S144*(Initiatives!$L$8=1)+S158*(Initiatives!$M$8=1)+S172*(Initiatives!$N$8=1)+S186*(Initiatives!$O$8=1)</f>
+        <v>-26984.7067408256</v>
       </c>
       <c r="T192" s="8" t="n">
-        <f aca="false">T18*(1-Initiatives!$C$8)+T32*(1-Initiatives!$D$8)+T46*(1-Initiatives!$E$8)+T60*(1-Initiatives!$F$8)+T74*(1-Initiatives!$G$8)+T88*(1-Initiatives!$H$8)+T102*(1-Initiatives!$I$8)+T116*(1-Initiatives!$J$8)+T130*(1-Initiatives!$K$8)+T144*(1-Initiatives!$L$8)+T158*(1-Initiatives!$M$8)+T172*(1-Initiatives!$N$8)+T186*(1-Initiatives!$O$8)</f>
-        <v>-23876.4265463954</v>
+        <f aca="false">T18*(Initiatives!$C$8=1)+T32*(Initiatives!$D$8=1)+T46*(Initiatives!$E$8=1)+T60*(Initiatives!$F$8=1)+T74*(Initiatives!$G$8=1)+T88*(Initiatives!$H$8=1)+T102*(Initiatives!$I$8=1)+T116*(Initiatives!$J$8=1)+T130*(Initiatives!$K$8=1)+T144*(Initiatives!$L$8=1)+T158*(Initiatives!$M$8=1)+T172*(Initiatives!$N$8=1)+T186*(Initiatives!$O$8=1)</f>
+        <v>-24023.3119857756</v>
       </c>
       <c r="U192" s="8" t="n">
-        <f aca="false">U18*(1-Initiatives!$C$8)+U32*(1-Initiatives!$D$8)+U46*(1-Initiatives!$E$8)+U60*(1-Initiatives!$F$8)+U74*(1-Initiatives!$G$8)+U88*(1-Initiatives!$H$8)+U102*(1-Initiatives!$I$8)+U116*(1-Initiatives!$J$8)+U130*(1-Initiatives!$K$8)+U144*(1-Initiatives!$L$8)+U158*(1-Initiatives!$M$8)+U172*(1-Initiatives!$N$8)+U186*(1-Initiatives!$O$8)</f>
-        <v>-20981.3964436521</v>
+        <f aca="false">U18*(Initiatives!$C$8=1)+U32*(Initiatives!$D$8=1)+U46*(Initiatives!$E$8=1)+U60*(Initiatives!$F$8=1)+U74*(Initiatives!$G$8=1)+U88*(Initiatives!$H$8=1)+U102*(Initiatives!$I$8=1)+U116*(Initiatives!$J$8=1)+U130*(Initiatives!$K$8=1)+U144*(Initiatives!$L$8=1)+U158*(Initiatives!$M$8=1)+U172*(Initiatives!$N$8=1)+U186*(Initiatives!$O$8=1)</f>
+        <v>-21143.4270898186</v>
       </c>
       <c r="V192" s="8" t="n">
-        <f aca="false">V18*(1-Initiatives!$C$8)+V32*(1-Initiatives!$D$8)+V46*(1-Initiatives!$E$8)+V60*(1-Initiatives!$F$8)+V74*(1-Initiatives!$G$8)+V88*(1-Initiatives!$H$8)+V102*(1-Initiatives!$I$8)+V116*(1-Initiatives!$J$8)+V130*(1-Initiatives!$K$8)+V144*(1-Initiatives!$L$8)+V158*(1-Initiatives!$M$8)+V172*(1-Initiatives!$N$8)+V186*(1-Initiatives!$O$8)</f>
-        <v>-18166.5476729804</v>
+        <f aca="false">V18*(Initiatives!$C$8=1)+V32*(Initiatives!$D$8=1)+V46*(Initiatives!$E$8=1)+V60*(Initiatives!$F$8=1)+V74*(Initiatives!$G$8=1)+V88*(Initiatives!$H$8=1)+V102*(Initiatives!$I$8=1)+V116*(Initiatives!$J$8=1)+V130*(Initiatives!$K$8=1)+V144*(Initiatives!$L$8=1)+V158*(Initiatives!$M$8=1)+V172*(Initiatives!$N$8=1)+V186*(Initiatives!$O$8=1)</f>
+        <v>-18343.2881659708</v>
       </c>
       <c r="W192" s="8" t="n">
-        <f aca="false">W18*(1-Initiatives!$C$8)+W32*(1-Initiatives!$D$8)+W46*(1-Initiatives!$E$8)+W60*(1-Initiatives!$F$8)+W74*(1-Initiatives!$G$8)+W88*(1-Initiatives!$H$8)+W102*(1-Initiatives!$I$8)+W116*(1-Initiatives!$J$8)+W130*(1-Initiatives!$K$8)+W144*(1-Initiatives!$L$8)+W158*(1-Initiatives!$M$8)+W172*(1-Initiatives!$N$8)+W186*(1-Initiatives!$O$8)</f>
-        <v>-15430.1417127654</v>
+        <f aca="false">W18*(Initiatives!$C$8=1)+W32*(Initiatives!$D$8=1)+W46*(Initiatives!$E$8=1)+W60*(Initiatives!$F$8=1)+W74*(Initiatives!$G$8=1)+W88*(Initiatives!$H$8=1)+W102*(Initiatives!$I$8=1)+W116*(Initiatives!$J$8=1)+W130*(Initiatives!$K$8=1)+W144*(Initiatives!$L$8=1)+W158*(Initiatives!$M$8=1)+W172*(Initiatives!$N$8=1)+W186*(Initiatives!$O$8=1)</f>
+        <v>-15621.1657211993</v>
       </c>
       <c r="X192" s="8" t="n">
-        <f aca="false">X18*(1-Initiatives!$C$8)+X32*(1-Initiatives!$D$8)+X46*(1-Initiatives!$E$8)+X60*(1-Initiatives!$F$8)+X74*(1-Initiatives!$G$8)+X88*(1-Initiatives!$H$8)+X102*(1-Initiatives!$I$8)+X116*(1-Initiatives!$J$8)+X130*(1-Initiatives!$K$8)+X144*(1-Initiatives!$L$8)+X158*(1-Initiatives!$M$8)+X172*(1-Initiatives!$N$8)+X186*(1-Initiatives!$O$8)</f>
-        <v>-12770.4739680488</v>
+        <f aca="false">X18*(Initiatives!$C$8=1)+X32*(Initiatives!$D$8=1)+X46*(Initiatives!$E$8=1)+X60*(Initiatives!$F$8=1)+X74*(Initiatives!$G$8=1)+X88*(Initiatives!$H$8=1)+X102*(Initiatives!$I$8=1)+X116*(Initiatives!$J$8=1)+X130*(Initiatives!$K$8=1)+X144*(Initiatives!$L$8=1)+X158*(Initiatives!$M$8=1)+X172*(Initiatives!$N$8=1)+X186*(Initiatives!$O$8=1)</f>
+        <v>-12975.3640237203</v>
       </c>
       <c r="Y192" s="8" t="n">
-        <f aca="false">Y18*(1-Initiatives!$C$8)+Y32*(1-Initiatives!$D$8)+Y46*(1-Initiatives!$E$8)+Y60*(1-Initiatives!$F$8)+Y74*(1-Initiatives!$G$8)+Y88*(1-Initiatives!$H$8)+Y102*(1-Initiatives!$I$8)+Y116*(1-Initiatives!$J$8)+Y130*(1-Initiatives!$K$8)+Y144*(1-Initiatives!$L$8)+Y158*(1-Initiatives!$M$8)+Y172*(1-Initiatives!$N$8)+Y186*(1-Initiatives!$O$8)</f>
-        <v>-10185.8731462019</v>
+        <f aca="false">Y18*(Initiatives!$C$8=1)+Y32*(Initiatives!$D$8=1)+Y46*(Initiatives!$E$8=1)+Y60*(Initiatives!$F$8=1)+Y74*(Initiatives!$G$8=1)+Y88*(Initiatives!$H$8=1)+Y102*(Initiatives!$I$8=1)+Y116*(Initiatives!$J$8=1)+Y130*(Initiatives!$K$8=1)+Y144*(Initiatives!$L$8=1)+Y158*(Initiatives!$M$8=1)+Y172*(Initiatives!$N$8=1)+Y186*(Initiatives!$O$8=1)</f>
+        <v>-10404.2204815142</v>
       </c>
       <c r="Z192" s="8" t="n">
-        <f aca="false">Z18*(1-Initiatives!$C$8)+Z32*(1-Initiatives!$D$8)+Z46*(1-Initiatives!$E$8)+Z60*(1-Initiatives!$F$8)+Z74*(1-Initiatives!$G$8)+Z88*(1-Initiatives!$H$8)+Z102*(1-Initiatives!$I$8)+Z116*(1-Initiatives!$J$8)+Z130*(1-Initiatives!$K$8)+Z144*(1-Initiatives!$L$8)+Z158*(1-Initiatives!$M$8)+Z172*(1-Initiatives!$N$8)+Z186*(1-Initiatives!$O$8)</f>
-        <v>-7674.70064366713</v>
+        <f aca="false">Z18*(Initiatives!$C$8=1)+Z32*(Initiatives!$D$8=1)+Z46*(Initiatives!$E$8=1)+Z60*(Initiatives!$F$8=1)+Z74*(Initiatives!$G$8=1)+Z88*(Initiatives!$H$8=1)+Z102*(Initiatives!$I$8=1)+Z116*(Initiatives!$J$8=1)+Z130*(Initiatives!$K$8=1)+Z144*(Initiatives!$L$8=1)+Z158*(Initiatives!$M$8=1)+Z172*(Initiatives!$N$8=1)+Z186*(Initiatives!$O$8=1)</f>
+        <v>-7906.10503185982</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24900,100 +24903,100 @@
       </c>
       <c r="B193" s="4"/>
       <c r="C193" s="8" t="n">
-        <f aca="false">C17*(1-Initiatives!$C$8)+C31*(1-Initiatives!$D$8)+C45*(1-Initiatives!$E$8)+C59*(1-Initiatives!$F$8)+C73*(1-Initiatives!$G$8)+C87*(1-Initiatives!$H$8)+C101*(1-Initiatives!$I$8)+C115*(1-Initiatives!$J$8)+C129*(1-Initiatives!$K$8)+C143*(1-Initiatives!$L$8)+C157*(1-Initiatives!$M$8)+C171*(1-Initiatives!$N$8)+C185*(1-Initiatives!$O$8)</f>
-        <v>-4997835497.8355</v>
+        <f aca="false">C17*(Initiatives!$C$8=1)+C31*(Initiatives!$D$8=1)+C45*(Initiatives!$E$8=1)+C59*(Initiatives!$F$8=1)+C73*(Initiatives!$G$8=1)+C87*(Initiatives!$H$8=1)+C101*(Initiatives!$I$8=1)+C115*(Initiatives!$J$8=1)+C129*(Initiatives!$K$8=1)+C143*(Initiatives!$L$8=1)+C157*(Initiatives!$M$8=1)+C171*(Initiatives!$N$8=1)+C185*(Initiatives!$O$8=1)</f>
+        <v>-4581168831.16883</v>
       </c>
       <c r="D193" s="8" t="n">
-        <f aca="false">D17*(1-Initiatives!$C$8)+D31*(1-Initiatives!$D$8)+D45*(1-Initiatives!$E$8)+D59*(1-Initiatives!$F$8)+D73*(1-Initiatives!$G$8)+D87*(1-Initiatives!$H$8)+D101*(1-Initiatives!$I$8)+D115*(1-Initiatives!$J$8)+D129*(1-Initiatives!$K$8)+D143*(1-Initiatives!$L$8)+D157*(1-Initiatives!$M$8)+D171*(1-Initiatives!$N$8)+D185*(1-Initiatives!$O$8)</f>
-        <v>-1425814216.69264</v>
+        <f aca="false">D17*(Initiatives!$C$8=1)+D31*(Initiatives!$D$8=1)+D45*(Initiatives!$E$8=1)+D59*(Initiatives!$F$8=1)+D73*(Initiatives!$G$8=1)+D87*(Initiatives!$H$8=1)+D101*(Initiatives!$I$8=1)+D115*(Initiatives!$J$8=1)+D129*(Initiatives!$K$8=1)+D143*(Initiatives!$L$8=1)+D157*(Initiatives!$M$8=1)+D171*(Initiatives!$N$8=1)+D185*(Initiatives!$O$8=1)</f>
+        <v>-1009147550.02597</v>
       </c>
       <c r="E193" s="8" t="n">
-        <f aca="false">E17*(1-Initiatives!$C$8)+E31*(1-Initiatives!$D$8)+E45*(1-Initiatives!$E$8)+E59*(1-Initiatives!$F$8)+E73*(1-Initiatives!$G$8)+E87*(1-Initiatives!$H$8)+E101*(1-Initiatives!$I$8)+E115*(1-Initiatives!$J$8)+E129*(1-Initiatives!$K$8)+E143*(1-Initiatives!$L$8)+E157*(1-Initiatives!$M$8)+E171*(1-Initiatives!$N$8)+E185*(1-Initiatives!$O$8)</f>
-        <v>-828407222.545222</v>
+        <f aca="false">E17*(Initiatives!$C$8=1)+E31*(Initiatives!$D$8=1)+E45*(Initiatives!$E$8=1)+E59*(Initiatives!$F$8=1)+E73*(Initiatives!$G$8=1)+E87*(Initiatives!$H$8=1)+E101*(Initiatives!$I$8=1)+E115*(Initiatives!$J$8=1)+E129*(Initiatives!$K$8=1)+E143*(Initiatives!$L$8=1)+E157*(Initiatives!$M$8=1)+E171*(Initiatives!$N$8=1)+E185*(Initiatives!$O$8=1)</f>
+        <v>-411740555.878556</v>
       </c>
       <c r="F193" s="8" t="n">
-        <f aca="false">F17*(1-Initiatives!$C$8)+F31*(1-Initiatives!$D$8)+F45*(1-Initiatives!$E$8)+F59*(1-Initiatives!$F$8)+F73*(1-Initiatives!$G$8)+F87*(1-Initiatives!$H$8)+F101*(1-Initiatives!$I$8)+F115*(1-Initiatives!$J$8)+F129*(1-Initiatives!$K$8)+F143*(1-Initiatives!$L$8)+F157*(1-Initiatives!$M$8)+F171*(1-Initiatives!$N$8)+F185*(1-Initiatives!$O$8)</f>
-        <v>-397526388.884916</v>
+        <f aca="false">F17*(Initiatives!$C$8=1)+F31*(Initiatives!$D$8=1)+F45*(Initiatives!$E$8=1)+F59*(Initiatives!$F$8=1)+F73*(Initiatives!$G$8=1)+F87*(Initiatives!$H$8=1)+F101*(Initiatives!$I$8=1)+F115*(Initiatives!$J$8=1)+F129*(Initiatives!$K$8=1)+F143*(Initiatives!$L$8=1)+F157*(Initiatives!$M$8=1)+F171*(Initiatives!$N$8=1)+F185*(Initiatives!$O$8=1)</f>
+        <v>19140277.7817504</v>
       </c>
       <c r="G193" s="8" t="n">
-        <f aca="false">G17*(1-Initiatives!$C$8)+G31*(1-Initiatives!$D$8)+G45*(1-Initiatives!$E$8)+G59*(1-Initiatives!$F$8)+G73*(1-Initiatives!$G$8)+G87*(1-Initiatives!$H$8)+G101*(1-Initiatives!$I$8)+G115*(1-Initiatives!$J$8)+G129*(1-Initiatives!$K$8)+G143*(1-Initiatives!$L$8)+G157*(1-Initiatives!$M$8)+G171*(1-Initiatives!$N$8)+G185*(1-Initiatives!$O$8)</f>
-        <v>-181313760.922441</v>
+        <f aca="false">G17*(Initiatives!$C$8=1)+G31*(Initiatives!$D$8=1)+G45*(Initiatives!$E$8=1)+G59*(Initiatives!$F$8=1)+G73*(Initiatives!$G$8=1)+G87*(Initiatives!$H$8=1)+G101*(Initiatives!$I$8=1)+G115*(Initiatives!$J$8=1)+G129*(Initiatives!$K$8=1)+G143*(Initiatives!$L$8=1)+G157*(Initiatives!$M$8=1)+G171*(Initiatives!$N$8=1)+G185*(Initiatives!$O$8=1)</f>
+        <v>235352905.744226</v>
       </c>
       <c r="H193" s="8" t="n">
-        <f aca="false">H17*(1-Initiatives!$C$8)+H31*(1-Initiatives!$D$8)+H45*(1-Initiatives!$E$8)+H59*(1-Initiatives!$F$8)+H73*(1-Initiatives!$G$8)+H87*(1-Initiatives!$H$8)+H101*(1-Initiatives!$I$8)+H115*(1-Initiatives!$J$8)+H129*(1-Initiatives!$K$8)+H143*(1-Initiatives!$L$8)+H157*(1-Initiatives!$M$8)+H171*(1-Initiatives!$N$8)+H185*(1-Initiatives!$O$8)</f>
-        <v>323586440.517738</v>
+        <f aca="false">H17*(Initiatives!$C$8=1)+H31*(Initiatives!$D$8=1)+H45*(Initiatives!$E$8=1)+H59*(Initiatives!$F$8=1)+H73*(Initiatives!$G$8=1)+H87*(Initiatives!$H$8=1)+H101*(Initiatives!$I$8=1)+H115*(Initiatives!$J$8=1)+H129*(Initiatives!$K$8=1)+H143*(Initiatives!$L$8=1)+H157*(Initiatives!$M$8=1)+H171*(Initiatives!$N$8=1)+H185*(Initiatives!$O$8=1)</f>
+        <v>740253107.184405</v>
       </c>
       <c r="I193" s="8" t="n">
-        <f aca="false">I17*(1-Initiatives!$C$8)+I31*(1-Initiatives!$D$8)+I45*(1-Initiatives!$E$8)+I59*(1-Initiatives!$F$8)+I73*(1-Initiatives!$G$8)+I87*(1-Initiatives!$H$8)+I101*(1-Initiatives!$I$8)+I115*(1-Initiatives!$J$8)+I129*(1-Initiatives!$K$8)+I143*(1-Initiatives!$L$8)+I157*(1-Initiatives!$M$8)+I171*(1-Initiatives!$N$8)+I185*(1-Initiatives!$O$8)</f>
-        <v>672712756.724584</v>
+        <f aca="false">I17*(Initiatives!$C$8=1)+I31*(Initiatives!$D$8=1)+I45*(Initiatives!$E$8=1)+I59*(Initiatives!$F$8=1)+I73*(Initiatives!$G$8=1)+I87*(Initiatives!$H$8=1)+I101*(Initiatives!$I$8=1)+I115*(Initiatives!$J$8=1)+I129*(Initiatives!$K$8=1)+I143*(Initiatives!$L$8=1)+I157*(Initiatives!$M$8=1)+I171*(Initiatives!$N$8=1)+I185*(Initiatives!$O$8=1)</f>
+        <v>797301876.724584</v>
       </c>
       <c r="J193" s="8" t="n">
-        <f aca="false">J17*(1-Initiatives!$C$8)+J31*(1-Initiatives!$D$8)+J45*(1-Initiatives!$E$8)+J59*(1-Initiatives!$F$8)+J73*(1-Initiatives!$G$8)+J87*(1-Initiatives!$H$8)+J101*(1-Initiatives!$I$8)+J115*(1-Initiatives!$J$8)+J129*(1-Initiatives!$K$8)+J143*(1-Initiatives!$L$8)+J157*(1-Initiatives!$M$8)+J171*(1-Initiatives!$N$8)+J185*(1-Initiatives!$O$8)</f>
-        <v>2243467270.64348</v>
+        <f aca="false">J17*(Initiatives!$C$8=1)+J31*(Initiatives!$D$8=1)+J45*(Initiatives!$E$8=1)+J59*(Initiatives!$F$8=1)+J73*(Initiatives!$G$8=1)+J87*(Initiatives!$H$8=1)+J101*(Initiatives!$I$8=1)+J115*(Initiatives!$J$8=1)+J129*(Initiatives!$K$8=1)+J143*(Initiatives!$L$8=1)+J157*(Initiatives!$M$8=1)+J171*(Initiatives!$N$8=1)+J185*(Initiatives!$O$8=1)</f>
+        <v>2320482275.33682</v>
       </c>
       <c r="K193" s="8" t="n">
-        <f aca="false">K17*(1-Initiatives!$C$8)+K31*(1-Initiatives!$D$8)+K45*(1-Initiatives!$E$8)+K59*(1-Initiatives!$F$8)+K73*(1-Initiatives!$G$8)+K87*(1-Initiatives!$H$8)+K101*(1-Initiatives!$I$8)+K115*(1-Initiatives!$J$8)+K129*(1-Initiatives!$K$8)+K143*(1-Initiatives!$L$8)+K157*(1-Initiatives!$M$8)+K171*(1-Initiatives!$N$8)+K185*(1-Initiatives!$O$8)</f>
-        <v>3125389376.28866</v>
+        <f aca="false">K17*(Initiatives!$C$8=1)+K31*(Initiatives!$D$8=1)+K45*(Initiatives!$E$8=1)+K59*(Initiatives!$F$8=1)+K73*(Initiatives!$G$8=1)+K87*(Initiatives!$H$8=1)+K101*(Initiatives!$I$8=1)+K115*(Initiatives!$J$8=1)+K129*(Initiatives!$K$8=1)+K143*(Initiatives!$L$8=1)+K157*(Initiatives!$M$8=1)+K171*(Initiatives!$N$8=1)+K185*(Initiatives!$O$8=1)</f>
+        <v>3194325248.26701</v>
       </c>
       <c r="L193" s="8" t="n">
-        <f aca="false">L17*(1-Initiatives!$C$8)+L31*(1-Initiatives!$D$8)+L45*(1-Initiatives!$E$8)+L59*(1-Initiatives!$F$8)+L73*(1-Initiatives!$G$8)+L87*(1-Initiatives!$H$8)+L101*(1-Initiatives!$I$8)+L115*(1-Initiatives!$J$8)+L129*(1-Initiatives!$K$8)+L143*(1-Initiatives!$L$8)+L157*(1-Initiatives!$M$8)+L171*(1-Initiatives!$N$8)+L185*(1-Initiatives!$O$8)</f>
-        <v>3650026630.07038</v>
+        <f aca="false">L17*(Initiatives!$C$8=1)+L31*(Initiatives!$D$8=1)+L45*(Initiatives!$E$8=1)+L59*(Initiatives!$F$8=1)+L73*(Initiatives!$G$8=1)+L87*(Initiatives!$H$8=1)+L101*(Initiatives!$I$8=1)+L115*(Initiatives!$J$8=1)+L129*(Initiatives!$K$8=1)+L143*(Initiatives!$L$8=1)+L157*(Initiatives!$M$8=1)+L171*(Initiatives!$N$8=1)+L185*(Initiatives!$O$8=1)</f>
+        <v>3710953902.4162</v>
       </c>
       <c r="M193" s="8" t="n">
-        <f aca="false">M17*(1-Initiatives!$C$8)+M31*(1-Initiatives!$D$8)+M45*(1-Initiatives!$E$8)+M59*(1-Initiatives!$F$8)+M73*(1-Initiatives!$G$8)+M87*(1-Initiatives!$H$8)+M101*(1-Initiatives!$I$8)+M115*(1-Initiatives!$J$8)+M129*(1-Initiatives!$K$8)+M143*(1-Initiatives!$L$8)+M157*(1-Initiatives!$M$8)+M171*(1-Initiatives!$N$8)+M185*(1-Initiatives!$O$8)</f>
-        <v>4088044869.5943</v>
+        <f aca="false">M17*(Initiatives!$C$8=1)+M31*(Initiatives!$D$8=1)+M45*(Initiatives!$E$8=1)+M59*(Initiatives!$F$8=1)+M73*(Initiatives!$G$8=1)+M87*(Initiatives!$H$8=1)+M101*(Initiatives!$I$8=1)+M115*(Initiatives!$J$8=1)+M129*(Initiatives!$K$8=1)+M143*(Initiatives!$L$8=1)+M157*(Initiatives!$M$8=1)+M171*(Initiatives!$N$8=1)+M185*(Initiatives!$O$8=1)</f>
+        <v>4141033625.24072</v>
       </c>
       <c r="N193" s="8" t="n">
-        <f aca="false">N17*(1-Initiatives!$C$8)+N31*(1-Initiatives!$D$8)+N45*(1-Initiatives!$E$8)+N59*(1-Initiatives!$F$8)+N73*(1-Initiatives!$G$8)+N87*(1-Initiatives!$H$8)+N101*(1-Initiatives!$I$8)+N115*(1-Initiatives!$J$8)+N129*(1-Initiatives!$K$8)+N143*(1-Initiatives!$L$8)+N157*(1-Initiatives!$M$8)+N171*(1-Initiatives!$N$8)+N185*(1-Initiatives!$O$8)</f>
-        <v>8161988278.86868</v>
+        <f aca="false">N17*(Initiatives!$C$8=1)+N31*(Initiatives!$D$8=1)+N45*(Initiatives!$E$8=1)+N59*(Initiatives!$F$8=1)+N73*(Initiatives!$G$8=1)+N87*(Initiatives!$H$8=1)+N101*(Initiatives!$I$8=1)+N115*(Initiatives!$J$8=1)+N129*(Initiatives!$K$8=1)+N143*(Initiatives!$L$8=1)+N157*(Initiatives!$M$8=1)+N171*(Initiatives!$N$8=1)+N185*(Initiatives!$O$8=1)</f>
+        <v>8207108150.05755</v>
       </c>
       <c r="O193" s="8" t="n">
-        <f aca="false">O17*(1-Initiatives!$C$8)+O31*(1-Initiatives!$D$8)+O45*(1-Initiatives!$E$8)+O59*(1-Initiatives!$F$8)+O73*(1-Initiatives!$G$8)+O87*(1-Initiatives!$H$8)+O101*(1-Initiatives!$I$8)+O115*(1-Initiatives!$J$8)+O129*(1-Initiatives!$K$8)+O143*(1-Initiatives!$L$8)+O157*(1-Initiatives!$M$8)+O171*(1-Initiatives!$N$8)+O185*(1-Initiatives!$O$8)</f>
-        <v>8088720842.95584</v>
+        <f aca="false">O17*(Initiatives!$C$8=1)+O31*(Initiatives!$D$8=1)+O45*(Initiatives!$E$8=1)+O59*(Initiatives!$F$8=1)+O73*(Initiatives!$G$8=1)+O87*(Initiatives!$H$8=1)+O101*(Initiatives!$I$8=1)+O115*(Initiatives!$J$8=1)+O129*(Initiatives!$K$8=1)+O143*(Initiatives!$L$8=1)+O157*(Initiatives!$M$8=1)+O171*(Initiatives!$N$8=1)+O185*(Initiatives!$O$8=1)</f>
+        <v>8080875890.7915</v>
       </c>
       <c r="P193" s="8" t="n">
-        <f aca="false">P17*(1-Initiatives!$C$8)+P31*(1-Initiatives!$D$8)+P45*(1-Initiatives!$E$8)+P59*(1-Initiatives!$F$8)+P73*(1-Initiatives!$G$8)+P87*(1-Initiatives!$H$8)+P101*(1-Initiatives!$I$8)+P115*(1-Initiatives!$J$8)+P129*(1-Initiatives!$K$8)+P143*(1-Initiatives!$L$8)+P157*(1-Initiatives!$M$8)+P171*(1-Initiatives!$N$8)+P185*(1-Initiatives!$O$8)</f>
-        <v>8004378485.04526</v>
+        <f aca="false">P17*(Initiatives!$C$8=1)+P31*(Initiatives!$D$8=1)+P45*(Initiatives!$E$8=1)+P59*(Initiatives!$F$8=1)+P73*(Initiatives!$G$8=1)+P87*(Initiatives!$H$8=1)+P101*(Initiatives!$I$8=1)+P115*(Initiatives!$J$8=1)+P129*(Initiatives!$K$8=1)+P143*(Initiatives!$L$8=1)+P157*(Initiatives!$M$8=1)+P171*(Initiatives!$N$8=1)+P185*(Initiatives!$O$8=1)</f>
+        <v>7996952674.44811</v>
       </c>
       <c r="Q193" s="8" t="n">
-        <f aca="false">Q17*(1-Initiatives!$C$8)+Q31*(1-Initiatives!$D$8)+Q45*(1-Initiatives!$E$8)+Q59*(1-Initiatives!$F$8)+Q73*(1-Initiatives!$G$8)+Q87*(1-Initiatives!$H$8)+Q101*(1-Initiatives!$I$8)+Q115*(1-Initiatives!$J$8)+Q129*(1-Initiatives!$K$8)+Q143*(1-Initiatives!$L$8)+Q157*(1-Initiatives!$M$8)+Q171*(1-Initiatives!$N$8)+Q185*(1-Initiatives!$O$8)</f>
-        <v>7920979973.71165</v>
+        <f aca="false">Q17*(Initiatives!$C$8=1)+Q31*(Initiatives!$D$8=1)+Q45*(Initiatives!$E$8=1)+Q59*(Initiatives!$F$8=1)+Q73*(Initiatives!$G$8=1)+Q87*(Initiatives!$H$8=1)+Q101*(Initiatives!$I$8=1)+Q115*(Initiatives!$J$8=1)+Q129*(Initiatives!$K$8=1)+Q143*(Initiatives!$L$8=1)+Q157*(Initiatives!$M$8=1)+Q171*(Initiatives!$N$8=1)+Q185*(Initiatives!$O$8=1)</f>
+        <v>7913970599.95076</v>
       </c>
       <c r="R193" s="8" t="n">
-        <f aca="false">R17*(1-Initiatives!$C$8)+R31*(1-Initiatives!$D$8)+R45*(1-Initiatives!$E$8)+R59*(1-Initiatives!$F$8)+R73*(1-Initiatives!$G$8)+R87*(1-Initiatives!$H$8)+R101*(1-Initiatives!$I$8)+R115*(1-Initiatives!$J$8)+R129*(1-Initiatives!$K$8)+R143*(1-Initiatives!$L$8)+R157*(1-Initiatives!$M$8)+R171*(1-Initiatives!$N$8)+R185*(1-Initiatives!$O$8)</f>
-        <v>7838492649.92963</v>
+        <f aca="false">R17*(Initiatives!$C$8=1)+R31*(Initiatives!$D$8=1)+R45*(Initiatives!$E$8=1)+R59*(Initiatives!$F$8=1)+R73*(Initiatives!$G$8=1)+R87*(Initiatives!$H$8=1)+R101*(Initiatives!$I$8=1)+R115*(Initiatives!$J$8=1)+R129*(Initiatives!$K$8=1)+R143*(Initiatives!$L$8=1)+R157*(Initiatives!$M$8=1)+R171*(Initiatives!$N$8=1)+R185*(Initiatives!$O$8=1)</f>
+        <v>7831897005.85633</v>
       </c>
       <c r="S193" s="8" t="n">
-        <f aca="false">S17*(1-Initiatives!$C$8)+S31*(1-Initiatives!$D$8)+S45*(1-Initiatives!$E$8)+S59*(1-Initiatives!$F$8)+S73*(1-Initiatives!$G$8)+S87*(1-Initiatives!$H$8)+S101*(1-Initiatives!$I$8)+S115*(1-Initiatives!$J$8)+S129*(1-Initiatives!$K$8)+S143*(1-Initiatives!$L$8)+S157*(1-Initiatives!$M$8)+S171*(1-Initiatives!$N$8)+S185*(1-Initiatives!$O$8)</f>
-        <v>7756886535.74136</v>
+        <f aca="false">S17*(Initiatives!$C$8=1)+S31*(Initiatives!$D$8=1)+S45*(Initiatives!$E$8=1)+S59*(Initiatives!$F$8=1)+S73*(Initiatives!$G$8=1)+S87*(Initiatives!$H$8=1)+S101*(Initiatives!$I$8=1)+S115*(Initiatives!$J$8=1)+S129*(Initiatives!$K$8=1)+S143*(Initiatives!$L$8=1)+S157*(Initiatives!$M$8=1)+S171*(Initiatives!$N$8=1)+S185*(Initiatives!$O$8=1)</f>
+        <v>7750701912.34135</v>
       </c>
       <c r="T193" s="8" t="n">
-        <f aca="false">T17*(1-Initiatives!$C$8)+T31*(1-Initiatives!$D$8)+T45*(1-Initiatives!$E$8)+T59*(1-Initiatives!$F$8)+T73*(1-Initiatives!$G$8)+T87*(1-Initiatives!$H$8)+T101*(1-Initiatives!$I$8)+T115*(1-Initiatives!$J$8)+T129*(1-Initiatives!$K$8)+T143*(1-Initiatives!$L$8)+T157*(1-Initiatives!$M$8)+T171*(1-Initiatives!$N$8)+T185*(1-Initiatives!$O$8)</f>
-        <v>7676134102.19912</v>
+        <f aca="false">T17*(Initiatives!$C$8=1)+T31*(Initiatives!$D$8=1)+T45*(Initiatives!$E$8=1)+T59*(Initiatives!$F$8=1)+T73*(Initiatives!$G$8=1)+T87*(Initiatives!$H$8=1)+T101*(Initiatives!$I$8=1)+T115*(Initiatives!$J$8=1)+T129*(Initiatives!$K$8=1)+T143*(Initiatives!$L$8=1)+T157*(Initiatives!$M$8=1)+T171*(Initiatives!$N$8=1)+T185*(Initiatives!$O$8=1)</f>
+        <v>7670357789.13017</v>
       </c>
       <c r="U193" s="8" t="n">
-        <f aca="false">U17*(1-Initiatives!$C$8)+U31*(1-Initiatives!$D$8)+U45*(1-Initiatives!$E$8)+U59*(1-Initiatives!$F$8)+U73*(1-Initiatives!$G$8)+U87*(1-Initiatives!$H$8)+U101*(1-Initiatives!$I$8)+U115*(1-Initiatives!$J$8)+U129*(1-Initiatives!$K$8)+U143*(1-Initiatives!$L$8)+U157*(1-Initiatives!$M$8)+U171*(1-Initiatives!$N$8)+U185*(1-Initiatives!$O$8)</f>
-        <v>7596210056.89584</v>
+        <f aca="false">U17*(Initiatives!$C$8=1)+U31*(Initiatives!$D$8=1)+U45*(Initiatives!$E$8=1)+U59*(Initiatives!$F$8=1)+U73*(Initiatives!$G$8=1)+U87*(Initiatives!$H$8=1)+U101*(Initiatives!$I$8=1)+U115*(Initiatives!$J$8=1)+U129*(Initiatives!$K$8=1)+U143*(Initiatives!$L$8=1)+U157*(Initiatives!$M$8=1)+U171*(Initiatives!$N$8=1)+U185*(Initiatives!$O$8=1)</f>
+        <v>7590839343.01122</v>
       </c>
       <c r="V193" s="8" t="n">
-        <f aca="false">V17*(1-Initiatives!$C$8)+V31*(1-Initiatives!$D$8)+V45*(1-Initiatives!$E$8)+V59*(1-Initiatives!$F$8)+V73*(1-Initiatives!$G$8)+V87*(1-Initiatives!$H$8)+V101*(1-Initiatives!$I$8)+V115*(1-Initiatives!$J$8)+V129*(1-Initiatives!$K$8)+V143*(1-Initiatives!$L$8)+V157*(1-Initiatives!$M$8)+V171*(1-Initiatives!$N$8)+V185*(1-Initiatives!$O$8)</f>
-        <v>7517091149.44668</v>
+        <f aca="false">V17*(Initiatives!$C$8=1)+V31*(Initiatives!$D$8=1)+V45*(Initiatives!$E$8=1)+V59*(Initiatives!$F$8=1)+V73*(Initiatives!$G$8=1)+V87*(Initiatives!$H$8=1)+V101*(Initiatives!$I$8=1)+V115*(Initiatives!$J$8=1)+V129*(Initiatives!$K$8=1)+V143*(Initiatives!$L$8=1)+V157*(Initiatives!$M$8=1)+V171*(Initiatives!$N$8=1)+V185*(Initiatives!$O$8=1)</f>
+        <v>7512123323.30476</v>
       </c>
       <c r="W193" s="8" t="n">
-        <f aca="false">W17*(1-Initiatives!$C$8)+W31*(1-Initiatives!$D$8)+W45*(1-Initiatives!$E$8)+W59*(1-Initiatives!$F$8)+W73*(1-Initiatives!$G$8)+W87*(1-Initiatives!$H$8)+W101*(1-Initiatives!$I$8)+W115*(1-Initiatives!$J$8)+W129*(1-Initiatives!$K$8)+W143*(1-Initiatives!$L$8)+W157*(1-Initiatives!$M$8)+W171*(1-Initiatives!$N$8)+W185*(1-Initiatives!$O$8)</f>
-        <v>7438755993.42174</v>
+        <f aca="false">W17*(Initiatives!$C$8=1)+W31*(Initiatives!$D$8=1)+W45*(Initiatives!$E$8=1)+W59*(Initiatives!$F$8=1)+W73*(Initiatives!$G$8=1)+W87*(Initiatives!$H$8=1)+W101*(Initiatives!$I$8=1)+W115*(Initiatives!$J$8=1)+W129*(Initiatives!$K$8=1)+W143*(Initiatives!$L$8=1)+W157*(Initiatives!$M$8=1)+W171*(Initiatives!$N$8=1)+W185*(Initiatives!$O$8=1)</f>
+        <v>7434188343.78197</v>
       </c>
       <c r="X193" s="8" t="n">
-        <f aca="false">X17*(1-Initiatives!$C$8)+X31*(1-Initiatives!$D$8)+X45*(1-Initiatives!$E$8)+X59*(1-Initiatives!$F$8)+X73*(1-Initiatives!$G$8)+X87*(1-Initiatives!$H$8)+X101*(1-Initiatives!$I$8)+X115*(1-Initiatives!$J$8)+X129*(1-Initiatives!$K$8)+X143*(1-Initiatives!$L$8)+X157*(1-Initiatives!$M$8)+X171*(1-Initiatives!$N$8)+X185*(1-Initiatives!$O$8)</f>
-        <v>7361184903.3544</v>
+        <f aca="false">X17*(Initiatives!$C$8=1)+X31*(Initiatives!$D$8=1)+X45*(Initiatives!$E$8=1)+X59*(Initiatives!$F$8=1)+X73*(Initiatives!$G$8=1)+X87*(Initiatives!$H$8=1)+X101*(Initiatives!$I$8=1)+X115*(Initiatives!$J$8=1)+X129*(Initiatives!$K$8=1)+X143*(Initiatives!$L$8=1)+X157*(Initiatives!$M$8=1)+X171*(Initiatives!$N$8=1)+X185*(Initiatives!$O$8=1)</f>
+        <v>7357014719.65992</v>
       </c>
       <c r="Y193" s="8" t="n">
-        <f aca="false">Y17*(1-Initiatives!$C$8)+Y31*(1-Initiatives!$D$8)+Y45*(1-Initiatives!$E$8)+Y59*(1-Initiatives!$F$8)+Y73*(1-Initiatives!$G$8)+Y87*(1-Initiatives!$H$8)+Y101*(1-Initiatives!$I$8)+Y115*(1-Initiatives!$J$8)+Y129*(1-Initiatives!$K$8)+Y143*(1-Initiatives!$L$8)+Y157*(1-Initiatives!$M$8)+Y171*(1-Initiatives!$N$8)+Y185*(1-Initiatives!$O$8)</f>
-        <v>7284359745.56471</v>
+        <f aca="false">Y17*(Initiatives!$C$8=1)+Y31*(Initiatives!$D$8=1)+Y45*(Initiatives!$E$8=1)+Y59*(Initiatives!$F$8=1)+Y73*(Initiatives!$G$8=1)+Y87*(Initiatives!$H$8=1)+Y101*(Initiatives!$I$8=1)+Y115*(Initiatives!$J$8=1)+Y129*(Initiatives!$K$8=1)+Y143*(Initiatives!$L$8=1)+Y157*(Initiatives!$M$8=1)+Y171*(Initiatives!$N$8=1)+Y185*(Initiatives!$O$8=1)</f>
+        <v>7280584318.41195</v>
       </c>
       <c r="Z193" s="8" t="n">
-        <f aca="false">Z17*(1-Initiatives!$C$8)+Z31*(1-Initiatives!$D$8)+Z45*(1-Initiatives!$E$8)+Z59*(1-Initiatives!$F$8)+Z73*(1-Initiatives!$G$8)+Z87*(1-Initiatives!$H$8)+Z101*(1-Initiatives!$I$8)+Z115*(1-Initiatives!$J$8)+Z129*(1-Initiatives!$K$8)+Z143*(1-Initiatives!$L$8)+Z157*(1-Initiatives!$M$8)+Z171*(1-Initiatives!$N$8)+Z185*(1-Initiatives!$O$8)</f>
-        <v>7208263801.64238</v>
+        <f aca="false">Z17*(Initiatives!$C$8=1)+Z31*(Initiatives!$D$8=1)+Z45*(Initiatives!$E$8=1)+Z59*(Initiatives!$F$8=1)+Z73*(Initiatives!$G$8=1)+Z87*(Initiatives!$H$8=1)+Z101*(Initiatives!$I$8=1)+Z115*(Initiatives!$J$8=1)+Z129*(Initiatives!$K$8=1)+Z143*(Initiatives!$L$8=1)+Z157*(Initiatives!$M$8=1)+Z171*(Initiatives!$N$8=1)+Z185*(Initiatives!$O$8=1)</f>
+        <v>7204880423.23776</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25002,100 +25005,100 @@
       </c>
       <c r="B194" s="4"/>
       <c r="C194" s="8" t="n">
-        <f aca="false">C14+C28+C42+C56+C70+C84+C98+C112+C126+C140+C154+C168+C182</f>
+        <f aca="false">C14*(Initiatives!$C$8&gt;=1)+C28*(Initiatives!$D$8&gt;=1)+C42*(Initiatives!$E$8&gt;=1)+C56*(Initiatives!$F$8&gt;=1)+C70*(Initiatives!$G$8&gt;=1)+C84*(Initiatives!$H$8&gt;=1)+C98*(Initiatives!$I$8&gt;=1)+C112*(Initiatives!$J$8&gt;=1)+C126*(Initiatives!$K$8&gt;=1)+C140*(Initiatives!$L$8&gt;=1)+C154*(Initiatives!$M$8&gt;=1)+C168*(Initiatives!$N$8&gt;=1)+C182*(Initiatives!$O$8&gt;=1)</f>
         <v>0</v>
       </c>
       <c r="D194" s="8" t="n">
-        <f aca="false">D14+D28+D42+D56+D70+D84+D98+D112+D126+D140+D154+D168+D182</f>
+        <f aca="false">D14*(Initiatives!$C$8&gt;=1)+D28*(Initiatives!$D$8&gt;=1)+D42*(Initiatives!$E$8&gt;=1)+D56*(Initiatives!$F$8&gt;=1)+D70*(Initiatives!$G$8&gt;=1)+D84*(Initiatives!$H$8&gt;=1)+D98*(Initiatives!$I$8&gt;=1)+D112*(Initiatives!$J$8&gt;=1)+D126*(Initiatives!$K$8&gt;=1)+D140*(Initiatives!$L$8&gt;=1)+D154*(Initiatives!$M$8&gt;=1)+D168*(Initiatives!$N$8&gt;=1)+D182*(Initiatives!$O$8&gt;=1)</f>
         <v>3129569897.14286</v>
       </c>
       <c r="E194" s="8" t="n">
-        <f aca="false">E14+E28+E42+E56+E70+E84+E98+E112+E126+E140+E154+E168+E182</f>
+        <f aca="false">E14*(Initiatives!$C$8&gt;=1)+E28*(Initiatives!$D$8&gt;=1)+E42*(Initiatives!$E$8&gt;=1)+E56*(Initiatives!$F$8&gt;=1)+E70*(Initiatives!$G$8&gt;=1)+E84*(Initiatives!$H$8&gt;=1)+E98*(Initiatives!$I$8&gt;=1)+E112*(Initiatives!$J$8&gt;=1)+E126*(Initiatives!$K$8&gt;=1)+E140*(Initiatives!$L$8&gt;=1)+E154*(Initiatives!$M$8&gt;=1)+E168*(Initiatives!$N$8&gt;=1)+E182*(Initiatives!$O$8&gt;=1)</f>
         <v>3414492594.76167</v>
       </c>
       <c r="F194" s="8" t="n">
-        <f aca="false">F14+F28+F42+F56+F70+F84+F98+F112+F126+F140+F154+F168+F182</f>
+        <f aca="false">F14*(Initiatives!$C$8&gt;=1)+F28*(Initiatives!$D$8&gt;=1)+F42*(Initiatives!$E$8&gt;=1)+F56*(Initiatives!$F$8&gt;=1)+F70*(Initiatives!$G$8&gt;=1)+F84*(Initiatives!$H$8&gt;=1)+F98*(Initiatives!$I$8&gt;=1)+F112*(Initiatives!$J$8&gt;=1)+F126*(Initiatives!$K$8&gt;=1)+F140*(Initiatives!$L$8&gt;=1)+F154*(Initiatives!$M$8&gt;=1)+F168*(Initiatives!$N$8&gt;=1)+F182*(Initiatives!$O$8&gt;=1)</f>
         <v>3780561440.85284</v>
       </c>
       <c r="G194" s="8" t="n">
-        <f aca="false">G14+G28+G42+G56+G70+G84+G98+G112+G126+G140+G154+G168+G182</f>
+        <f aca="false">G14*(Initiatives!$C$8&gt;=1)+G28*(Initiatives!$D$8&gt;=1)+G42*(Initiatives!$E$8&gt;=1)+G56*(Initiatives!$F$8&gt;=1)+G70*(Initiatives!$G$8&gt;=1)+G84*(Initiatives!$H$8&gt;=1)+G98*(Initiatives!$I$8&gt;=1)+G112*(Initiatives!$J$8&gt;=1)+G126*(Initiatives!$K$8&gt;=1)+G140*(Initiatives!$L$8&gt;=1)+G154*(Initiatives!$M$8&gt;=1)+G168*(Initiatives!$N$8&gt;=1)+G182*(Initiatives!$O$8&gt;=1)</f>
         <v>4048474712.29852</v>
       </c>
       <c r="H194" s="8" t="n">
-        <f aca="false">H14+H28+H42+H56+H70+H84+H98+H112+H126+H140+H154+H168+H182</f>
+        <f aca="false">H14*(Initiatives!$C$8&gt;=1)+H28*(Initiatives!$D$8&gt;=1)+H42*(Initiatives!$E$8&gt;=1)+H56*(Initiatives!$F$8&gt;=1)+H70*(Initiatives!$G$8&gt;=1)+H84*(Initiatives!$H$8&gt;=1)+H98*(Initiatives!$I$8&gt;=1)+H112*(Initiatives!$J$8&gt;=1)+H126*(Initiatives!$K$8&gt;=1)+H140*(Initiatives!$L$8&gt;=1)+H154*(Initiatives!$M$8&gt;=1)+H168*(Initiatives!$N$8&gt;=1)+H182*(Initiatives!$O$8&gt;=1)</f>
         <v>4133341488.32033</v>
       </c>
       <c r="I194" s="8" t="n">
-        <f aca="false">I14+I28+I42+I56+I70+I84+I98+I112+I126+I140+I154+I168+I182</f>
-        <v>4170600474.76252</v>
+        <f aca="false">I14*(Initiatives!$C$8&gt;=1)+I28*(Initiatives!$D$8&gt;=1)+I42*(Initiatives!$E$8&gt;=1)+I56*(Initiatives!$F$8&gt;=1)+I70*(Initiatives!$G$8&gt;=1)+I84*(Initiatives!$H$8&gt;=1)+I98*(Initiatives!$I$8&gt;=1)+I112*(Initiatives!$J$8&gt;=1)+I126*(Initiatives!$K$8&gt;=1)+I140*(Initiatives!$L$8&gt;=1)+I154*(Initiatives!$M$8&gt;=1)+I168*(Initiatives!$N$8&gt;=1)+I182*(Initiatives!$O$8&gt;=1)</f>
+        <v>4159923141.42919</v>
       </c>
       <c r="J194" s="8" t="n">
-        <f aca="false">J14+J28+J42+J56+J70+J84+J98+J112+J126+J140+J154+J168+J182</f>
-        <v>4652264753.93452</v>
+        <f aca="false">J14*(Initiatives!$C$8&gt;=1)+J28*(Initiatives!$D$8&gt;=1)+J42*(Initiatives!$E$8&gt;=1)+J56*(Initiatives!$F$8&gt;=1)+J70*(Initiatives!$G$8&gt;=1)+J84*(Initiatives!$H$8&gt;=1)+J98*(Initiatives!$I$8&gt;=1)+J112*(Initiatives!$J$8&gt;=1)+J126*(Initiatives!$K$8&gt;=1)+J140*(Initiatives!$L$8&gt;=1)+J154*(Initiatives!$M$8&gt;=1)+J168*(Initiatives!$N$8&gt;=1)+J182*(Initiatives!$O$8&gt;=1)</f>
+        <v>4631006183.26785</v>
       </c>
       <c r="K194" s="8" t="n">
-        <f aca="false">K14+K28+K42+K56+K70+K84+K98+K112+K126+K140+K154+K168+K182</f>
-        <v>5157982161.11338</v>
+        <f aca="false">K14*(Initiatives!$C$8&gt;=1)+K28*(Initiatives!$D$8&gt;=1)+K42*(Initiatives!$E$8&gt;=1)+K56*(Initiatives!$F$8&gt;=1)+K70*(Initiatives!$G$8&gt;=1)+K84*(Initiatives!$H$8&gt;=1)+K98*(Initiatives!$I$8&gt;=1)+K112*(Initiatives!$J$8&gt;=1)+K126*(Initiatives!$K$8&gt;=1)+K140*(Initiatives!$L$8&gt;=1)+K154*(Initiatives!$M$8&gt;=1)+K168*(Initiatives!$N$8&gt;=1)+K182*(Initiatives!$O$8&gt;=1)</f>
+        <v>5126237776.44138</v>
       </c>
       <c r="L194" s="8" t="n">
-        <f aca="false">L14+L28+L42+L56+L70+L84+L98+L112+L126+L140+L154+L168+L182</f>
-        <v>5661543864.11443</v>
+        <f aca="false">L14*(Initiatives!$C$8&gt;=1)+L28*(Initiatives!$D$8&gt;=1)+L42*(Initiatives!$E$8&gt;=1)+L56*(Initiatives!$F$8&gt;=1)+L70*(Initiatives!$G$8&gt;=1)+L84*(Initiatives!$H$8&gt;=1)+L98*(Initiatives!$I$8&gt;=1)+L112*(Initiatives!$J$8&gt;=1)+L126*(Initiatives!$K$8&gt;=1)+L140*(Initiatives!$L$8&gt;=1)+L154*(Initiatives!$M$8&gt;=1)+L168*(Initiatives!$N$8&gt;=1)+L182*(Initiatives!$O$8&gt;=1)</f>
+        <v>5619408416.95796</v>
       </c>
       <c r="M194" s="8" t="n">
-        <f aca="false">M14+M28+M42+M56+M70+M84+M98+M112+M126+M140+M154+M168+M182</f>
-        <v>6162706605.69958</v>
+        <f aca="false">M14*(Initiatives!$C$8&gt;=1)+M28*(Initiatives!$D$8&gt;=1)+M42*(Initiatives!$E$8&gt;=1)+M56*(Initiatives!$F$8&gt;=1)+M70*(Initiatives!$G$8&gt;=1)+M84*(Initiatives!$H$8&gt;=1)+M98*(Initiatives!$I$8&gt;=1)+M112*(Initiatives!$J$8&gt;=1)+M126*(Initiatives!$K$8&gt;=1)+M140*(Initiatives!$L$8&gt;=1)+M154*(Initiatives!$M$8&gt;=1)+M168*(Initiatives!$N$8&gt;=1)+M182*(Initiatives!$O$8&gt;=1)</f>
+        <v>6110274176.73496</v>
       </c>
       <c r="N194" s="8" t="n">
-        <f aca="false">N14+N28+N42+N56+N70+N84+N98+N112+N126+N140+N154+N168+N182</f>
-        <v>10195808742.3138</v>
+        <f aca="false">N14*(Initiatives!$C$8&gt;=1)+N28*(Initiatives!$D$8&gt;=1)+N42*(Initiatives!$E$8&gt;=1)+N56*(Initiatives!$F$8&gt;=1)+N70*(Initiatives!$G$8&gt;=1)+N84*(Initiatives!$H$8&gt;=1)+N98*(Initiatives!$I$8&gt;=1)+N112*(Initiatives!$J$8&gt;=1)+N126*(Initiatives!$K$8&gt;=1)+N140*(Initiatives!$L$8&gt;=1)+N154*(Initiatives!$M$8&gt;=1)+N168*(Initiatives!$N$8&gt;=1)+N182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10133172742.4303</v>
       </c>
       <c r="O194" s="8" t="n">
-        <f aca="false">O14+O28+O42+O56+O70+O84+O98+O112+O126+O140+O154+O168+O182</f>
-        <v>9830944741.69652</v>
+        <f aca="false">O14*(Initiatives!$C$8&gt;=1)+O28*(Initiatives!$D$8&gt;=1)+O42*(Initiatives!$E$8&gt;=1)+O56*(Initiatives!$F$8&gt;=1)+O70*(Initiatives!$G$8&gt;=1)+O84*(Initiatives!$H$8&gt;=1)+O98*(Initiatives!$I$8&gt;=1)+O112*(Initiatives!$J$8&gt;=1)+O126*(Initiatives!$K$8&gt;=1)+O140*(Initiatives!$L$8&gt;=1)+O154*(Initiatives!$M$8&gt;=1)+O168*(Initiatives!$N$8&gt;=1)+O182*(Initiatives!$O$8&gt;=1)</f>
+        <v>9768875246.47958</v>
       </c>
       <c r="P194" s="8" t="n">
-        <f aca="false">P14+P28+P42+P56+P70+P84+P98+P112+P126+P140+P154+P168+P182</f>
-        <v>11710043963.6025</v>
+        <f aca="false">P14*(Initiatives!$C$8&gt;=1)+P28*(Initiatives!$D$8&gt;=1)+P42*(Initiatives!$E$8&gt;=1)+P56*(Initiatives!$F$8&gt;=1)+P70*(Initiatives!$G$8&gt;=1)+P84*(Initiatives!$H$8&gt;=1)+P98*(Initiatives!$I$8&gt;=1)+P112*(Initiatives!$J$8&gt;=1)+P126*(Initiatives!$K$8&gt;=1)+P140*(Initiatives!$L$8&gt;=1)+P154*(Initiatives!$M$8&gt;=1)+P168*(Initiatives!$N$8&gt;=1)+P182*(Initiatives!$O$8&gt;=1)</f>
+        <v>11648536951.906</v>
       </c>
       <c r="Q194" s="8" t="n">
-        <f aca="false">Q14+Q28+Q42+Q56+Q70+Q84+Q98+Q112+Q126+Q140+Q154+Q168+Q182</f>
-        <v>11398416978.9282</v>
+        <f aca="false">Q14*(Initiatives!$C$8&gt;=1)+Q28*(Initiatives!$D$8&gt;=1)+Q42*(Initiatives!$E$8&gt;=1)+Q56*(Initiatives!$F$8&gt;=1)+Q70*(Initiatives!$G$8&gt;=1)+Q84*(Initiatives!$H$8&gt;=1)+Q98*(Initiatives!$I$8&gt;=1)+Q112*(Initiatives!$J$8&gt;=1)+Q126*(Initiatives!$K$8&gt;=1)+Q140*(Initiatives!$L$8&gt;=1)+Q154*(Initiatives!$M$8&gt;=1)+Q168*(Initiatives!$N$8&gt;=1)+Q182*(Initiatives!$O$8&gt;=1)</f>
+        <v>11337468436.2064</v>
       </c>
       <c r="R194" s="8" t="n">
-        <f aca="false">R14+R28+R42+R56+R70+R84+R98+R112+R126+R140+R154+R168+R182</f>
-        <v>11278302091.7877</v>
+        <f aca="false">R14*(Initiatives!$C$8&gt;=1)+R28*(Initiatives!$D$8&gt;=1)+R42*(Initiatives!$E$8&gt;=1)+R56*(Initiatives!$F$8&gt;=1)+R70*(Initiatives!$G$8&gt;=1)+R84*(Initiatives!$H$8&gt;=1)+R98*(Initiatives!$I$8&gt;=1)+R112*(Initiatives!$J$8&gt;=1)+R126*(Initiatives!$K$8&gt;=1)+R140*(Initiatives!$L$8&gt;=1)+R154*(Initiatives!$M$8&gt;=1)+R168*(Initiatives!$N$8&gt;=1)+R182*(Initiatives!$O$8&gt;=1)</f>
+        <v>11217908010.6402</v>
       </c>
       <c r="S194" s="8" t="n">
-        <f aca="false">S14+S28+S42+S56+S70+S84+S98+S112+S126+S140+S154+S168+S182</f>
-        <v>11159543748.6207</v>
+        <f aca="false">S14*(Initiatives!$C$8&gt;=1)+S28*(Initiatives!$D$8&gt;=1)+S42*(Initiatives!$E$8&gt;=1)+S56*(Initiatives!$F$8&gt;=1)+S70*(Initiatives!$G$8&gt;=1)+S84*(Initiatives!$H$8&gt;=1)+S98*(Initiatives!$I$8&gt;=1)+S112*(Initiatives!$J$8&gt;=1)+S126*(Initiatives!$K$8&gt;=1)+S140*(Initiatives!$L$8&gt;=1)+S154*(Initiatives!$M$8&gt;=1)+S168*(Initiatives!$N$8&gt;=1)+S182*(Initiatives!$O$8&gt;=1)</f>
+        <v>11099700129.3228</v>
       </c>
       <c r="T194" s="8" t="n">
-        <f aca="false">T14+T28+T42+T56+T70+T84+T98+T112+T126+T140+T154+T168+T182</f>
-        <v>11042105077.5515</v>
+        <f aca="false">T14*(Initiatives!$C$8&gt;=1)+T28*(Initiatives!$D$8&gt;=1)+T42*(Initiatives!$E$8&gt;=1)+T56*(Initiatives!$F$8&gt;=1)+T70*(Initiatives!$G$8&gt;=1)+T84*(Initiatives!$H$8&gt;=1)+T98*(Initiatives!$I$8&gt;=1)+T112*(Initiatives!$J$8&gt;=1)+T126*(Initiatives!$K$8&gt;=1)+T140*(Initiatives!$L$8&gt;=1)+T154*(Initiatives!$M$8&gt;=1)+T168*(Initiatives!$N$8&gt;=1)+T182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10982807928.5678</v>
       </c>
       <c r="U194" s="8" t="n">
-        <f aca="false">U14+U28+U42+U56+U70+U84+U98+U112+U126+U140+U154+U168+U182</f>
-        <v>10925951901.4624</v>
+        <f aca="false">U14*(Initiatives!$C$8&gt;=1)+U28*(Initiatives!$D$8&gt;=1)+U42*(Initiatives!$E$8&gt;=1)+U56*(Initiatives!$F$8&gt;=1)+U70*(Initiatives!$G$8&gt;=1)+U84*(Initiatives!$H$8&gt;=1)+U98*(Initiatives!$I$8&gt;=1)+U112*(Initiatives!$J$8&gt;=1)+U126*(Initiatives!$K$8&gt;=1)+U140*(Initiatives!$L$8&gt;=1)+U154*(Initiatives!$M$8&gt;=1)+U168*(Initiatives!$N$8&gt;=1)+U182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10867197239.9459</v>
       </c>
       <c r="V194" s="8" t="n">
-        <f aca="false">V14+V28+V42+V56+V70+V84+V98+V112+V126+V140+V154+V168+V182</f>
-        <v>10811052508.2408</v>
+        <f aca="false">V14*(Initiatives!$C$8&gt;=1)+V28*(Initiatives!$D$8&gt;=1)+V42*(Initiatives!$E$8&gt;=1)+V56*(Initiatives!$F$8&gt;=1)+V70*(Initiatives!$G$8&gt;=1)+V84*(Initiatives!$H$8&gt;=1)+V98*(Initiatives!$I$8&gt;=1)+V112*(Initiatives!$J$8&gt;=1)+V126*(Initiatives!$K$8&gt;=1)+V140*(Initiatives!$L$8&gt;=1)+V154*(Initiatives!$M$8&gt;=1)+V168*(Initiatives!$N$8&gt;=1)+V182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10752836360.5167</v>
       </c>
       <c r="W194" s="8" t="n">
-        <f aca="false">W14+W28+W42+W56+W70+W84+W98+W112+W126+W140+W154+W168+W182</f>
-        <v>10697377440.393</v>
+        <f aca="false">W14*(Initiatives!$C$8&gt;=1)+W28*(Initiatives!$D$8&gt;=1)+W42*(Initiatives!$E$8&gt;=1)+W56*(Initiatives!$F$8&gt;=1)+W70*(Initiatives!$G$8&gt;=1)+W84*(Initiatives!$H$8&gt;=1)+W98*(Initiatives!$I$8&gt;=1)+W112*(Initiatives!$J$8&gt;=1)+W126*(Initiatives!$K$8&gt;=1)+W140*(Initiatives!$L$8&gt;=1)+W154*(Initiatives!$M$8&gt;=1)+W168*(Initiatives!$N$8&gt;=1)+W182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10639695842.4281</v>
       </c>
       <c r="X194" s="8" t="n">
-        <f aca="false">X14+X28+X42+X56+X70+X84+X98+X112+X126+X140+X154+X168+X182</f>
-        <v>10584899302.4078</v>
+        <f aca="false">X14*(Initiatives!$C$8&gt;=1)+X28*(Initiatives!$D$8&gt;=1)+X42*(Initiatives!$E$8&gt;=1)+X56*(Initiatives!$F$8&gt;=1)+X70*(Initiatives!$G$8&gt;=1)+X84*(Initiatives!$H$8&gt;=1)+X98*(Initiatives!$I$8&gt;=1)+X112*(Initiatives!$J$8&gt;=1)+X126*(Initiatives!$K$8&gt;=1)+X140*(Initiatives!$L$8&gt;=1)+X154*(Initiatives!$M$8&gt;=1)+X168*(Initiatives!$N$8&gt;=1)+X182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10527748300.265</v>
       </c>
       <c r="Y194" s="8" t="n">
-        <f aca="false">Y14+Y28+Y42+Y56+Y70+Y84+Y98+Y112+Y126+Y140+Y154+Y168+Y182</f>
-        <v>10473592584.3844</v>
+        <f aca="false">Y14*(Initiatives!$C$8&gt;=1)+Y28*(Initiatives!$D$8&gt;=1)+Y42*(Initiatives!$E$8&gt;=1)+Y56*(Initiatives!$F$8&gt;=1)+Y70*(Initiatives!$G$8&gt;=1)+Y84*(Initiatives!$H$8&gt;=1)+Y98*(Initiatives!$I$8&gt;=1)+Y112*(Initiatives!$J$8&gt;=1)+Y126*(Initiatives!$K$8&gt;=1)+Y140*(Initiatives!$L$8&gt;=1)+Y154*(Initiatives!$M$8&gt;=1)+Y168*(Initiatives!$N$8&gt;=1)+Y182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10416968234.6643</v>
       </c>
       <c r="Z194" s="8" t="n">
-        <f aca="false">Z14+Z28+Z42+Z56+Z70+Z84+Z98+Z112+Z126+Z140+Z154+Z168+Z182</f>
-        <v>10363433500.5681</v>
+        <f aca="false">Z14*(Initiatives!$C$8&gt;=1)+Z28*(Initiatives!$D$8&gt;=1)+Z42*(Initiatives!$E$8&gt;=1)+Z56*(Initiatives!$F$8&gt;=1)+Z70*(Initiatives!$G$8&gt;=1)+Z84*(Initiatives!$H$8&gt;=1)+Z98*(Initiatives!$I$8&gt;=1)+Z112*(Initiatives!$J$8&gt;=1)+Z126*(Initiatives!$K$8&gt;=1)+Z140*(Initiatives!$L$8&gt;=1)+Z154*(Initiatives!$M$8&gt;=1)+Z168*(Initiatives!$N$8&gt;=1)+Z182*(Initiatives!$O$8&gt;=1)</f>
+        <v>10307331870.8356</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25104,100 +25107,100 @@
       </c>
       <c r="B195" s="4"/>
       <c r="C195" s="8" t="n">
-        <f aca="false">C18+C32+C46+C60+C74+C88+C102+C116+C130+C144+C158+C172+C186</f>
+        <f aca="false">C18*(Initiatives!$C$8&gt;=1)+C32*(Initiatives!$D$8&gt;=1)+C46*(Initiatives!$E$8&gt;=1)+C60*(Initiatives!$F$8&gt;=1)+C74*(Initiatives!$G$8&gt;=1)+C88*(Initiatives!$H$8&gt;=1)+C102*(Initiatives!$I$8&gt;=1)+C116*(Initiatives!$J$8&gt;=1)+C130*(Initiatives!$K$8&gt;=1)+C144*(Initiatives!$L$8&gt;=1)+C158*(Initiatives!$M$8&gt;=1)+C172*(Initiatives!$N$8&gt;=1)+C186*(Initiatives!$O$8&gt;=1)</f>
         <v>0</v>
       </c>
       <c r="D195" s="8" t="n">
-        <f aca="false">D18+D32+D46+D60+D74+D88+D102+D116+D130+D144+D158+D172+D186</f>
+        <f aca="false">D18*(Initiatives!$C$8&gt;=1)+D32*(Initiatives!$D$8&gt;=1)+D46*(Initiatives!$E$8&gt;=1)+D60*(Initiatives!$F$8&gt;=1)+D74*(Initiatives!$G$8&gt;=1)+D88*(Initiatives!$H$8&gt;=1)+D102*(Initiatives!$I$8&gt;=1)+D116*(Initiatives!$J$8&gt;=1)+D130*(Initiatives!$K$8&gt;=1)+D144*(Initiatives!$L$8&gt;=1)+D158*(Initiatives!$M$8&gt;=1)+D172*(Initiatives!$N$8&gt;=1)+D186*(Initiatives!$O$8&gt;=1)</f>
         <v>-10597.5466666667</v>
       </c>
       <c r="E195" s="8" t="n">
-        <f aca="false">E18+E32+E46+E60+E74+E88+E102+E116+E130+E144+E158+E172+E186</f>
+        <f aca="false">E18*(Initiatives!$C$8&gt;=1)+E32*(Initiatives!$D$8&gt;=1)+E46*(Initiatives!$E$8&gt;=1)+E60*(Initiatives!$F$8&gt;=1)+E74*(Initiatives!$G$8&gt;=1)+E88*(Initiatives!$H$8&gt;=1)+E102*(Initiatives!$I$8&gt;=1)+E116*(Initiatives!$J$8&gt;=1)+E130*(Initiatives!$K$8&gt;=1)+E144*(Initiatives!$L$8&gt;=1)+E158*(Initiatives!$M$8&gt;=1)+E172*(Initiatives!$N$8&gt;=1)+E186*(Initiatives!$O$8&gt;=1)</f>
         <v>-20957.9254133333</v>
       </c>
       <c r="F195" s="8" t="n">
-        <f aca="false">F18+F32+F46+F60+F74+F88+F102+F116+F130+F144+F158+F172+F186</f>
+        <f aca="false">F18*(Initiatives!$C$8&gt;=1)+F32*(Initiatives!$D$8&gt;=1)+F46*(Initiatives!$E$8&gt;=1)+F60*(Initiatives!$F$8&gt;=1)+F74*(Initiatives!$G$8&gt;=1)+F88*(Initiatives!$H$8&gt;=1)+F102*(Initiatives!$I$8&gt;=1)+F116*(Initiatives!$J$8&gt;=1)+F130*(Initiatives!$K$8&gt;=1)+F144*(Initiatives!$L$8&gt;=1)+F158*(Initiatives!$M$8&gt;=1)+F172*(Initiatives!$N$8&gt;=1)+F186*(Initiatives!$O$8&gt;=1)</f>
         <v>-21364.48141542</v>
       </c>
       <c r="G195" s="8" t="n">
-        <f aca="false">G18+G32+G46+G60+G74+G88+G102+G116+G130+G144+G158+G172+G186</f>
+        <f aca="false">G18*(Initiatives!$C$8&gt;=1)+G32*(Initiatives!$D$8&gt;=1)+G46*(Initiatives!$E$8&gt;=1)+G60*(Initiatives!$F$8&gt;=1)+G74*(Initiatives!$G$8&gt;=1)+G88*(Initiatives!$H$8&gt;=1)+G102*(Initiatives!$I$8&gt;=1)+G116*(Initiatives!$J$8&gt;=1)+G130*(Initiatives!$K$8&gt;=1)+G144*(Initiatives!$L$8&gt;=1)+G158*(Initiatives!$M$8&gt;=1)+G172*(Initiatives!$N$8&gt;=1)+G186*(Initiatives!$O$8&gt;=1)</f>
         <v>-20742.2805700105</v>
       </c>
       <c r="H195" s="8" t="n">
-        <f aca="false">H18+H32+H46+H60+H74+H88+H102+H116+H130+H144+H158+H172+H186</f>
+        <f aca="false">H18*(Initiatives!$C$8&gt;=1)+H32*(Initiatives!$D$8&gt;=1)+H46*(Initiatives!$E$8&gt;=1)+H60*(Initiatives!$F$8&gt;=1)+H74*(Initiatives!$G$8&gt;=1)+H88*(Initiatives!$H$8&gt;=1)+H102*(Initiatives!$I$8&gt;=1)+H116*(Initiatives!$J$8&gt;=1)+H130*(Initiatives!$K$8&gt;=1)+H144*(Initiatives!$L$8&gt;=1)+H158*(Initiatives!$M$8&gt;=1)+H172*(Initiatives!$N$8&gt;=1)+H186*(Initiatives!$O$8&gt;=1)</f>
         <v>-20042.5530540993</v>
       </c>
       <c r="I195" s="8" t="n">
-        <f aca="false">I18+I32+I46+I60+I74+I88+I102+I116+I130+I144+I158+I172+I186</f>
+        <f aca="false">I18*(Initiatives!$C$8&gt;=1)+I32*(Initiatives!$D$8&gt;=1)+I46*(Initiatives!$E$8&gt;=1)+I60*(Initiatives!$F$8&gt;=1)+I74*(Initiatives!$G$8&gt;=1)+I88*(Initiatives!$H$8&gt;=1)+I102*(Initiatives!$I$8&gt;=1)+I116*(Initiatives!$J$8&gt;=1)+I130*(Initiatives!$K$8&gt;=1)+I144*(Initiatives!$L$8&gt;=1)+I158*(Initiatives!$M$8&gt;=1)+I172*(Initiatives!$N$8&gt;=1)+I186*(Initiatives!$O$8&gt;=1)</f>
         <v>-19297.1486654805</v>
       </c>
       <c r="J195" s="8" t="n">
-        <f aca="false">J18+J32+J46+J60+J74+J88+J102+J116+J130+J144+J158+J172+J186</f>
-        <v>-17937.9123744474</v>
+        <f aca="false">J18*(Initiatives!$C$8&gt;=1)+J32*(Initiatives!$D$8&gt;=1)+J46*(Initiatives!$E$8&gt;=1)+J60*(Initiatives!$F$8&gt;=1)+J74*(Initiatives!$G$8&gt;=1)+J88*(Initiatives!$H$8&gt;=1)+J102*(Initiatives!$I$8&gt;=1)+J116*(Initiatives!$J$8&gt;=1)+J130*(Initiatives!$K$8&gt;=1)+J144*(Initiatives!$L$8&gt;=1)+J158*(Initiatives!$M$8&gt;=1)+J172*(Initiatives!$N$8&gt;=1)+J186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-17941.1155744474</v>
       </c>
       <c r="K195" s="8" t="n">
-        <f aca="false">K18+K32+K46+K60+K74+K88+K102+K116+K130+K144+K158+K172+K186</f>
-        <v>-15992.1366008654</v>
+        <f aca="false">K18*(Initiatives!$C$8&gt;=1)+K32*(Initiatives!$D$8&gt;=1)+K46*(Initiatives!$E$8&gt;=1)+K60*(Initiatives!$F$8&gt;=1)+K74*(Initiatives!$G$8&gt;=1)+K88*(Initiatives!$H$8&gt;=1)+K102*(Initiatives!$I$8&gt;=1)+K116*(Initiatives!$J$8&gt;=1)+K130*(Initiatives!$K$8&gt;=1)+K144*(Initiatives!$L$8&gt;=1)+K158*(Initiatives!$M$8&gt;=1)+K172*(Initiatives!$N$8&gt;=1)+K186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-16001.6597144654</v>
       </c>
       <c r="L195" s="8" t="n">
-        <f aca="false">L18+L32+L46+L60+L74+L88+L102+L116+L130+L144+L158+L172+L186</f>
-        <v>-13506.2607593227</v>
+        <f aca="false">L18*(Initiatives!$C$8&gt;=1)+L32*(Initiatives!$D$8&gt;=1)+L46*(Initiatives!$E$8&gt;=1)+L60*(Initiatives!$F$8&gt;=1)+L74*(Initiatives!$G$8&gt;=1)+L88*(Initiatives!$H$8&gt;=1)+L102*(Initiatives!$I$8&gt;=1)+L116*(Initiatives!$J$8&gt;=1)+L130*(Initiatives!$K$8&gt;=1)+L144*(Initiatives!$L$8&gt;=1)+L158*(Initiatives!$M$8&gt;=1)+L172*(Initiatives!$N$8&gt;=1)+L186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-13525.1357722795</v>
       </c>
       <c r="M195" s="8" t="n">
-        <f aca="false">M18+M32+M46+M60+M74+M88+M102+M116+M130+M144+M158+M172+M186</f>
-        <v>-10505.3373797927</v>
+        <f aca="false">M18*(Initiatives!$C$8&gt;=1)+M32*(Initiatives!$D$8&gt;=1)+M46*(Initiatives!$E$8&gt;=1)+M60*(Initiatives!$F$8&gt;=1)+M74*(Initiatives!$G$8&gt;=1)+M88*(Initiatives!$H$8&gt;=1)+M102*(Initiatives!$I$8&gt;=1)+M116*(Initiatives!$J$8&gt;=1)+M130*(Initiatives!$K$8&gt;=1)+M144*(Initiatives!$L$8&gt;=1)+M158*(Initiatives!$M$8&gt;=1)+M172*(Initiatives!$N$8&gt;=1)+M186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-10536.5132766632</v>
       </c>
       <c r="N195" s="8" t="n">
-        <f aca="false">N18+N32+N46+N60+N74+N88+N102+N116+N130+N144+N158+N172+N186</f>
-        <v>-25164.1894003527</v>
+        <f aca="false">N18*(Initiatives!$C$8&gt;=1)+N32*(Initiatives!$D$8&gt;=1)+N46*(Initiatives!$E$8&gt;=1)+N60*(Initiatives!$F$8&gt;=1)+N74*(Initiatives!$G$8&gt;=1)+N88*(Initiatives!$H$8&gt;=1)+N102*(Initiatives!$I$8&gt;=1)+N116*(Initiatives!$J$8&gt;=1)+N130*(Initiatives!$K$8&gt;=1)+N144*(Initiatives!$L$8&gt;=1)+N158*(Initiatives!$M$8&gt;=1)+N172*(Initiatives!$N$8&gt;=1)+N186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-25210.5338597689</v>
       </c>
       <c r="O195" s="8" t="n">
-        <f aca="false">O18+O32+O46+O60+O74+O88+O102+O116+O130+O144+O158+O172+O186</f>
-        <v>-39617.6012178299</v>
+        <f aca="false">O18*(Initiatives!$C$8&gt;=1)+O32*(Initiatives!$D$8&gt;=1)+O46*(Initiatives!$E$8&gt;=1)+O60*(Initiatives!$F$8&gt;=1)+O74*(Initiatives!$G$8&gt;=1)+O88*(Initiatives!$H$8&gt;=1)+O102*(Initiatives!$I$8&gt;=1)+O116*(Initiatives!$J$8&gt;=1)+O130*(Initiatives!$K$8&gt;=1)+O144*(Initiatives!$L$8&gt;=1)+O158*(Initiatives!$M$8&gt;=1)+O172*(Initiatives!$N$8&gt;=1)+O186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-39681.9022769417</v>
       </c>
       <c r="P195" s="8" t="n">
-        <f aca="false">P18+P32+P46+P60+P74+P88+P102+P116+P130+P144+P158+P172+P186</f>
-        <v>-42982.3540588546</v>
+        <f aca="false">P18*(Initiatives!$C$8&gt;=1)+P32*(Initiatives!$D$8&gt;=1)+P46*(Initiatives!$E$8&gt;=1)+P60*(Initiatives!$F$8&gt;=1)+P74*(Initiatives!$G$8&gt;=1)+P88*(Initiatives!$H$8&gt;=1)+P102*(Initiatives!$I$8&gt;=1)+P116*(Initiatives!$J$8&gt;=1)+P130*(Initiatives!$K$8&gt;=1)+P144*(Initiatives!$L$8&gt;=1)+P158*(Initiatives!$M$8&gt;=1)+P172*(Initiatives!$N$8&gt;=1)+P186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-43064.1185474674</v>
       </c>
       <c r="Q195" s="8" t="n">
-        <f aca="false">Q18+Q32+Q46+Q60+Q74+Q88+Q102+Q116+Q130+Q144+Q158+Q172+Q186</f>
-        <v>-46336.1923908484</v>
+        <f aca="false">Q18*(Initiatives!$C$8&gt;=1)+Q32*(Initiatives!$D$8&gt;=1)+Q46*(Initiatives!$E$8&gt;=1)+Q60*(Initiatives!$F$8&gt;=1)+Q74*(Initiatives!$G$8&gt;=1)+Q88*(Initiatives!$H$8&gt;=1)+Q102*(Initiatives!$I$8&gt;=1)+Q116*(Initiatives!$J$8&gt;=1)+Q130*(Initiatives!$K$8&gt;=1)+Q144*(Initiatives!$L$8&gt;=1)+Q158*(Initiatives!$M$8&gt;=1)+Q172*(Initiatives!$N$8&gt;=1)+Q186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-46434.9372221752</v>
       </c>
       <c r="R195" s="8" t="n">
-        <f aca="false">R18+R32+R46+R60+R74+R88+R102+R116+R130+R144+R158+R172+R186</f>
-        <v>-42990.7030928351</v>
+        <f aca="false">R18*(Initiatives!$C$8&gt;=1)+R32*(Initiatives!$D$8&gt;=1)+R46*(Initiatives!$E$8&gt;=1)+R60*(Initiatives!$F$8&gt;=1)+R74*(Initiatives!$G$8&gt;=1)+R88*(Initiatives!$H$8&gt;=1)+R102*(Initiatives!$I$8&gt;=1)+R116*(Initiatives!$J$8&gt;=1)+R130*(Initiatives!$K$8&gt;=1)+R144*(Initiatives!$L$8&gt;=1)+R158*(Initiatives!$M$8&gt;=1)+R172*(Initiatives!$N$8&gt;=1)+R186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-43105.9550800145</v>
       </c>
       <c r="S195" s="8" t="n">
-        <f aca="false">S18+S32+S46+S60+S74+S88+S102+S116+S130+S144+S158+S172+S186</f>
-        <v>-39733.8076930712</v>
+        <f aca="false">S18*(Initiatives!$C$8&gt;=1)+S32*(Initiatives!$D$8&gt;=1)+S46*(Initiatives!$E$8&gt;=1)+S60*(Initiatives!$F$8&gt;=1)+S74*(Initiatives!$G$8&gt;=1)+S88*(Initiatives!$H$8&gt;=1)+S102*(Initiatives!$I$8&gt;=1)+S116*(Initiatives!$J$8&gt;=1)+S130*(Initiatives!$K$8&gt;=1)+S144*(Initiatives!$L$8&gt;=1)+S158*(Initiatives!$M$8&gt;=1)+S172*(Initiatives!$N$8&gt;=1)+S186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-39865.1033688256</v>
       </c>
       <c r="T195" s="8" t="n">
-        <f aca="false">T18+T32+T46+T60+T74+T88+T102+T116+T130+T144+T158+T172+T186</f>
-        <v>-36563.6172249754</v>
+        <f aca="false">T18*(Initiatives!$C$8&gt;=1)+T32*(Initiatives!$D$8&gt;=1)+T46*(Initiatives!$E$8&gt;=1)+T60*(Initiatives!$F$8&gt;=1)+T74*(Initiatives!$G$8&gt;=1)+T88*(Initiatives!$H$8&gt;=1)+T102*(Initiatives!$I$8&gt;=1)+T116*(Initiatives!$J$8&gt;=1)+T130*(Initiatives!$K$8&gt;=1)+T144*(Initiatives!$L$8&gt;=1)+T158*(Initiatives!$M$8&gt;=1)+T172*(Initiatives!$N$8&gt;=1)+T186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-36710.5026643556</v>
       </c>
       <c r="U195" s="8" t="n">
-        <f aca="false">U18+U32+U46+U60+U74+U88+U102+U116+U130+U144+U158+U172+U186</f>
-        <v>-33478.2792620534</v>
+        <f aca="false">U18*(Initiatives!$C$8&gt;=1)+U32*(Initiatives!$D$8&gt;=1)+U46*(Initiatives!$E$8&gt;=1)+U60*(Initiatives!$F$8&gt;=1)+U74*(Initiatives!$G$8&gt;=1)+U88*(Initiatives!$H$8&gt;=1)+U102*(Initiatives!$I$8&gt;=1)+U116*(Initiatives!$J$8&gt;=1)+U130*(Initiatives!$K$8&gt;=1)+U144*(Initiatives!$L$8&gt;=1)+U158*(Initiatives!$M$8&gt;=1)+U172*(Initiatives!$N$8&gt;=1)+U186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-33640.3099082199</v>
       </c>
       <c r="V195" s="8" t="n">
-        <f aca="false">V18+V32+V46+V60+V74+V88+V102+V116+V130+V144+V158+V172+V186</f>
-        <v>-30475.9772491057</v>
+        <f aca="false">V18*(Initiatives!$C$8&gt;=1)+V32*(Initiatives!$D$8&gt;=1)+V46*(Initiatives!$E$8&gt;=1)+V60*(Initiatives!$F$8&gt;=1)+V74*(Initiatives!$G$8&gt;=1)+V88*(Initiatives!$H$8&gt;=1)+V102*(Initiatives!$I$8&gt;=1)+V116*(Initiatives!$J$8&gt;=1)+V130*(Initiatives!$K$8&gt;=1)+V144*(Initiatives!$L$8&gt;=1)+V158*(Initiatives!$M$8&gt;=1)+V172*(Initiatives!$N$8&gt;=1)+V186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-30652.7177420961</v>
       </c>
       <c r="W195" s="8" t="n">
-        <f aca="false">W18+W32+W46+W60+W74+W88+W102+W116+W130+W144+W158+W172+W186</f>
-        <v>-27554.9298452488</v>
+        <f aca="false">W18*(Initiatives!$C$8&gt;=1)+W32*(Initiatives!$D$8&gt;=1)+W46*(Initiatives!$E$8&gt;=1)+W60*(Initiatives!$F$8&gt;=1)+W74*(Initiatives!$G$8&gt;=1)+W88*(Initiatives!$H$8&gt;=1)+W102*(Initiatives!$I$8&gt;=1)+W116*(Initiatives!$J$8&gt;=1)+W130*(Initiatives!$K$8&gt;=1)+W144*(Initiatives!$L$8&gt;=1)+W158*(Initiatives!$M$8&gt;=1)+W172*(Initiatives!$N$8&gt;=1)+W186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-27745.9538536827</v>
       </c>
       <c r="X195" s="8" t="n">
-        <f aca="false">X18+X32+X46+X60+X74+X88+X102+X116+X130+X144+X158+X172+X186</f>
-        <v>-24713.3902785449</v>
+        <f aca="false">X18*(Initiatives!$C$8&gt;=1)+X32*(Initiatives!$D$8&gt;=1)+X46*(Initiatives!$E$8&gt;=1)+X60*(Initiatives!$F$8&gt;=1)+X74*(Initiatives!$G$8&gt;=1)+X88*(Initiatives!$H$8&gt;=1)+X102*(Initiatives!$I$8&gt;=1)+X116*(Initiatives!$J$8&gt;=1)+X130*(Initiatives!$K$8&gt;=1)+X144*(Initiatives!$L$8&gt;=1)+X158*(Initiatives!$M$8&gt;=1)+X172*(Initiatives!$N$8&gt;=1)+X186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-24918.2803342164</v>
       </c>
       <c r="Y195" s="8" t="n">
-        <f aca="false">Y18+Y32+Y46+Y60+Y74+Y88+Y102+Y116+Y130+Y144+Y158+Y172+Y186</f>
-        <v>-21949.6457120406</v>
+        <f aca="false">Y18*(Initiatives!$C$8&gt;=1)+Y32*(Initiatives!$D$8&gt;=1)+Y46*(Initiatives!$E$8&gt;=1)+Y60*(Initiatives!$F$8&gt;=1)+Y74*(Initiatives!$G$8&gt;=1)+Y88*(Initiatives!$H$8&gt;=1)+Y102*(Initiatives!$I$8&gt;=1)+Y116*(Initiatives!$J$8&gt;=1)+Y130*(Initiatives!$K$8&gt;=1)+Y144*(Initiatives!$L$8&gt;=1)+Y158*(Initiatives!$M$8&gt;=1)+Y172*(Initiatives!$N$8&gt;=1)+Y186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-22167.9930473529</v>
       </c>
       <c r="Z195" s="8" t="n">
-        <f aca="false">Z18+Z32+Z46+Z60+Z74+Z88+Z102+Z116+Z130+Z144+Z158+Z172+Z186</f>
-        <v>-19262.0166210183</v>
+        <f aca="false">Z18*(Initiatives!$C$8&gt;=1)+Z32*(Initiatives!$D$8&gt;=1)+Z46*(Initiatives!$E$8&gt;=1)+Z60*(Initiatives!$F$8&gt;=1)+Z74*(Initiatives!$G$8&gt;=1)+Z88*(Initiatives!$H$8&gt;=1)+Z102*(Initiatives!$I$8&gt;=1)+Z116*(Initiatives!$J$8&gt;=1)+Z130*(Initiatives!$K$8&gt;=1)+Z144*(Initiatives!$L$8&gt;=1)+Z158*(Initiatives!$M$8&gt;=1)+Z172*(Initiatives!$N$8&gt;=1)+Z186*(Initiatives!$O$8&gt;=1)</f>
+        <v>-19493.4210092109</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25231,75 +25234,75 @@
       </c>
       <c r="I196" s="8" t="n">
         <f aca="false">(I$5+I190*(1-Portfolio!$C$3))/(I$4+I192*(1-Portfolio!$C$3))</f>
-        <v>19649.4338061145</v>
+        <v>19646.7231218537</v>
       </c>
       <c r="J196" s="8" t="n">
         <f aca="false">(J$5+J190*(1-Portfolio!$C$3))/(J$4+J192*(1-Portfolio!$C$3))</f>
-        <v>19784.2463109601</v>
+        <v>19778.7849861664</v>
       </c>
       <c r="K196" s="8" t="n">
         <f aca="false">(K$5+K190*(1-Portfolio!$C$3))/(K$4+K192*(1-Portfolio!$C$3))</f>
-        <v>19926.0528703808</v>
+        <v>19917.8020406495</v>
       </c>
       <c r="L196" s="8" t="n">
         <f aca="false">(L$5+L190*(1-Portfolio!$C$3))/(L$4+L192*(1-Portfolio!$C$3))</f>
-        <v>20068.3011793924</v>
+        <v>20057.2230530363</v>
       </c>
       <c r="M196" s="8" t="n">
         <f aca="false">(M$5+M190*(1-Portfolio!$C$3))/(M$4+M192*(1-Portfolio!$C$3))</f>
-        <v>20210.9249745345</v>
+        <v>20196.9828821747</v>
       </c>
       <c r="N196" s="8" t="n">
         <f aca="false">(N$5+N190*(1-Portfolio!$C$3))/(N$4+N192*(1-Portfolio!$C$3))</f>
-        <v>21424.9103070361</v>
+        <v>21407.9984883237</v>
       </c>
       <c r="O196" s="8" t="n">
         <f aca="false">(O$5+O190*(1-Portfolio!$C$3))/(O$4+O192*(1-Portfolio!$C$3))</f>
-        <v>21454.5070021941</v>
+        <v>21437.5329108861</v>
       </c>
       <c r="P196" s="8" t="n">
         <f aca="false">(P$5+P190*(1-Portfolio!$C$3))/(P$4+P192*(1-Portfolio!$C$3))</f>
-        <v>21452.5616923652</v>
+        <v>21435.6082148227</v>
       </c>
       <c r="Q196" s="8" t="n">
         <f aca="false">(Q$5+Q190*(1-Portfolio!$C$3))/(Q$4+Q192*(1-Portfolio!$C$3))</f>
-        <v>21450.7175292681</v>
+        <v>21433.7846458861</v>
       </c>
       <c r="R196" s="8" t="n">
         <f aca="false">(R$5+R190*(1-Portfolio!$C$3))/(R$4+R192*(1-Portfolio!$C$3))</f>
-        <v>21448.9678422815</v>
+        <v>21432.0555348432</v>
       </c>
       <c r="S196" s="8" t="n">
         <f aca="false">(S$5+S190*(1-Portfolio!$C$3))/(S$4+S192*(1-Portfolio!$C$3))</f>
-        <v>21447.3064283895</v>
+        <v>21430.414679949</v>
       </c>
       <c r="T196" s="8" t="n">
         <f aca="false">(T$5+T190*(1-Portfolio!$C$3))/(T$4+T192*(1-Portfolio!$C$3))</f>
-        <v>21445.7275194475</v>
+        <v>21428.8563142234</v>
       </c>
       <c r="U196" s="8" t="n">
         <f aca="false">(U$5+U190*(1-Portfolio!$C$3))/(U$4+U192*(1-Portfolio!$C$3))</f>
-        <v>21444.22575174</v>
+        <v>21427.375075018</v>
       </c>
       <c r="V196" s="8" t="n">
         <f aca="false">(V$5+V190*(1-Portfolio!$C$3))/(V$4+V192*(1-Portfolio!$C$3))</f>
-        <v>21442.7961376696</v>
+        <v>21425.965975714</v>
       </c>
       <c r="W196" s="8" t="n">
         <f aca="false">(W$5+W190*(1-Portfolio!$C$3))/(W$4+W192*(1-Portfolio!$C$3))</f>
-        <v>21441.4340394282</v>
+        <v>21424.6243794012</v>
       </c>
       <c r="X196" s="8" t="n">
         <f aca="false">(X$5+X190*(1-Portfolio!$C$3))/(X$4+X192*(1-Portfolio!$C$3))</f>
-        <v>21440.1351445118</v>
+        <v>21423.3459744003</v>
       </c>
       <c r="Y196" s="8" t="n">
         <f aca="false">(Y$5+Y190*(1-Portfolio!$C$3))/(Y$4+Y192*(1-Portfolio!$C$3))</f>
-        <v>21438.8954429497</v>
+        <v>21422.1267514981</v>
       </c>
       <c r="Z196" s="8" t="n">
         <f aca="false">(Z$5+Z190*(1-Portfolio!$C$3))/(Z$4+Z192*(1-Portfolio!$C$3))</f>
-        <v>21437.7112061271</v>
+        <v>21420.9629827772</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25333,75 +25336,75 @@
       </c>
       <c r="I197" s="24" t="n">
         <f aca="false">I196/Inputs!$C$8-1</f>
-        <v>0.0621315570872716</v>
+        <v>0.061985033613716</v>
       </c>
       <c r="J197" s="24" t="n">
         <f aca="false">J196/Inputs!$C$8-1</f>
-        <v>0.069418719511358</v>
+        <v>0.0691235127657535</v>
       </c>
       <c r="K197" s="24" t="n">
         <f aca="false">K196/Inputs!$C$8-1</f>
-        <v>0.0770839389395031</v>
+        <v>0.0766379481432185</v>
       </c>
       <c r="L197" s="24" t="n">
         <f aca="false">L196/Inputs!$C$8-1</f>
-        <v>0.0847730367239115</v>
+        <v>0.084174219083041</v>
       </c>
       <c r="M197" s="24" t="n">
         <f aca="false">M196/Inputs!$C$8-1</f>
-        <v>0.0924824310559202</v>
+        <v>0.0917288044418745</v>
       </c>
       <c r="N197" s="24" t="n">
         <f aca="false">N196/Inputs!$C$8-1</f>
-        <v>0.15810325983979</v>
+        <v>0.157189107476957</v>
       </c>
       <c r="O197" s="24" t="n">
         <f aca="false">O196/Inputs!$C$8-1</f>
-        <v>0.159703081199678</v>
+        <v>0.158785562750602</v>
       </c>
       <c r="P197" s="24" t="n">
         <f aca="false">P196/Inputs!$C$8-1</f>
-        <v>0.159597929317036</v>
+        <v>0.158681525125549</v>
       </c>
       <c r="Q197" s="24" t="n">
         <f aca="false">Q196/Inputs!$C$8-1</f>
-        <v>0.159498244825305</v>
+        <v>0.158582953831683</v>
       </c>
       <c r="R197" s="24" t="n">
         <f aca="false">R196/Inputs!$C$8-1</f>
-        <v>0.159403667150353</v>
+        <v>0.158489488369902</v>
       </c>
       <c r="S197" s="24" t="n">
         <f aca="false">S196/Inputs!$C$8-1</f>
-        <v>0.159313860994026</v>
+        <v>0.158400793510755</v>
       </c>
       <c r="T197" s="24" t="n">
         <f aca="false">T196/Inputs!$C$8-1</f>
-        <v>0.159228514564728</v>
+        <v>0.158316557525587</v>
       </c>
       <c r="U197" s="24" t="n">
         <f aca="false">U196/Inputs!$C$8-1</f>
-        <v>0.15914733793189</v>
+        <v>0.158236490541512</v>
       </c>
       <c r="V197" s="24" t="n">
         <f aca="false">V196/Inputs!$C$8-1</f>
-        <v>0.159070061495652</v>
+        <v>0.158160323011566</v>
       </c>
       <c r="W197" s="24" t="n">
         <f aca="false">W196/Inputs!$C$8-1</f>
-        <v>0.158996434563685</v>
+        <v>0.158087804291958</v>
       </c>
       <c r="X197" s="24" t="n">
         <f aca="false">X196/Inputs!$C$8-1</f>
-        <v>0.158926224027667</v>
+        <v>0.158018701318935</v>
       </c>
       <c r="Y197" s="24" t="n">
         <f aca="false">Y196/Inputs!$C$8-1</f>
-        <v>0.158859213132414</v>
+        <v>0.157952797378276</v>
       </c>
       <c r="Z197" s="24" t="n">
         <f aca="false">Z196/Inputs!$C$8-1</f>
-        <v>0.158795200331197</v>
+        <v>0.157889890960932</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25435,75 +25438,75 @@
       </c>
       <c r="I198" s="8" t="n">
         <f aca="false">(I$5+I194*(1-Portfolio!$C$3))/(I$4+I195*(1-Portfolio!$C$3))</f>
-        <v>19649.4338061145</v>
+        <v>19646.7231218537</v>
       </c>
       <c r="J198" s="8" t="n">
         <f aca="false">(J$5+J194*(1-Portfolio!$C$3))/(J$4+J195*(1-Portfolio!$C$3))</f>
-        <v>19784.2463109601</v>
+        <v>19778.7849861664</v>
       </c>
       <c r="K198" s="8" t="n">
         <f aca="false">(K$5+K194*(1-Portfolio!$C$3))/(K$4+K195*(1-Portfolio!$C$3))</f>
-        <v>19926.0528703808</v>
+        <v>19917.8020406495</v>
       </c>
       <c r="L198" s="8" t="n">
         <f aca="false">(L$5+L194*(1-Portfolio!$C$3))/(L$4+L195*(1-Portfolio!$C$3))</f>
-        <v>20068.3011793924</v>
+        <v>20057.2230530363</v>
       </c>
       <c r="M198" s="8" t="n">
         <f aca="false">(M$5+M194*(1-Portfolio!$C$3))/(M$4+M195*(1-Portfolio!$C$3))</f>
-        <v>20210.9249745345</v>
+        <v>20196.9828821747</v>
       </c>
       <c r="N198" s="8" t="n">
         <f aca="false">(N$5+N194*(1-Portfolio!$C$3))/(N$4+N195*(1-Portfolio!$C$3))</f>
-        <v>21424.9103070361</v>
+        <v>21407.9984883237</v>
       </c>
       <c r="O198" s="8" t="n">
         <f aca="false">(O$5+O194*(1-Portfolio!$C$3))/(O$4+O195*(1-Portfolio!$C$3))</f>
-        <v>21454.5070021941</v>
+        <v>21437.5329108861</v>
       </c>
       <c r="P198" s="8" t="n">
         <f aca="false">(P$5+P194*(1-Portfolio!$C$3))/(P$4+P195*(1-Portfolio!$C$3))</f>
-        <v>22054.7204640584</v>
+        <v>22037.7487509765</v>
       </c>
       <c r="Q198" s="8" t="n">
         <f aca="false">(Q$5+Q194*(1-Portfolio!$C$3))/(Q$4+Q195*(1-Portfolio!$C$3))</f>
-        <v>22040.913237271</v>
+        <v>22023.9322422923</v>
       </c>
       <c r="R198" s="8" t="n">
         <f aca="false">(R$5+R194*(1-Portfolio!$C$3))/(R$4+R195*(1-Portfolio!$C$3))</f>
-        <v>22038.6983639755</v>
+        <v>22021.7411569791</v>
       </c>
       <c r="S198" s="8" t="n">
         <f aca="false">(S$5+S194*(1-Portfolio!$C$3))/(S$4+S195*(1-Portfolio!$C$3))</f>
-        <v>22036.5725883364</v>
+        <v>22019.6391519605</v>
       </c>
       <c r="T198" s="8" t="n">
         <f aca="false">(T$5+T194*(1-Portfolio!$C$3))/(T$4+T195*(1-Portfolio!$C$3))</f>
-        <v>22034.5301180519</v>
+        <v>22017.6204361195</v>
       </c>
       <c r="U198" s="8" t="n">
         <f aca="false">(U$5+U194*(1-Portfolio!$C$3))/(U$4+U195*(1-Portfolio!$C$3))</f>
-        <v>22032.5655668686</v>
+        <v>22015.6796242888</v>
       </c>
       <c r="V198" s="8" t="n">
         <f aca="false">(V$5+V194*(1-Portfolio!$C$3))/(V$4+V195*(1-Portfolio!$C$3))</f>
-        <v>22030.6739261555</v>
+        <v>22013.8117088351</v>
       </c>
       <c r="W198" s="8" t="n">
         <f aca="false">(W$5+W194*(1-Portfolio!$C$3))/(W$4+W195*(1-Portfolio!$C$3))</f>
-        <v>22028.8505384698</v>
+        <v>22012.0120332312</v>
       </c>
       <c r="X198" s="8" t="n">
         <f aca="false">(X$5+X194*(1-Portfolio!$C$3))/(X$4+X195*(1-Portfolio!$C$3))</f>
-        <v>22027.0910729724</v>
+        <v>22010.27626748</v>
       </c>
       <c r="Y198" s="8" t="n">
         <f aca="false">(Y$5+Y194*(1-Portfolio!$C$3))/(Y$4+Y195*(1-Portfolio!$C$3))</f>
-        <v>22025.3915025653</v>
+        <v>22008.600385258</v>
       </c>
       <c r="Z198" s="8" t="n">
         <f aca="false">(Z$5+Z194*(1-Portfolio!$C$3))/(Z$4+Z195*(1-Portfolio!$C$3))</f>
-        <v>22023.7480826293</v>
+        <v>22006.9806426595</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25537,75 +25540,75 @@
       </c>
       <c r="I199" s="24" t="n">
         <f aca="false">I198/Inputs!$C$8-1</f>
-        <v>0.0621315570872716</v>
+        <v>0.061985033613716</v>
       </c>
       <c r="J199" s="24" t="n">
         <f aca="false">J198/Inputs!$C$8-1</f>
-        <v>0.069418719511358</v>
+        <v>0.0691235127657535</v>
       </c>
       <c r="K199" s="24" t="n">
         <f aca="false">K198/Inputs!$C$8-1</f>
-        <v>0.0770839389395031</v>
+        <v>0.0766379481432185</v>
       </c>
       <c r="L199" s="24" t="n">
         <f aca="false">L198/Inputs!$C$8-1</f>
-        <v>0.0847730367239115</v>
+        <v>0.084174219083041</v>
       </c>
       <c r="M199" s="24" t="n">
         <f aca="false">M198/Inputs!$C$8-1</f>
-        <v>0.0924824310559202</v>
+        <v>0.0917288044418745</v>
       </c>
       <c r="N199" s="24" t="n">
         <f aca="false">N198/Inputs!$C$8-1</f>
-        <v>0.15810325983979</v>
+        <v>0.157189107476957</v>
       </c>
       <c r="O199" s="24" t="n">
         <f aca="false">O198/Inputs!$C$8-1</f>
-        <v>0.159703081199678</v>
+        <v>0.158785562750602</v>
       </c>
       <c r="P199" s="24" t="n">
         <f aca="false">P198/Inputs!$C$8-1</f>
-        <v>0.192147052111267</v>
+        <v>0.191229662214945</v>
       </c>
       <c r="Q199" s="24" t="n">
         <f aca="false">Q198/Inputs!$C$8-1</f>
-        <v>0.19140071552816</v>
+        <v>0.190482823907693</v>
       </c>
       <c r="R199" s="24" t="n">
         <f aca="false">R198/Inputs!$C$8-1</f>
-        <v>0.191280992647323</v>
+        <v>0.190364386863735</v>
       </c>
       <c r="S199" s="24" t="n">
         <f aca="false">S198/Inputs!$C$8-1</f>
-        <v>0.191166085856019</v>
+        <v>0.190250764970839</v>
       </c>
       <c r="T199" s="24" t="n">
         <f aca="false">T198/Inputs!$C$8-1</f>
-        <v>0.191055682056861</v>
+        <v>0.190141645195647</v>
       </c>
       <c r="U199" s="24" t="n">
         <f aca="false">U198/Inputs!$C$8-1</f>
-        <v>0.190949490101003</v>
+        <v>0.190036736448046</v>
       </c>
       <c r="V199" s="24" t="n">
         <f aca="false">V198/Inputs!$C$8-1</f>
-        <v>0.190847239251648</v>
+        <v>0.18993576804514</v>
       </c>
       <c r="W199" s="24" t="n">
         <f aca="false">W198/Inputs!$C$8-1</f>
-        <v>0.190748677755125</v>
+        <v>0.189838488282769</v>
       </c>
       <c r="X199" s="24" t="n">
         <f aca="false">X198/Inputs!$C$8-1</f>
-        <v>0.190653571512023</v>
+        <v>0.189744663107028</v>
       </c>
       <c r="Y199" s="24" t="n">
         <f aca="false">Y198/Inputs!$C$8-1</f>
-        <v>0.190561702841365</v>
+        <v>0.189654074878809</v>
       </c>
       <c r="Z199" s="24" t="n">
         <f aca="false">Z198/Inputs!$C$8-1</f>
-        <v>0.190472869331314</v>
+        <v>0.189566521224838</v>
       </c>
     </row>
   </sheetData>
@@ -25792,7 +25795,9 @@
       <c r="M5" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="N5" s="4"/>
+      <c r="N5" s="5" t="s">
+        <v>276</v>
+      </c>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -25820,7 +25825,7 @@
       </c>
       <c r="D6" s="20" t="n">
         <f aca="false">Initiatives!C8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">Initiatives!C51</f>
@@ -25838,27 +25843,30 @@
         <f aca="false">Initiatives!C56</f>
         <v>11860393422.3971</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="20" t="n">
+        <f aca="false">Initiatives!C55</f>
+        <v>1560701440</v>
+      </c>
+      <c r="J6" s="27" t="n">
         <f aca="false">Initiatives!C57</f>
         <v>7.59939929471526</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="K6" s="22" t="n">
         <f aca="false">Initiatives!C58</f>
         <v>0.0140794054644096</v>
       </c>
-      <c r="K6" s="28" t="n">
+      <c r="L6" s="28" t="n">
         <f aca="false">Initiatives!C61</f>
         <v>0.00291688581386411</v>
       </c>
-      <c r="L6" s="29" t="n">
+      <c r="M6" s="29" t="n">
         <f aca="false">Initiatives!C35</f>
         <v>0.92</v>
       </c>
-      <c r="M6" s="20" t="n">
+      <c r="N6" s="20" t="n">
         <f aca="false">Initiatives!C62</f>
         <v>10911561948.6053</v>
       </c>
-      <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -25886,7 +25894,7 @@
       </c>
       <c r="D7" s="20" t="n">
         <f aca="false">Initiatives!D8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">Initiatives!D51</f>
@@ -25904,27 +25912,30 @@
         <f aca="false">Initiatives!D56</f>
         <v>42853249062.6846</v>
       </c>
-      <c r="I7" s="27" t="n">
+      <c r="I7" s="20" t="n">
+        <f aca="false">Initiatives!D55</f>
+        <v>6264379729.49241</v>
+      </c>
+      <c r="J7" s="27" t="n">
         <f aca="false">Initiatives!D57</f>
         <v>6.84078087746397</v>
       </c>
-      <c r="J7" s="22" t="n">
+      <c r="K7" s="22" t="n">
         <f aca="false">Initiatives!D58</f>
         <v>0.045519115304399</v>
       </c>
-      <c r="K7" s="28" t="n">
+      <c r="L7" s="28" t="n">
         <f aca="false">Initiatives!D61</f>
         <v>-0.0383269133106458</v>
       </c>
-      <c r="L7" s="29" t="n">
+      <c r="M7" s="29" t="n">
         <f aca="false">Initiatives!D35</f>
         <v>0.8</v>
       </c>
-      <c r="M7" s="20" t="n">
+      <c r="N7" s="20" t="n">
         <f aca="false">Initiatives!D62</f>
         <v>34282599250.1477</v>
       </c>
-      <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
@@ -25952,7 +25963,7 @@
       </c>
       <c r="D8" s="20" t="n">
         <f aca="false">Initiatives!E8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="20" t="n">
         <f aca="false">Initiatives!E51</f>
@@ -25970,27 +25981,30 @@
         <f aca="false">Initiatives!E56</f>
         <v>1711952400.16244</v>
       </c>
-      <c r="I8" s="27" t="n">
+      <c r="I8" s="20" t="n">
+        <f aca="false">Initiatives!E55</f>
+        <v>1098446639.45585</v>
+      </c>
+      <c r="J8" s="27" t="n">
         <f aca="false">Initiatives!E57</f>
         <v>1.55852122321618</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="K8" s="22" t="n">
         <f aca="false">Initiatives!E58</f>
         <v>0.00266500342391263</v>
       </c>
-      <c r="K8" s="28" t="n">
+      <c r="L8" s="28" t="n">
         <f aca="false">Initiatives!E61</f>
         <v>0.00217117401781624</v>
       </c>
-      <c r="L8" s="29" t="n">
+      <c r="M8" s="29" t="n">
         <f aca="false">Initiatives!E35</f>
         <v>0.9</v>
       </c>
-      <c r="M8" s="20" t="n">
+      <c r="N8" s="20" t="n">
         <f aca="false">Initiatives!E62</f>
         <v>1540757160.1462</v>
       </c>
-      <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
@@ -26018,7 +26032,7 @@
       </c>
       <c r="D9" s="20" t="n">
         <f aca="false">Initiatives!F8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="20" t="n">
         <f aca="false">Initiatives!F51</f>
@@ -26036,27 +26050,30 @@
         <f aca="false">Initiatives!F56</f>
         <v>3075572916.01749</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="20" t="n">
+        <f aca="false">Initiatives!F55</f>
+        <v>907441423.875801</v>
+      </c>
+      <c r="J9" s="27" t="n">
         <f aca="false">Initiatives!F57</f>
         <v>3.38927983128798</v>
       </c>
-      <c r="J9" s="22" t="n">
+      <c r="K9" s="22" t="n">
         <f aca="false">Initiatives!F58</f>
         <v>0.00381928320992175</v>
       </c>
-      <c r="K9" s="28" t="n">
+      <c r="L9" s="28" t="n">
         <f aca="false">Initiatives!F61</f>
         <v>0.00102423676759064</v>
       </c>
-      <c r="L9" s="29" t="n">
+      <c r="M9" s="29" t="n">
         <f aca="false">Initiatives!F35</f>
         <v>0.9</v>
       </c>
-      <c r="M9" s="20" t="n">
+      <c r="N9" s="20" t="n">
         <f aca="false">Initiatives!F62</f>
         <v>2768015624.41574</v>
       </c>
-      <c r="N9" s="4"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
@@ -26084,7 +26101,7 @@
       </c>
       <c r="D10" s="20" t="n">
         <f aca="false">Initiatives!G8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="20" t="n">
         <f aca="false">Initiatives!G51</f>
@@ -26102,27 +26119,30 @@
         <f aca="false">Initiatives!G56</f>
         <v>843367623.111454</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="20" t="n">
+        <f aca="false">Initiatives!G55</f>
+        <v>567840000</v>
+      </c>
+      <c r="J10" s="27" t="n">
         <f aca="false">Initiatives!G57</f>
         <v>1.48522052534421</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="K10" s="22" t="n">
         <f aca="false">Initiatives!G58</f>
         <v>0.00414336405929094</v>
       </c>
-      <c r="K10" s="28" t="n">
+      <c r="L10" s="28" t="n">
         <f aca="false">Initiatives!G61</f>
         <v>0.00309113677385265</v>
       </c>
-      <c r="L10" s="29" t="n">
+      <c r="M10" s="29" t="n">
         <f aca="false">Initiatives!G35</f>
         <v>0.85</v>
       </c>
-      <c r="M10" s="20" t="n">
+      <c r="N10" s="20" t="n">
         <f aca="false">Initiatives!G62</f>
         <v>716862479.644736</v>
       </c>
-      <c r="N10" s="4"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
@@ -26150,7 +26170,7 @@
       </c>
       <c r="D11" s="20" t="n">
         <f aca="false">Initiatives!H8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="20" t="n">
         <f aca="false">Initiatives!H51</f>
@@ -26168,27 +26188,30 @@
         <f aca="false">Initiatives!H56</f>
         <v>915418332.8176</v>
       </c>
-      <c r="I11" s="27" t="n">
+      <c r="I11" s="20" t="n">
+        <f aca="false">Initiatives!H55</f>
+        <v>524883200</v>
+      </c>
+      <c r="J11" s="27" t="n">
         <f aca="false">Initiatives!H57</f>
         <v>1.74404197508627</v>
       </c>
-      <c r="J11" s="22" t="n">
+      <c r="K11" s="22" t="n">
         <f aca="false">Initiatives!H58</f>
         <v>0.00130097398539686</v>
       </c>
-      <c r="K11" s="28" t="n">
+      <c r="L11" s="28" t="n">
         <f aca="false">Initiatives!H61</f>
         <v>0</v>
       </c>
-      <c r="L11" s="29" t="n">
+      <c r="M11" s="29" t="n">
         <f aca="false">Initiatives!H35</f>
         <v>0.92</v>
       </c>
-      <c r="M11" s="20" t="n">
+      <c r="N11" s="20" t="n">
         <f aca="false">Initiatives!H62</f>
         <v>842184866.192192</v>
       </c>
-      <c r="N11" s="4"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
@@ -26216,7 +26239,7 @@
       </c>
       <c r="D12" s="20" t="n">
         <f aca="false">Initiatives!I8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="20" t="n">
         <f aca="false">Initiatives!I51</f>
@@ -26234,27 +26257,30 @@
         <f aca="false">Initiatives!I56</f>
         <v>1501373785.04368</v>
       </c>
-      <c r="I12" s="27" t="n">
+      <c r="I12" s="20" t="n">
+        <f aca="false">Initiatives!I55</f>
+        <v>395344000</v>
+      </c>
+      <c r="J12" s="27" t="n">
         <f aca="false">Initiatives!I57</f>
         <v>3.79763898034035</v>
       </c>
-      <c r="J12" s="22" t="n">
+      <c r="K12" s="22" t="n">
         <f aca="false">Initiatives!I58</f>
         <v>0.00264450830931495</v>
       </c>
-      <c r="K12" s="28" t="n">
+      <c r="L12" s="28" t="n">
         <f aca="false">Initiatives!I61</f>
         <v>0.00289539747901643</v>
       </c>
-      <c r="L12" s="29" t="n">
+      <c r="M12" s="29" t="n">
         <f aca="false">Initiatives!I35</f>
         <v>0.9</v>
       </c>
-      <c r="M12" s="20" t="n">
+      <c r="N12" s="20" t="n">
         <f aca="false">Initiatives!I62</f>
         <v>1351236406.53931</v>
       </c>
-      <c r="N12" s="4"/>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
@@ -26282,7 +26308,7 @@
       </c>
       <c r="D13" s="20" t="n">
         <f aca="false">Initiatives!J8</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="20" t="n">
         <f aca="false">Initiatives!J51</f>
@@ -26300,27 +26326,30 @@
         <f aca="false">Initiatives!J56</f>
         <v>16723014930.3044</v>
       </c>
-      <c r="I13" s="27" t="n">
+      <c r="I13" s="20" t="n">
+        <f aca="false">Initiatives!J55</f>
+        <v>1691296549.5085</v>
+      </c>
+      <c r="J13" s="27" t="n">
         <f aca="false">Initiatives!J57</f>
         <v>9.88768937958528</v>
       </c>
-      <c r="J13" s="22" t="n">
+      <c r="K13" s="22" t="n">
         <f aca="false">Initiatives!J58</f>
         <v>0.0387801322064303</v>
       </c>
-      <c r="K13" s="28" t="n">
+      <c r="L13" s="28" t="n">
         <f aca="false">Initiatives!J61</f>
         <v>-0.031746071170825</v>
       </c>
-      <c r="L13" s="29" t="n">
+      <c r="M13" s="29" t="n">
         <f aca="false">Initiatives!J35</f>
         <v>0.65</v>
       </c>
-      <c r="M13" s="20" t="n">
+      <c r="N13" s="20" t="n">
         <f aca="false">Initiatives!J62</f>
         <v>10869959704.6979</v>
       </c>
-      <c r="N13" s="4"/>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
@@ -26348,7 +26377,7 @@
       </c>
       <c r="D14" s="20" t="n">
         <f aca="false">Initiatives!K8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="20" t="n">
         <f aca="false">Initiatives!K51</f>
@@ -26366,27 +26395,30 @@
         <f aca="false">Initiatives!K56</f>
         <v>12494217707.9468</v>
       </c>
-      <c r="I14" s="27" t="n">
+      <c r="I14" s="20" t="n">
+        <f aca="false">Initiatives!K55</f>
+        <v>11550000000</v>
+      </c>
+      <c r="J14" s="27" t="n">
         <f aca="false">Initiatives!K57</f>
         <v>1.08175045090448</v>
       </c>
-      <c r="J14" s="22" t="n">
+      <c r="K14" s="22" t="n">
         <f aca="false">Initiatives!K58</f>
         <v>0.0297655959320351</v>
       </c>
-      <c r="K14" s="28" t="n">
+      <c r="L14" s="28" t="n">
         <f aca="false">Initiatives!K61</f>
         <v>0.078003177188188</v>
       </c>
-      <c r="L14" s="29" t="n">
+      <c r="M14" s="29" t="n">
         <f aca="false">Initiatives!K35</f>
         <v>0.65</v>
       </c>
-      <c r="M14" s="20" t="n">
+      <c r="N14" s="20" t="n">
         <f aca="false">Initiatives!K62</f>
         <v>8121241510.16542</v>
       </c>
-      <c r="N14" s="4"/>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
@@ -26414,7 +26446,7 @@
       </c>
       <c r="D15" s="20" t="n">
         <f aca="false">Initiatives!L8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="20" t="n">
         <f aca="false">Initiatives!L51</f>
@@ -26432,27 +26464,30 @@
         <f aca="false">Initiatives!L56</f>
         <v>-66043748.2423842</v>
       </c>
-      <c r="I15" s="27" t="n">
+      <c r="I15" s="20" t="n">
+        <f aca="false">Initiatives!L55</f>
+        <v>6498116683.79822</v>
+      </c>
+      <c r="J15" s="27" t="n">
         <f aca="false">Initiatives!L57</f>
         <v>-0.010163521441074</v>
       </c>
-      <c r="J15" s="22" t="n">
+      <c r="K15" s="22" t="n">
         <f aca="false">Initiatives!L58</f>
         <v>0.00853419017545098</v>
       </c>
-      <c r="K15" s="28" t="n">
+      <c r="L15" s="28" t="n">
         <f aca="false">Initiatives!L61</f>
         <v>0.0221414531827016</v>
       </c>
-      <c r="L15" s="29" t="n">
+      <c r="M15" s="29" t="n">
         <f aca="false">Initiatives!L35</f>
         <v>0.65</v>
       </c>
-      <c r="M15" s="20" t="n">
+      <c r="N15" s="20" t="n">
         <f aca="false">Initiatives!L62</f>
         <v>-42928436.3575497</v>
       </c>
-      <c r="N15" s="4"/>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
@@ -26480,7 +26515,7 @@
       </c>
       <c r="D16" s="20" t="n">
         <f aca="false">Initiatives!M8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="20" t="n">
         <f aca="false">Initiatives!M51</f>
@@ -26498,27 +26533,30 @@
         <f aca="false">Initiatives!M56</f>
         <v>34053675364.5812</v>
       </c>
-      <c r="I16" s="27" t="n">
+      <c r="I16" s="20" t="n">
+        <f aca="false">Initiatives!M55</f>
+        <v>10025933082.141</v>
+      </c>
+      <c r="J16" s="27" t="n">
         <f aca="false">Initiatives!M57</f>
         <v>3.39655921155512</v>
       </c>
-      <c r="J16" s="22" t="n">
+      <c r="K16" s="22" t="n">
         <f aca="false">Initiatives!M58</f>
         <v>0.0808810562761764</v>
       </c>
-      <c r="K16" s="28" t="n">
+      <c r="L16" s="28" t="n">
         <f aca="false">Initiatives!M61</f>
         <v>-0.0810548207939834</v>
       </c>
-      <c r="L16" s="29" t="n">
+      <c r="M16" s="29" t="n">
         <f aca="false">Initiatives!M35</f>
         <v>0.6</v>
       </c>
-      <c r="M16" s="20" t="n">
+      <c r="N16" s="20" t="n">
         <f aca="false">Initiatives!M62</f>
         <v>20432205218.7487</v>
       </c>
-      <c r="N16" s="4"/>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
@@ -26564,27 +26602,30 @@
         <f aca="false">Initiatives!N56</f>
         <v>-2862503999.86999</v>
       </c>
-      <c r="I17" s="27" t="n">
+      <c r="I17" s="20" t="n">
+        <f aca="false">Initiatives!N55</f>
+        <v>3652556434.53057</v>
+      </c>
+      <c r="J17" s="27" t="n">
         <f aca="false">Initiatives!N57</f>
         <v>-0.783698774044509</v>
       </c>
-      <c r="J17" s="22" t="n">
+      <c r="K17" s="22" t="n">
         <f aca="false">Initiatives!N58</f>
         <v>0.00114043578504597</v>
       </c>
-      <c r="K17" s="28" t="n">
+      <c r="L17" s="28" t="n">
         <f aca="false">Initiatives!N61</f>
         <v>0.000633984625185446</v>
       </c>
-      <c r="L17" s="29" t="n">
+      <c r="M17" s="29" t="n">
         <f aca="false">Initiatives!N35</f>
         <v>0.6</v>
       </c>
-      <c r="M17" s="20" t="n">
+      <c r="N17" s="20" t="n">
         <f aca="false">Initiatives!N62</f>
         <v>-1717502399.92199</v>
       </c>
-      <c r="N17" s="4"/>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
@@ -26612,7 +26653,7 @@
       </c>
       <c r="D18" s="20" t="n">
         <f aca="false">Initiatives!O8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" s="20" t="n">
         <f aca="false">Initiatives!O51</f>
@@ -26630,27 +26671,30 @@
         <f aca="false">Initiatives!O56</f>
         <v>-254896090.914283</v>
       </c>
-      <c r="I18" s="27" t="n">
+      <c r="I18" s="20" t="n">
+        <f aca="false">Initiatives!O55</f>
+        <v>3307520000</v>
+      </c>
+      <c r="J18" s="27" t="n">
         <f aca="false">Initiatives!O57</f>
         <v>-0.0770656234623774</v>
       </c>
-      <c r="J18" s="22" t="n">
+      <c r="K18" s="22" t="n">
         <f aca="false">Initiatives!O58</f>
         <v>0.00434526650248546</v>
       </c>
-      <c r="K18" s="28" t="n">
+      <c r="L18" s="28" t="n">
         <f aca="false">Initiatives!O61</f>
         <v>0.00474744855864609</v>
       </c>
-      <c r="L18" s="29" t="n">
+      <c r="M18" s="29" t="n">
         <f aca="false">Initiatives!O35</f>
         <v>0.7</v>
       </c>
-      <c r="M18" s="20" t="n">
+      <c r="N18" s="20" t="n">
         <f aca="false">Initiatives!O62</f>
         <v>-178427263.639998</v>
       </c>
-      <c r="N18" s="4"/>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
@@ -26694,7 +26738,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -26724,12 +26768,12 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="13" t="n">
-        <f aca="false">SUMIFS(E6:E18,$D$6:$D$18,0)*(1-$C$3)</f>
-        <v>43798486275.1951</v>
+        <f aca="false">SUMIFS(E6:E18,$D$6:$D$18,1)*(1-$C$3)</f>
+        <v>43621778943.4539</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
@@ -26757,12 +26801,12 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="13" t="n">
-        <f aca="false">SUMIFS(F6:F18,$D$6:$D$18,0)*(1-$C$3)</f>
-        <v>90348337791.4445</v>
+        <f aca="false">SUMIFS(F6:F18,$D$6:$D$18,1)*(1-$C$3)</f>
+        <v>89781466361.1523</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
@@ -26790,12 +26834,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="13" t="n">
-        <f aca="false">SUMIFS(G6:G18,$D$6:$D$18,0)*(1-$C$3)</f>
-        <v>85568895751.9332</v>
+        <f aca="false">SUMIFS(G6:G18,$D$6:$D$18,1)*(1-$C$3)</f>
+        <v>85030320106.5008</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
@@ -26823,12 +26867,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="30" t="n">
         <f aca="false">C23/Inputs!$C$11</f>
-        <v>7071809.56627547</v>
+        <v>7027299.18235543</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
@@ -26856,12 +26900,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="13" t="n">
-        <f aca="false">SUMIFS(H6:H18,$D$6:$D$18,0)-$C$3*MAX(SUMIFS(H6:H18,$D$6:$D$18,0),0)</f>
-        <v>84900621420.5886</v>
+        <f aca="false">(SUMIFS(H6:H18,$D$6:$D$18,1)+SUMIFS(I6:I18,$D$6:$D$18,1))*(1-$C$3)-SUMIFS(I6:I18,$D$6:$D$18,1)</f>
+        <v>78650503380.7319</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
@@ -26889,7 +26933,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="13" t="n">
@@ -26922,12 +26966,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="13" t="n">
         <f aca="false">Monthly!N196</f>
-        <v>21424.9103070361</v>
+        <v>21407.9984883237</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
@@ -26955,12 +26999,12 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="13" t="n">
         <f aca="false">Monthly!Z196</f>
-        <v>21437.7112061271</v>
+        <v>21420.9629827772</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
@@ -26988,12 +27032,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="12" t="n">
         <f aca="false">Monthly!N197</f>
-        <v>0.15810325983979</v>
+        <v>0.157189107476957</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
@@ -27021,12 +27065,12 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="12" t="n">
         <f aca="false">Monthly!Z197</f>
-        <v>0.158795200331197</v>
+        <v>0.157889890960932</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
@@ -27054,12 +27098,12 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="12" t="n">
         <f aca="false">Monthly!Z199</f>
-        <v>0.190472869331314</v>
+        <v>0.189566521224838</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
@@ -27087,12 +27131,12 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="12" t="n">
         <f aca="false">IF(Inputs!C13&gt;0,C23/(Inputs!C13*12),0)</f>
-        <v>0.109501555784108</v>
+        <v>0.108812346573634</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
@@ -27120,12 +27164,12 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="31" t="n">
-        <f aca="false">SUMIFS(K6:K18,$D$6:$D$18,0)*(1-$C$3)</f>
-        <v>-0.00140547175821443</v>
+        <f aca="false">SUMIFS(L6:L18,$D$6:$D$18,1)*(1-$C$3)</f>
+        <v>-0.00191265945836279</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
@@ -27209,7 +27253,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -27317,7 +27361,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="29" t="n">
@@ -27346,80 +27390,80 @@
       </c>
       <c r="I38" s="29" t="n">
         <f aca="false">Monthly!I197</f>
-        <v>0.0621315570872716</v>
+        <v>0.061985033613716</v>
       </c>
       <c r="J38" s="29" t="n">
         <f aca="false">Monthly!J197</f>
-        <v>0.069418719511358</v>
+        <v>0.0691235127657535</v>
       </c>
       <c r="K38" s="29" t="n">
         <f aca="false">Monthly!K197</f>
-        <v>0.0770839389395031</v>
+        <v>0.0766379481432185</v>
       </c>
       <c r="L38" s="29" t="n">
         <f aca="false">Monthly!L197</f>
-        <v>0.0847730367239115</v>
+        <v>0.084174219083041</v>
       </c>
       <c r="M38" s="29" t="n">
         <f aca="false">Monthly!M197</f>
-        <v>0.0924824310559202</v>
+        <v>0.0917288044418745</v>
       </c>
       <c r="N38" s="29" t="n">
         <f aca="false">Monthly!N197</f>
-        <v>0.15810325983979</v>
+        <v>0.157189107476957</v>
       </c>
       <c r="O38" s="29" t="n">
         <f aca="false">Monthly!O197</f>
-        <v>0.159703081199678</v>
+        <v>0.158785562750602</v>
       </c>
       <c r="P38" s="29" t="n">
         <f aca="false">Monthly!P197</f>
-        <v>0.159597929317036</v>
+        <v>0.158681525125549</v>
       </c>
       <c r="Q38" s="29" t="n">
         <f aca="false">Monthly!Q197</f>
-        <v>0.159498244825305</v>
+        <v>0.158582953831683</v>
       </c>
       <c r="R38" s="29" t="n">
         <f aca="false">Monthly!R197</f>
-        <v>0.159403667150353</v>
+        <v>0.158489488369902</v>
       </c>
       <c r="S38" s="29" t="n">
         <f aca="false">Monthly!S197</f>
-        <v>0.159313860994026</v>
+        <v>0.158400793510755</v>
       </c>
       <c r="T38" s="29" t="n">
         <f aca="false">Monthly!T197</f>
-        <v>0.159228514564728</v>
+        <v>0.158316557525587</v>
       </c>
       <c r="U38" s="29" t="n">
         <f aca="false">Monthly!U197</f>
-        <v>0.15914733793189</v>
+        <v>0.158236490541512</v>
       </c>
       <c r="V38" s="29" t="n">
         <f aca="false">Monthly!V197</f>
-        <v>0.159070061495652</v>
+        <v>0.158160323011566</v>
       </c>
       <c r="W38" s="29" t="n">
         <f aca="false">Monthly!W197</f>
-        <v>0.158996434563685</v>
+        <v>0.158087804291958</v>
       </c>
       <c r="X38" s="29" t="n">
         <f aca="false">Monthly!X197</f>
-        <v>0.158926224027667</v>
+        <v>0.158018701318935</v>
       </c>
       <c r="Y38" s="29" t="n">
         <f aca="false">Monthly!Y197</f>
-        <v>0.158859213132414</v>
+        <v>0.157952797378276</v>
       </c>
       <c r="Z38" s="29" t="n">
         <f aca="false">Monthly!Z197</f>
-        <v>0.158795200331197</v>
+        <v>0.157889890960932</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="29" t="n">
@@ -27448,75 +27492,75 @@
       </c>
       <c r="I39" s="29" t="n">
         <f aca="false">Monthly!I199</f>
-        <v>0.0621315570872716</v>
+        <v>0.061985033613716</v>
       </c>
       <c r="J39" s="29" t="n">
         <f aca="false">Monthly!J199</f>
-        <v>0.069418719511358</v>
+        <v>0.0691235127657535</v>
       </c>
       <c r="K39" s="29" t="n">
         <f aca="false">Monthly!K199</f>
-        <v>0.0770839389395031</v>
+        <v>0.0766379481432185</v>
       </c>
       <c r="L39" s="29" t="n">
         <f aca="false">Monthly!L199</f>
-        <v>0.0847730367239115</v>
+        <v>0.084174219083041</v>
       </c>
       <c r="M39" s="29" t="n">
         <f aca="false">Monthly!M199</f>
-        <v>0.0924824310559202</v>
+        <v>0.0917288044418745</v>
       </c>
       <c r="N39" s="29" t="n">
         <f aca="false">Monthly!N199</f>
-        <v>0.15810325983979</v>
+        <v>0.157189107476957</v>
       </c>
       <c r="O39" s="29" t="n">
         <f aca="false">Monthly!O199</f>
-        <v>0.159703081199678</v>
+        <v>0.158785562750602</v>
       </c>
       <c r="P39" s="29" t="n">
         <f aca="false">Monthly!P199</f>
-        <v>0.192147052111267</v>
+        <v>0.191229662214945</v>
       </c>
       <c r="Q39" s="29" t="n">
         <f aca="false">Monthly!Q199</f>
-        <v>0.19140071552816</v>
+        <v>0.190482823907693</v>
       </c>
       <c r="R39" s="29" t="n">
         <f aca="false">Monthly!R199</f>
-        <v>0.191280992647323</v>
+        <v>0.190364386863735</v>
       </c>
       <c r="S39" s="29" t="n">
         <f aca="false">Monthly!S199</f>
-        <v>0.191166085856019</v>
+        <v>0.190250764970839</v>
       </c>
       <c r="T39" s="29" t="n">
         <f aca="false">Monthly!T199</f>
-        <v>0.191055682056861</v>
+        <v>0.190141645195647</v>
       </c>
       <c r="U39" s="29" t="n">
         <f aca="false">Monthly!U199</f>
-        <v>0.190949490101003</v>
+        <v>0.190036736448046</v>
       </c>
       <c r="V39" s="29" t="n">
         <f aca="false">Monthly!V199</f>
-        <v>0.190847239251648</v>
+        <v>0.18993576804514</v>
       </c>
       <c r="W39" s="29" t="n">
         <f aca="false">Monthly!W199</f>
-        <v>0.190748677755125</v>
+        <v>0.189838488282769</v>
       </c>
       <c r="X39" s="29" t="n">
         <f aca="false">Monthly!X199</f>
-        <v>0.190653571512023</v>
+        <v>0.189744663107028</v>
       </c>
       <c r="Y39" s="29" t="n">
         <f aca="false">Monthly!Y199</f>
-        <v>0.190561702841365</v>
+        <v>0.189654074878809</v>
       </c>
       <c r="Z39" s="29" t="n">
         <f aca="false">Monthly!Z199</f>
-        <v>0.190472869331314</v>
+        <v>0.189566521224838</v>
       </c>
     </row>
   </sheetData>
@@ -27545,7 +27589,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B1" s="4"/>
     </row>
@@ -27555,7 +27599,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>0.05</v>
@@ -27563,7 +27607,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>0.8</v>
@@ -27571,7 +27615,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B5" s="32" t="n">
         <v>1.2</v>
@@ -27579,7 +27623,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>0.03</v>
@@ -27591,7 +27635,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">ROUNDUP(2*(NORMSINV(1-B3/2)+NORMSINV(B4))^2*B5^2/B6^2,0)</f>
@@ -27604,7 +27648,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>0.1</v>
@@ -27612,7 +27656,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>0.11</v>
@@ -27620,7 +27664,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">ROUNDUP((NORMSINV(1-B3/2)*SQRT(2*((B10+B11)/2)*(1-(B10+B11)/2))+NORMSINV(B4)*SQRT(B10*(1-B10)+B11*(1-B11)))^2/(B11-B10)^2,0)</f>
@@ -27633,7 +27677,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B14" s="4"/>
     </row>
@@ -27663,7 +27707,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -27681,7 +27725,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -27724,37 +27768,37 @@
         <v>265</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28347,7 +28391,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -28365,83 +28409,83 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="9" t="n">
-        <v>0.11470935337184</v>
+        <v>0.114184816822331</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>0.0615791309015985</v>
+        <v>0.0609962280758441</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>0.115396552014496</v>
+        <v>0.11497886358154</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>0.169959922979799</v>
+        <v>0.169335118517538</v>
       </c>
       <c r="G21" s="16" t="n">
-        <v>36.9</v>
+        <v>36.7</v>
       </c>
       <c r="H21" s="16" t="n">
-        <v>65</v>
+        <v>64.6</v>
       </c>
       <c r="I21" s="16" t="n">
-        <v>58.6</v>
+        <v>53</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.61145</v>
+        <v>0.6068</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>0.2285</v>
+        <v>0.22355</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.01405</v>
+        <v>0.0134</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="9" t="n">
@@ -28463,7 +28507,7 @@
         <v>29.7</v>
       </c>
       <c r="I22" s="16" t="n">
-        <v>44.3</v>
+        <v>41.8</v>
       </c>
       <c r="J22" s="9" t="n">
         <v>0</v>
@@ -28479,35 +28523,35 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="9" t="n">
-        <v>0.0655693187125627</v>
+        <v>0.065073136936941</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>0.0113336019029391</v>
+        <v>0.0107105859421485</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>0.0669059035218867</v>
+        <v>0.0665313739896132</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>0.11297205557994</v>
+        <v>0.112358426611177</v>
       </c>
       <c r="G23" s="16" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="H23" s="16" t="n">
-        <v>36.2</v>
+        <v>35.8</v>
       </c>
       <c r="I23" s="16" t="n">
-        <v>16.8</v>
+        <v>13.5</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>0.1982</v>
+        <v>0.193</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>0.00435</v>
+        <v>0.0041</v>
       </c>
       <c r="L23" s="9" t="n">
         <v>0</v>
@@ -28517,38 +28561,38 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="9" t="n">
-        <v>0.114474198489721</v>
+        <v>0.114042333506375</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>0.0763168896552873</v>
+        <v>0.0759083228160557</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>0.134682976508839</v>
+        <v>0.13396485774192</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.19421287704953</v>
+        <v>0.193504197892996</v>
       </c>
       <c r="G24" s="16" t="n">
-        <v>36.9</v>
+        <v>36.7</v>
       </c>
       <c r="H24" s="16" t="n">
-        <v>74.1</v>
+        <v>73.6</v>
       </c>
       <c r="I24" s="16" t="n">
-        <v>66.4</v>
+        <v>60.4</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>0.75755</v>
+        <v>0.7527</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>0.38625</v>
+        <v>0.3825</v>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.0764</v>
+        <v>0.07445</v>
       </c>
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>

</xml_diff>